<commit_message>
Removed "GBR" from Scuba Diving Tours
</commit_message>
<xml_diff>
--- a/CDT AITP Go Live (2).xlsx
+++ b/CDT AITP Go Live (2).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/af3a32376182f586/Desktop/Cairns AI Planner/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="14_{082FEF11-AC35-4F61-BAA4-E1B03605CFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{620A443C-BD76-4250-8FE4-EAFAC0EF1C77}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="14_{082FEF11-AC35-4F61-BAA4-E1B03605CFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5963B9E-18B5-48D4-82E2-D8A6A227E1C1}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3975" uniqueCount="756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3972" uniqueCount="756">
   <si>
     <t>Cairns Must Do's</t>
   </si>
@@ -2961,6 +2961,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -3167,17 +3171,17 @@
   <cols>
     <col min="1" max="1" width="6.86328125" customWidth="1"/>
     <col min="2" max="2" width="48.46484375" customWidth="1"/>
-    <col min="3" max="3" width="9.3984375" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="31.1328125" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="35.3984375" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="20.796875" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="26.3984375" hidden="1" customWidth="1"/>
-    <col min="8" max="10" width="12.59765625" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="21.06640625" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="21.33203125" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="19.33203125" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="21.46484375" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="5.3984375" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="9.3984375" customWidth="1"/>
+    <col min="4" max="4" width="31.1328125" customWidth="1"/>
+    <col min="5" max="5" width="35.3984375" customWidth="1"/>
+    <col min="6" max="6" width="20.796875" customWidth="1"/>
+    <col min="7" max="7" width="26.3984375" customWidth="1"/>
+    <col min="8" max="10" width="12.59765625" customWidth="1"/>
+    <col min="11" max="11" width="21.06640625" customWidth="1"/>
+    <col min="12" max="12" width="21.33203125" customWidth="1"/>
+    <col min="13" max="13" width="19.33203125" customWidth="1"/>
+    <col min="14" max="14" width="21.46484375" customWidth="1"/>
+    <col min="15" max="15" width="5.3984375" customWidth="1"/>
     <col min="16" max="16" width="85.59765625" style="95" customWidth="1"/>
     <col min="17" max="18" width="27.33203125" style="95" customWidth="1"/>
     <col min="19" max="19" width="94.9296875" customWidth="1"/>
@@ -7284,13 +7288,13 @@
         <v>212</v>
       </c>
       <c r="K52" s="47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L52" s="47" t="b">
         <v>0</v>
       </c>
       <c r="M52" s="47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N52" s="47" t="b">
         <v>0</v>
@@ -7363,13 +7367,13 @@
         <v>212</v>
       </c>
       <c r="K53" s="47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L53" s="47" t="b">
         <v>0</v>
       </c>
       <c r="M53" s="47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N53" s="47" t="b">
         <v>0</v>
@@ -7440,13 +7444,13 @@
         <v>212</v>
       </c>
       <c r="K54" s="47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L54" s="47" t="b">
         <v>0</v>
       </c>
       <c r="M54" s="47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N54" s="47" t="b">
         <v>0</v>
@@ -10924,9 +10928,7 @@
       <c r="E98" s="65" t="s">
         <v>603</v>
       </c>
-      <c r="F98" s="65" t="s">
-        <v>5</v>
-      </c>
+      <c r="F98" s="65"/>
       <c r="G98" s="65" t="s">
         <v>18</v>
       </c>
@@ -10944,10 +10946,10 @@
         <v>1</v>
       </c>
       <c r="M98" s="67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N98" s="67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O98" s="66">
         <v>8</v>
@@ -11003,9 +11005,7 @@
       <c r="E99" s="65" t="s">
         <v>603</v>
       </c>
-      <c r="F99" s="65" t="s">
-        <v>5</v>
-      </c>
+      <c r="F99" s="65"/>
       <c r="G99" s="65" t="s">
         <v>18</v>
       </c>
@@ -11023,7 +11023,7 @@
         <v>1</v>
       </c>
       <c r="M99" s="67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N99" s="67" t="b">
         <v>0</v>
@@ -11082,9 +11082,7 @@
       <c r="E100" s="65" t="s">
         <v>603</v>
       </c>
-      <c r="F100" s="65" t="s">
-        <v>5</v>
-      </c>
+      <c r="F100" s="65"/>
       <c r="G100" s="65" t="s">
         <v>18</v>
       </c>
@@ -11102,10 +11100,10 @@
         <v>1</v>
       </c>
       <c r="M100" s="67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N100" s="67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O100" s="66">
         <v>8</v>

</xml_diff>

<commit_message>
Crocodile Encounter changed to "Experience"
</commit_message>
<xml_diff>
--- a/CDT AITP Go Live (2).xlsx
+++ b/CDT AITP Go Live (2).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/af3a32376182f586/Desktop/Cairns AI Planner/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="14_{082FEF11-AC35-4F61-BAA4-E1B03605CFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5963B9E-18B5-48D4-82E2-D8A6A227E1C1}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="14_{082FEF11-AC35-4F61-BAA4-E1B03605CFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4438CDE2-C964-45D8-B568-21B3115CD22D}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3972" uniqueCount="756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3972" uniqueCount="757">
   <si>
     <t>Cairns Must Do's</t>
   </si>
@@ -2346,6 +2346,9 @@
   </si>
   <si>
     <t>https://www.cairnsdiscoverytours.com/wp-content/uploads/2025/09/CDT_Green_Island_National_Park.jpg.webp</t>
+  </si>
+  <si>
+    <t>Crocodile Experience</t>
   </si>
 </sst>
 </file>
@@ -2908,15 +2911,30 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2925,23 +2943,8 @@
     <xf numFmtId="0" fontId="18" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3242,10 +3245,10 @@
       <c r="R1" s="85" t="s">
         <v>607</v>
       </c>
-      <c r="S1" s="112" t="s">
+      <c r="S1" s="108" t="s">
         <v>210</v>
       </c>
-      <c r="T1" s="112"/>
+      <c r="T1" s="108"/>
       <c r="U1" s="43"/>
       <c r="V1" s="43"/>
       <c r="W1" s="43"/>
@@ -3288,10 +3291,10 @@
       <c r="G2" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="H2" s="102" t="s">
+      <c r="H2" s="104" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="102"/>
+      <c r="I2" s="104"/>
       <c r="J2" s="43" t="s">
         <v>213</v>
       </c>
@@ -3319,14 +3322,14 @@
       <c r="R2" s="86" t="s">
         <v>609</v>
       </c>
-      <c r="S2" s="102" t="s">
+      <c r="S2" s="104" t="s">
         <v>184</v>
       </c>
-      <c r="T2" s="102"/>
-      <c r="U2" s="102"/>
-      <c r="V2" s="102"/>
-      <c r="W2" s="102"/>
-      <c r="X2" s="102"/>
+      <c r="T2" s="104"/>
+      <c r="U2" s="104"/>
+      <c r="V2" s="104"/>
+      <c r="W2" s="104"/>
+      <c r="X2" s="104"/>
       <c r="Y2" s="43"/>
       <c r="Z2" s="43"/>
       <c r="AA2" s="43"/>
@@ -3398,15 +3401,15 @@
       <c r="R3" s="86" t="s">
         <v>611</v>
       </c>
-      <c r="S3" s="102" t="s">
+      <c r="S3" s="104" t="s">
         <v>194</v>
       </c>
-      <c r="T3" s="102"/>
-      <c r="U3" s="102"/>
-      <c r="V3" s="102"/>
-      <c r="W3" s="102"/>
-      <c r="X3" s="102"/>
-      <c r="Y3" s="102"/>
+      <c r="T3" s="104"/>
+      <c r="U3" s="104"/>
+      <c r="V3" s="104"/>
+      <c r="W3" s="104"/>
+      <c r="X3" s="104"/>
+      <c r="Y3" s="104"/>
       <c r="Z3" s="43"/>
       <c r="AA3" s="43"/>
       <c r="AB3" s="43"/>
@@ -3477,14 +3480,14 @@
       <c r="R4" s="86" t="s">
         <v>612</v>
       </c>
-      <c r="S4" s="102" t="s">
+      <c r="S4" s="104" t="s">
         <v>214</v>
       </c>
-      <c r="T4" s="102"/>
-      <c r="U4" s="102"/>
-      <c r="V4" s="102"/>
-      <c r="W4" s="102"/>
-      <c r="X4" s="102"/>
+      <c r="T4" s="104"/>
+      <c r="U4" s="104"/>
+      <c r="V4" s="104"/>
+      <c r="W4" s="104"/>
+      <c r="X4" s="104"/>
       <c r="Y4" s="43"/>
       <c r="Z4" s="43"/>
       <c r="AA4" s="43"/>
@@ -3558,15 +3561,15 @@
       <c r="R5" s="86" t="s">
         <v>614</v>
       </c>
-      <c r="S5" s="102" t="s">
+      <c r="S5" s="104" t="s">
         <v>219</v>
       </c>
-      <c r="T5" s="102"/>
-      <c r="U5" s="102"/>
-      <c r="V5" s="102"/>
-      <c r="W5" s="102"/>
-      <c r="X5" s="102"/>
-      <c r="Y5" s="102"/>
+      <c r="T5" s="104"/>
+      <c r="U5" s="104"/>
+      <c r="V5" s="104"/>
+      <c r="W5" s="104"/>
+      <c r="X5" s="104"/>
+      <c r="Y5" s="104"/>
       <c r="Z5" s="43"/>
       <c r="AA5" s="43"/>
       <c r="AB5" s="43"/>
@@ -3635,15 +3638,15 @@
       <c r="R6" s="86" t="s">
         <v>616</v>
       </c>
-      <c r="S6" s="110" t="s">
+      <c r="S6" s="106" t="s">
         <v>72</v>
       </c>
-      <c r="T6" s="110"/>
-      <c r="U6" s="110"/>
-      <c r="V6" s="110"/>
-      <c r="W6" s="110"/>
-      <c r="X6" s="110"/>
-      <c r="Y6" s="110"/>
+      <c r="T6" s="106"/>
+      <c r="U6" s="106"/>
+      <c r="V6" s="106"/>
+      <c r="W6" s="106"/>
+      <c r="X6" s="106"/>
+      <c r="Y6" s="106"/>
       <c r="Z6" s="50"/>
       <c r="AA6" s="50"/>
       <c r="AB6" s="50"/>
@@ -3712,16 +3715,16 @@
       <c r="R7" s="86" t="s">
         <v>618</v>
       </c>
-      <c r="S7" s="110" t="s">
+      <c r="S7" s="106" t="s">
         <v>77</v>
       </c>
-      <c r="T7" s="110"/>
-      <c r="U7" s="110"/>
-      <c r="V7" s="110"/>
-      <c r="W7" s="110"/>
-      <c r="X7" s="110"/>
-      <c r="Y7" s="110"/>
-      <c r="Z7" s="110"/>
+      <c r="T7" s="106"/>
+      <c r="U7" s="106"/>
+      <c r="V7" s="106"/>
+      <c r="W7" s="106"/>
+      <c r="X7" s="106"/>
+      <c r="Y7" s="106"/>
+      <c r="Z7" s="106"/>
       <c r="AA7" s="50"/>
       <c r="AB7" s="50"/>
       <c r="AC7" s="50"/>
@@ -3791,15 +3794,15 @@
       <c r="R8" s="86" t="s">
         <v>619</v>
       </c>
-      <c r="S8" s="110" t="s">
+      <c r="S8" s="106" t="s">
         <v>190</v>
       </c>
-      <c r="T8" s="110"/>
-      <c r="U8" s="110"/>
-      <c r="V8" s="110"/>
-      <c r="W8" s="110"/>
-      <c r="X8" s="110"/>
-      <c r="Y8" s="110"/>
+      <c r="T8" s="106"/>
+      <c r="U8" s="106"/>
+      <c r="V8" s="106"/>
+      <c r="W8" s="106"/>
+      <c r="X8" s="106"/>
+      <c r="Y8" s="106"/>
       <c r="Z8" s="50"/>
       <c r="AA8" s="50"/>
       <c r="AB8" s="50"/>
@@ -3872,16 +3875,16 @@
       <c r="R9" s="86" t="s">
         <v>615</v>
       </c>
-      <c r="S9" s="108" t="s">
+      <c r="S9" s="107" t="s">
         <v>224</v>
       </c>
-      <c r="T9" s="108"/>
-      <c r="U9" s="108"/>
-      <c r="V9" s="108"/>
-      <c r="W9" s="108"/>
-      <c r="X9" s="108"/>
-      <c r="Y9" s="108"/>
-      <c r="Z9" s="108"/>
+      <c r="T9" s="107"/>
+      <c r="U9" s="107"/>
+      <c r="V9" s="107"/>
+      <c r="W9" s="107"/>
+      <c r="X9" s="107"/>
+      <c r="Y9" s="107"/>
+      <c r="Z9" s="107"/>
       <c r="AA9" s="54"/>
       <c r="AB9" s="54"/>
       <c r="AC9" s="54"/>
@@ -3953,15 +3956,15 @@
       <c r="R10" s="86" t="s">
         <v>610</v>
       </c>
-      <c r="S10" s="104" t="s">
+      <c r="S10" s="105" t="s">
         <v>221</v>
       </c>
-      <c r="T10" s="104"/>
-      <c r="U10" s="104"/>
-      <c r="V10" s="104"/>
-      <c r="W10" s="104"/>
-      <c r="X10" s="104"/>
-      <c r="Y10" s="104"/>
+      <c r="T10" s="105"/>
+      <c r="U10" s="105"/>
+      <c r="V10" s="105"/>
+      <c r="W10" s="105"/>
+      <c r="X10" s="105"/>
+      <c r="Y10" s="105"/>
       <c r="Z10" s="65"/>
       <c r="AA10" s="65"/>
       <c r="AB10" s="65"/>
@@ -4034,15 +4037,15 @@
       <c r="R11" s="86" t="s">
         <v>623</v>
       </c>
-      <c r="S11" s="104" t="s">
+      <c r="S11" s="105" t="s">
         <v>222</v>
       </c>
-      <c r="T11" s="104"/>
-      <c r="U11" s="104"/>
-      <c r="V11" s="104"/>
-      <c r="W11" s="104"/>
-      <c r="X11" s="104"/>
-      <c r="Y11" s="104"/>
+      <c r="T11" s="105"/>
+      <c r="U11" s="105"/>
+      <c r="V11" s="105"/>
+      <c r="W11" s="105"/>
+      <c r="X11" s="105"/>
+      <c r="Y11" s="105"/>
       <c r="Z11" s="65"/>
       <c r="AA11" s="65"/>
       <c r="AB11" s="65"/>
@@ -4115,16 +4118,16 @@
       <c r="R12" s="86" t="s">
         <v>612</v>
       </c>
-      <c r="S12" s="104" t="s">
+      <c r="S12" s="105" t="s">
         <v>226</v>
       </c>
-      <c r="T12" s="104"/>
-      <c r="U12" s="104"/>
-      <c r="V12" s="104"/>
-      <c r="W12" s="104"/>
-      <c r="X12" s="104"/>
-      <c r="Y12" s="104"/>
-      <c r="Z12" s="104"/>
+      <c r="T12" s="105"/>
+      <c r="U12" s="105"/>
+      <c r="V12" s="105"/>
+      <c r="W12" s="105"/>
+      <c r="X12" s="105"/>
+      <c r="Y12" s="105"/>
+      <c r="Z12" s="105"/>
       <c r="AA12" s="65"/>
       <c r="AB12" s="65"/>
       <c r="AC12" s="65"/>
@@ -4159,7 +4162,7 @@
       </c>
       <c r="F13" s="43"/>
       <c r="G13" s="43" t="s">
-        <v>22</v>
+        <v>756</v>
       </c>
       <c r="H13" s="43" t="s">
         <v>10</v>
@@ -4194,16 +4197,16 @@
       <c r="R13" s="86" t="s">
         <v>625</v>
       </c>
-      <c r="S13" s="102" t="s">
+      <c r="S13" s="104" t="s">
         <v>231</v>
       </c>
-      <c r="T13" s="102"/>
-      <c r="U13" s="102"/>
-      <c r="V13" s="102"/>
-      <c r="W13" s="102"/>
-      <c r="X13" s="102"/>
-      <c r="Y13" s="102"/>
-      <c r="Z13" s="102"/>
+      <c r="T13" s="104"/>
+      <c r="U13" s="104"/>
+      <c r="V13" s="104"/>
+      <c r="W13" s="104"/>
+      <c r="X13" s="104"/>
+      <c r="Y13" s="104"/>
+      <c r="Z13" s="104"/>
       <c r="AA13" s="43"/>
       <c r="AB13" s="43"/>
       <c r="AC13" s="43"/>
@@ -4238,7 +4241,7 @@
       </c>
       <c r="F14" s="43"/>
       <c r="G14" s="43" t="s">
-        <v>22</v>
+        <v>756</v>
       </c>
       <c r="H14" s="43" t="s">
         <v>23</v>
@@ -4271,15 +4274,15 @@
       <c r="R14" s="86" t="s">
         <v>627</v>
       </c>
-      <c r="S14" s="102" t="s">
+      <c r="S14" s="104" t="s">
         <v>148</v>
       </c>
-      <c r="T14" s="102"/>
-      <c r="U14" s="102"/>
-      <c r="V14" s="102"/>
-      <c r="W14" s="102"/>
-      <c r="X14" s="102"/>
-      <c r="Y14" s="102"/>
+      <c r="T14" s="104"/>
+      <c r="U14" s="104"/>
+      <c r="V14" s="104"/>
+      <c r="W14" s="104"/>
+      <c r="X14" s="104"/>
+      <c r="Y14" s="104"/>
       <c r="Z14" s="43"/>
       <c r="AA14" s="43"/>
       <c r="AB14" s="43"/>
@@ -4352,16 +4355,16 @@
       <c r="R15" s="86" t="s">
         <v>629</v>
       </c>
-      <c r="S15" s="105" t="s">
+      <c r="S15" s="103" t="s">
         <v>86</v>
       </c>
-      <c r="T15" s="105"/>
-      <c r="U15" s="105"/>
-      <c r="V15" s="105"/>
-      <c r="W15" s="105"/>
-      <c r="X15" s="105"/>
-      <c r="Y15" s="105"/>
-      <c r="Z15" s="105"/>
+      <c r="T15" s="103"/>
+      <c r="U15" s="103"/>
+      <c r="V15" s="103"/>
+      <c r="W15" s="103"/>
+      <c r="X15" s="103"/>
+      <c r="Y15" s="103"/>
+      <c r="Z15" s="103"/>
       <c r="AA15" s="51"/>
       <c r="AB15" s="43"/>
       <c r="AC15" s="43"/>
@@ -4433,17 +4436,17 @@
       <c r="R16" s="86" t="s">
         <v>630</v>
       </c>
-      <c r="S16" s="105" t="s">
+      <c r="S16" s="103" t="s">
         <v>234</v>
       </c>
-      <c r="T16" s="105"/>
-      <c r="U16" s="105"/>
-      <c r="V16" s="105"/>
-      <c r="W16" s="105"/>
-      <c r="X16" s="105"/>
-      <c r="Y16" s="105"/>
-      <c r="Z16" s="105"/>
-      <c r="AA16" s="105"/>
+      <c r="T16" s="103"/>
+      <c r="U16" s="103"/>
+      <c r="V16" s="103"/>
+      <c r="W16" s="103"/>
+      <c r="X16" s="103"/>
+      <c r="Y16" s="103"/>
+      <c r="Z16" s="103"/>
+      <c r="AA16" s="103"/>
       <c r="AB16" s="43"/>
       <c r="AC16" s="43"/>
       <c r="AD16" s="43"/>
@@ -4514,16 +4517,16 @@
       <c r="R17" s="86" t="s">
         <v>632</v>
       </c>
-      <c r="S17" s="105" t="s">
+      <c r="S17" s="103" t="s">
         <v>84</v>
       </c>
-      <c r="T17" s="105"/>
-      <c r="U17" s="105"/>
-      <c r="V17" s="105"/>
-      <c r="W17" s="105"/>
-      <c r="X17" s="105"/>
-      <c r="Y17" s="105"/>
-      <c r="Z17" s="105"/>
+      <c r="T17" s="103"/>
+      <c r="U17" s="103"/>
+      <c r="V17" s="103"/>
+      <c r="W17" s="103"/>
+      <c r="X17" s="103"/>
+      <c r="Y17" s="103"/>
+      <c r="Z17" s="103"/>
       <c r="AA17" s="51"/>
       <c r="AB17" s="43"/>
       <c r="AC17" s="43"/>
@@ -4595,14 +4598,14 @@
       <c r="R18" s="86" t="s">
         <v>632</v>
       </c>
-      <c r="S18" s="105" t="s">
+      <c r="S18" s="103" t="s">
         <v>82</v>
       </c>
-      <c r="T18" s="105"/>
-      <c r="U18" s="105"/>
-      <c r="V18" s="105"/>
-      <c r="W18" s="105"/>
-      <c r="X18" s="105"/>
+      <c r="T18" s="103"/>
+      <c r="U18" s="103"/>
+      <c r="V18" s="103"/>
+      <c r="W18" s="103"/>
+      <c r="X18" s="103"/>
       <c r="Y18" s="51"/>
       <c r="Z18" s="51"/>
       <c r="AA18" s="51"/>
@@ -4676,15 +4679,15 @@
       <c r="R19" s="86" t="s">
         <v>634</v>
       </c>
-      <c r="S19" s="105" t="s">
+      <c r="S19" s="103" t="s">
         <v>96</v>
       </c>
-      <c r="T19" s="105"/>
-      <c r="U19" s="105"/>
-      <c r="V19" s="105"/>
-      <c r="W19" s="105"/>
-      <c r="X19" s="105"/>
-      <c r="Y19" s="105"/>
+      <c r="T19" s="103"/>
+      <c r="U19" s="103"/>
+      <c r="V19" s="103"/>
+      <c r="W19" s="103"/>
+      <c r="X19" s="103"/>
+      <c r="Y19" s="103"/>
       <c r="Z19" s="51"/>
       <c r="AA19" s="51"/>
       <c r="AB19" s="43"/>
@@ -4757,16 +4760,16 @@
       <c r="R20" s="86" t="s">
         <v>636</v>
       </c>
-      <c r="S20" s="105" t="s">
+      <c r="S20" s="103" t="s">
         <v>235</v>
       </c>
-      <c r="T20" s="105"/>
-      <c r="U20" s="105"/>
-      <c r="V20" s="105"/>
-      <c r="W20" s="105"/>
-      <c r="X20" s="105"/>
-      <c r="Y20" s="105"/>
-      <c r="Z20" s="105"/>
+      <c r="T20" s="103"/>
+      <c r="U20" s="103"/>
+      <c r="V20" s="103"/>
+      <c r="W20" s="103"/>
+      <c r="X20" s="103"/>
+      <c r="Y20" s="103"/>
+      <c r="Z20" s="103"/>
       <c r="AA20" s="51"/>
       <c r="AB20" s="43"/>
       <c r="AC20" s="43"/>
@@ -4838,15 +4841,15 @@
       <c r="R21" s="86" t="s">
         <v>610</v>
       </c>
-      <c r="S21" s="105" t="s">
+      <c r="S21" s="103" t="s">
         <v>236</v>
       </c>
-      <c r="T21" s="105"/>
-      <c r="U21" s="105"/>
-      <c r="V21" s="105"/>
-      <c r="W21" s="105"/>
-      <c r="X21" s="105"/>
-      <c r="Y21" s="105"/>
+      <c r="T21" s="103"/>
+      <c r="U21" s="103"/>
+      <c r="V21" s="103"/>
+      <c r="W21" s="103"/>
+      <c r="X21" s="103"/>
+      <c r="Y21" s="103"/>
       <c r="Z21" s="51"/>
       <c r="AA21" s="51"/>
       <c r="AB21" s="43"/>
@@ -4919,16 +4922,16 @@
       <c r="R22" s="86" t="s">
         <v>639</v>
       </c>
-      <c r="S22" s="105" t="s">
+      <c r="S22" s="103" t="s">
         <v>238</v>
       </c>
-      <c r="T22" s="105"/>
-      <c r="U22" s="105"/>
-      <c r="V22" s="105"/>
-      <c r="W22" s="105"/>
-      <c r="X22" s="105"/>
-      <c r="Y22" s="105"/>
-      <c r="Z22" s="105"/>
+      <c r="T22" s="103"/>
+      <c r="U22" s="103"/>
+      <c r="V22" s="103"/>
+      <c r="W22" s="103"/>
+      <c r="X22" s="103"/>
+      <c r="Y22" s="103"/>
+      <c r="Z22" s="103"/>
       <c r="AA22" s="51"/>
       <c r="AB22" s="43"/>
       <c r="AC22" s="43"/>
@@ -5000,15 +5003,15 @@
       <c r="R23" s="86" t="s">
         <v>632</v>
       </c>
-      <c r="S23" s="105" t="s">
+      <c r="S23" s="103" t="s">
         <v>98</v>
       </c>
-      <c r="T23" s="105"/>
-      <c r="U23" s="105"/>
-      <c r="V23" s="105"/>
-      <c r="W23" s="105"/>
-      <c r="X23" s="105"/>
-      <c r="Y23" s="105"/>
+      <c r="T23" s="103"/>
+      <c r="U23" s="103"/>
+      <c r="V23" s="103"/>
+      <c r="W23" s="103"/>
+      <c r="X23" s="103"/>
+      <c r="Y23" s="103"/>
       <c r="Z23" s="51"/>
       <c r="AA23" s="51"/>
       <c r="AB23" s="43"/>
@@ -5081,15 +5084,15 @@
       <c r="R24" s="86" t="s">
         <v>641</v>
       </c>
-      <c r="S24" s="110" t="s">
+      <c r="S24" s="106" t="s">
         <v>240</v>
       </c>
-      <c r="T24" s="110"/>
-      <c r="U24" s="110"/>
-      <c r="V24" s="110"/>
-      <c r="W24" s="110"/>
-      <c r="X24" s="110"/>
-      <c r="Y24" s="110"/>
+      <c r="T24" s="106"/>
+      <c r="U24" s="106"/>
+      <c r="V24" s="106"/>
+      <c r="W24" s="106"/>
+      <c r="X24" s="106"/>
+      <c r="Y24" s="106"/>
       <c r="Z24" s="50"/>
       <c r="AA24" s="50"/>
       <c r="AB24" s="43"/>
@@ -5162,15 +5165,15 @@
       <c r="R25" s="86" t="s">
         <v>668</v>
       </c>
-      <c r="S25" s="110" t="s">
+      <c r="S25" s="106" t="s">
         <v>112</v>
       </c>
-      <c r="T25" s="110"/>
-      <c r="U25" s="110"/>
-      <c r="V25" s="110"/>
-      <c r="W25" s="110"/>
-      <c r="X25" s="110"/>
-      <c r="Y25" s="110"/>
+      <c r="T25" s="106"/>
+      <c r="U25" s="106"/>
+      <c r="V25" s="106"/>
+      <c r="W25" s="106"/>
+      <c r="X25" s="106"/>
+      <c r="Y25" s="106"/>
       <c r="Z25" s="50"/>
       <c r="AA25" s="50"/>
       <c r="AB25" s="43"/>
@@ -5243,15 +5246,15 @@
       <c r="R26" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S26" s="110" t="s">
+      <c r="S26" s="106" t="s">
         <v>108</v>
       </c>
-      <c r="T26" s="110"/>
-      <c r="U26" s="110"/>
-      <c r="V26" s="110"/>
-      <c r="W26" s="110"/>
-      <c r="X26" s="110"/>
-      <c r="Y26" s="110"/>
+      <c r="T26" s="106"/>
+      <c r="U26" s="106"/>
+      <c r="V26" s="106"/>
+      <c r="W26" s="106"/>
+      <c r="X26" s="106"/>
+      <c r="Y26" s="106"/>
       <c r="Z26" s="50"/>
       <c r="AA26" s="50"/>
       <c r="AB26" s="43"/>
@@ -5324,16 +5327,16 @@
       <c r="R27" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S27" s="110" t="s">
+      <c r="S27" s="106" t="s">
         <v>243</v>
       </c>
-      <c r="T27" s="110"/>
-      <c r="U27" s="110"/>
-      <c r="V27" s="110"/>
-      <c r="W27" s="110"/>
-      <c r="X27" s="110"/>
-      <c r="Y27" s="110"/>
-      <c r="Z27" s="110"/>
+      <c r="T27" s="106"/>
+      <c r="U27" s="106"/>
+      <c r="V27" s="106"/>
+      <c r="W27" s="106"/>
+      <c r="X27" s="106"/>
+      <c r="Y27" s="106"/>
+      <c r="Z27" s="106"/>
       <c r="AA27" s="50"/>
       <c r="AB27" s="43"/>
       <c r="AC27" s="43"/>
@@ -5405,16 +5408,16 @@
       <c r="R28" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S28" s="110" t="s">
+      <c r="S28" s="106" t="s">
         <v>245</v>
       </c>
-      <c r="T28" s="110"/>
-      <c r="U28" s="110"/>
-      <c r="V28" s="110"/>
-      <c r="W28" s="110"/>
-      <c r="X28" s="110"/>
-      <c r="Y28" s="110"/>
-      <c r="Z28" s="110"/>
+      <c r="T28" s="106"/>
+      <c r="U28" s="106"/>
+      <c r="V28" s="106"/>
+      <c r="W28" s="106"/>
+      <c r="X28" s="106"/>
+      <c r="Y28" s="106"/>
+      <c r="Z28" s="106"/>
       <c r="AA28" s="50"/>
       <c r="AB28" s="43"/>
       <c r="AC28" s="43"/>
@@ -5486,16 +5489,16 @@
       <c r="R29" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S29" s="110" t="s">
+      <c r="S29" s="106" t="s">
         <v>247</v>
       </c>
-      <c r="T29" s="110"/>
-      <c r="U29" s="110"/>
-      <c r="V29" s="110"/>
-      <c r="W29" s="110"/>
-      <c r="X29" s="110"/>
-      <c r="Y29" s="110"/>
-      <c r="Z29" s="110"/>
+      <c r="T29" s="106"/>
+      <c r="U29" s="106"/>
+      <c r="V29" s="106"/>
+      <c r="W29" s="106"/>
+      <c r="X29" s="106"/>
+      <c r="Y29" s="106"/>
+      <c r="Z29" s="106"/>
       <c r="AA29" s="50"/>
       <c r="AB29" s="43"/>
       <c r="AC29" s="43"/>
@@ -5567,15 +5570,15 @@
       <c r="R30" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S30" s="110" t="s">
+      <c r="S30" s="106" t="s">
         <v>249</v>
       </c>
-      <c r="T30" s="110"/>
-      <c r="U30" s="110"/>
-      <c r="V30" s="110"/>
-      <c r="W30" s="110"/>
-      <c r="X30" s="110"/>
-      <c r="Y30" s="110"/>
+      <c r="T30" s="106"/>
+      <c r="U30" s="106"/>
+      <c r="V30" s="106"/>
+      <c r="W30" s="106"/>
+      <c r="X30" s="106"/>
+      <c r="Y30" s="106"/>
       <c r="Z30" s="50"/>
       <c r="AA30" s="50"/>
       <c r="AB30" s="43"/>
@@ -5648,16 +5651,16 @@
       <c r="R31" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S31" s="111" t="s">
+      <c r="S31" s="109" t="s">
         <v>115</v>
       </c>
-      <c r="T31" s="111"/>
-      <c r="U31" s="111"/>
-      <c r="V31" s="111"/>
-      <c r="W31" s="111"/>
-      <c r="X31" s="111"/>
-      <c r="Y31" s="111"/>
-      <c r="Z31" s="111"/>
+      <c r="T31" s="109"/>
+      <c r="U31" s="109"/>
+      <c r="V31" s="109"/>
+      <c r="W31" s="109"/>
+      <c r="X31" s="109"/>
+      <c r="Y31" s="109"/>
+      <c r="Z31" s="109"/>
       <c r="AA31" s="52"/>
       <c r="AB31" s="43"/>
       <c r="AC31" s="43"/>
@@ -5725,15 +5728,15 @@
         <v>706</v>
       </c>
       <c r="R32" s="86"/>
-      <c r="S32" s="109" t="s">
+      <c r="S32" s="110" t="s">
         <v>252</v>
       </c>
-      <c r="T32" s="109"/>
-      <c r="U32" s="109"/>
-      <c r="V32" s="109"/>
-      <c r="W32" s="109"/>
-      <c r="X32" s="109"/>
-      <c r="Y32" s="109"/>
+      <c r="T32" s="110"/>
+      <c r="U32" s="110"/>
+      <c r="V32" s="110"/>
+      <c r="W32" s="110"/>
+      <c r="X32" s="110"/>
+      <c r="Y32" s="110"/>
       <c r="Z32" s="53"/>
       <c r="AA32" s="53"/>
       <c r="AB32" s="43"/>
@@ -5771,10 +5774,10 @@
       <c r="G33" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="H33" s="109" t="s">
+      <c r="H33" s="110" t="s">
         <v>7</v>
       </c>
-      <c r="I33" s="109"/>
+      <c r="I33" s="110"/>
       <c r="J33" s="53" t="s">
         <v>213</v>
       </c>
@@ -5802,16 +5805,16 @@
       <c r="R33" s="86" t="s">
         <v>708</v>
       </c>
-      <c r="S33" s="109" t="s">
+      <c r="S33" s="110" t="s">
         <v>253</v>
       </c>
-      <c r="T33" s="109"/>
-      <c r="U33" s="109"/>
-      <c r="V33" s="109"/>
-      <c r="W33" s="109"/>
-      <c r="X33" s="109"/>
-      <c r="Y33" s="109"/>
-      <c r="Z33" s="109"/>
+      <c r="T33" s="110"/>
+      <c r="U33" s="110"/>
+      <c r="V33" s="110"/>
+      <c r="W33" s="110"/>
+      <c r="X33" s="110"/>
+      <c r="Y33" s="110"/>
+      <c r="Z33" s="110"/>
       <c r="AA33" s="53"/>
       <c r="AB33" s="43"/>
       <c r="AC33" s="43"/>
@@ -5881,15 +5884,15 @@
       <c r="R34" s="86" t="s">
         <v>708</v>
       </c>
-      <c r="S34" s="109" t="s">
+      <c r="S34" s="110" t="s">
         <v>254</v>
       </c>
-      <c r="T34" s="109"/>
-      <c r="U34" s="109"/>
-      <c r="V34" s="109"/>
-      <c r="W34" s="109"/>
-      <c r="X34" s="109"/>
-      <c r="Y34" s="109"/>
+      <c r="T34" s="110"/>
+      <c r="U34" s="110"/>
+      <c r="V34" s="110"/>
+      <c r="W34" s="110"/>
+      <c r="X34" s="110"/>
+      <c r="Y34" s="110"/>
       <c r="Z34" s="53"/>
       <c r="AA34" s="53"/>
       <c r="AB34" s="43"/>
@@ -5958,15 +5961,15 @@
         <v>709</v>
       </c>
       <c r="R35" s="86"/>
-      <c r="S35" s="109" t="s">
+      <c r="S35" s="110" t="s">
         <v>255</v>
       </c>
-      <c r="T35" s="109"/>
-      <c r="U35" s="109"/>
-      <c r="V35" s="109"/>
-      <c r="W35" s="109"/>
-      <c r="X35" s="109"/>
-      <c r="Y35" s="109"/>
+      <c r="T35" s="110"/>
+      <c r="U35" s="110"/>
+      <c r="V35" s="110"/>
+      <c r="W35" s="110"/>
+      <c r="X35" s="110"/>
+      <c r="Y35" s="110"/>
       <c r="Z35" s="53"/>
       <c r="AA35" s="53"/>
       <c r="AB35" s="43"/>
@@ -6037,14 +6040,14 @@
       <c r="R36" s="86" t="s">
         <v>712</v>
       </c>
-      <c r="S36" s="109" t="s">
+      <c r="S36" s="110" t="s">
         <v>256</v>
       </c>
-      <c r="T36" s="109"/>
-      <c r="U36" s="109"/>
-      <c r="V36" s="109"/>
-      <c r="W36" s="109"/>
-      <c r="X36" s="109"/>
+      <c r="T36" s="110"/>
+      <c r="U36" s="110"/>
+      <c r="V36" s="110"/>
+      <c r="W36" s="110"/>
+      <c r="X36" s="110"/>
       <c r="Y36" s="53"/>
       <c r="Z36" s="53"/>
       <c r="AA36" s="53"/>
@@ -6114,16 +6117,16 @@
         <v>689</v>
       </c>
       <c r="R37" s="86"/>
-      <c r="S37" s="109" t="s">
+      <c r="S37" s="110" t="s">
         <v>257</v>
       </c>
-      <c r="T37" s="109"/>
-      <c r="U37" s="109"/>
-      <c r="V37" s="109"/>
-      <c r="W37" s="109"/>
-      <c r="X37" s="109"/>
-      <c r="Y37" s="109"/>
-      <c r="Z37" s="109"/>
+      <c r="T37" s="110"/>
+      <c r="U37" s="110"/>
+      <c r="V37" s="110"/>
+      <c r="W37" s="110"/>
+      <c r="X37" s="110"/>
+      <c r="Y37" s="110"/>
+      <c r="Z37" s="110"/>
       <c r="AA37" s="53"/>
       <c r="AB37" s="43"/>
       <c r="AC37" s="43"/>
@@ -6191,17 +6194,17 @@
         <v>689</v>
       </c>
       <c r="R38" s="86"/>
-      <c r="S38" s="109" t="s">
+      <c r="S38" s="110" t="s">
         <v>258</v>
       </c>
-      <c r="T38" s="109"/>
-      <c r="U38" s="109"/>
-      <c r="V38" s="109"/>
-      <c r="W38" s="109"/>
-      <c r="X38" s="109"/>
-      <c r="Y38" s="109"/>
-      <c r="Z38" s="109"/>
-      <c r="AA38" s="109"/>
+      <c r="T38" s="110"/>
+      <c r="U38" s="110"/>
+      <c r="V38" s="110"/>
+      <c r="W38" s="110"/>
+      <c r="X38" s="110"/>
+      <c r="Y38" s="110"/>
+      <c r="Z38" s="110"/>
+      <c r="AA38" s="110"/>
       <c r="AB38" s="43"/>
       <c r="AC38" s="43"/>
       <c r="AD38" s="43"/>
@@ -6272,14 +6275,14 @@
       <c r="R39" s="86" t="s">
         <v>715</v>
       </c>
-      <c r="S39" s="108" t="s">
+      <c r="S39" s="107" t="s">
         <v>166</v>
       </c>
-      <c r="T39" s="108"/>
-      <c r="U39" s="108"/>
-      <c r="V39" s="108"/>
-      <c r="W39" s="108"/>
-      <c r="X39" s="108"/>
+      <c r="T39" s="107"/>
+      <c r="U39" s="107"/>
+      <c r="V39" s="107"/>
+      <c r="W39" s="107"/>
+      <c r="X39" s="107"/>
       <c r="Y39" s="54"/>
       <c r="Z39" s="54"/>
       <c r="AA39" s="54"/>
@@ -6353,14 +6356,14 @@
       <c r="R40" s="86" t="s">
         <v>624</v>
       </c>
-      <c r="S40" s="108" t="s">
+      <c r="S40" s="107" t="s">
         <v>263</v>
       </c>
-      <c r="T40" s="108"/>
-      <c r="U40" s="108"/>
-      <c r="V40" s="108"/>
-      <c r="W40" s="108"/>
-      <c r="X40" s="108"/>
+      <c r="T40" s="107"/>
+      <c r="U40" s="107"/>
+      <c r="V40" s="107"/>
+      <c r="W40" s="107"/>
+      <c r="X40" s="107"/>
       <c r="Y40" s="54"/>
       <c r="Z40" s="54"/>
       <c r="AA40" s="54"/>
@@ -6432,16 +6435,16 @@
       <c r="R41" s="86" t="s">
         <v>719</v>
       </c>
-      <c r="S41" s="108" t="s">
+      <c r="S41" s="107" t="s">
         <v>264</v>
       </c>
-      <c r="T41" s="108"/>
-      <c r="U41" s="108"/>
-      <c r="V41" s="108"/>
-      <c r="W41" s="108"/>
-      <c r="X41" s="108"/>
-      <c r="Y41" s="108"/>
-      <c r="Z41" s="108"/>
+      <c r="T41" s="107"/>
+      <c r="U41" s="107"/>
+      <c r="V41" s="107"/>
+      <c r="W41" s="107"/>
+      <c r="X41" s="107"/>
+      <c r="Y41" s="107"/>
+      <c r="Z41" s="107"/>
       <c r="AA41" s="54"/>
       <c r="AB41" s="43"/>
       <c r="AC41" s="43"/>
@@ -6513,17 +6516,17 @@
       <c r="R42" s="86" t="s">
         <v>719</v>
       </c>
-      <c r="S42" s="108" t="s">
+      <c r="S42" s="107" t="s">
         <v>161</v>
       </c>
-      <c r="T42" s="108"/>
-      <c r="U42" s="108"/>
-      <c r="V42" s="108"/>
-      <c r="W42" s="108"/>
-      <c r="X42" s="108"/>
-      <c r="Y42" s="108"/>
-      <c r="Z42" s="108"/>
-      <c r="AA42" s="108"/>
+      <c r="T42" s="107"/>
+      <c r="U42" s="107"/>
+      <c r="V42" s="107"/>
+      <c r="W42" s="107"/>
+      <c r="X42" s="107"/>
+      <c r="Y42" s="107"/>
+      <c r="Z42" s="107"/>
+      <c r="AA42" s="107"/>
       <c r="AB42" s="43"/>
       <c r="AC42" s="43"/>
       <c r="AD42" s="43"/>
@@ -6594,16 +6597,16 @@
       <c r="R43" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S43" s="108" t="s">
+      <c r="S43" s="107" t="s">
         <v>265</v>
       </c>
-      <c r="T43" s="108"/>
-      <c r="U43" s="108"/>
-      <c r="V43" s="108"/>
-      <c r="W43" s="108"/>
-      <c r="X43" s="108"/>
-      <c r="Y43" s="108"/>
-      <c r="Z43" s="108"/>
+      <c r="T43" s="107"/>
+      <c r="U43" s="107"/>
+      <c r="V43" s="107"/>
+      <c r="W43" s="107"/>
+      <c r="X43" s="107"/>
+      <c r="Y43" s="107"/>
+      <c r="Z43" s="107"/>
       <c r="AA43" s="54"/>
       <c r="AB43" s="43"/>
       <c r="AC43" s="43"/>
@@ -6675,15 +6678,15 @@
       <c r="R44" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S44" s="108" t="s">
+      <c r="S44" s="107" t="s">
         <v>158</v>
       </c>
-      <c r="T44" s="108"/>
-      <c r="U44" s="108"/>
-      <c r="V44" s="108"/>
-      <c r="W44" s="108"/>
-      <c r="X44" s="108"/>
-      <c r="Y44" s="108"/>
+      <c r="T44" s="107"/>
+      <c r="U44" s="107"/>
+      <c r="V44" s="107"/>
+      <c r="W44" s="107"/>
+      <c r="X44" s="107"/>
+      <c r="Y44" s="107"/>
       <c r="Z44" s="54"/>
       <c r="AA44" s="54"/>
       <c r="AB44" s="43"/>
@@ -6754,16 +6757,16 @@
       <c r="R45" s="86" t="s">
         <v>719</v>
       </c>
-      <c r="S45" s="108" t="s">
+      <c r="S45" s="107" t="s">
         <v>266</v>
       </c>
-      <c r="T45" s="108"/>
-      <c r="U45" s="108"/>
-      <c r="V45" s="108"/>
-      <c r="W45" s="108"/>
-      <c r="X45" s="108"/>
-      <c r="Y45" s="108"/>
-      <c r="Z45" s="108"/>
+      <c r="T45" s="107"/>
+      <c r="U45" s="107"/>
+      <c r="V45" s="107"/>
+      <c r="W45" s="107"/>
+      <c r="X45" s="107"/>
+      <c r="Y45" s="107"/>
+      <c r="Z45" s="107"/>
       <c r="AA45" s="54"/>
       <c r="AB45" s="43"/>
       <c r="AC45" s="43"/>
@@ -6831,14 +6834,14 @@
       <c r="R46" s="86" t="s">
         <v>632</v>
       </c>
-      <c r="S46" s="108" t="s">
+      <c r="S46" s="107" t="s">
         <v>132</v>
       </c>
-      <c r="T46" s="108"/>
-      <c r="U46" s="108"/>
-      <c r="V46" s="108"/>
-      <c r="W46" s="108"/>
-      <c r="X46" s="108"/>
+      <c r="T46" s="107"/>
+      <c r="U46" s="107"/>
+      <c r="V46" s="107"/>
+      <c r="W46" s="107"/>
+      <c r="X46" s="107"/>
       <c r="Y46" s="54"/>
       <c r="Z46" s="54"/>
       <c r="AA46" s="54"/>
@@ -6912,15 +6915,15 @@
       <c r="R47" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S47" s="108" t="s">
+      <c r="S47" s="107" t="s">
         <v>136</v>
       </c>
-      <c r="T47" s="108"/>
-      <c r="U47" s="108"/>
-      <c r="V47" s="108"/>
-      <c r="W47" s="108"/>
-      <c r="X47" s="108"/>
-      <c r="Y47" s="108"/>
+      <c r="T47" s="107"/>
+      <c r="U47" s="107"/>
+      <c r="V47" s="107"/>
+      <c r="W47" s="107"/>
+      <c r="X47" s="107"/>
+      <c r="Y47" s="107"/>
       <c r="Z47" s="54"/>
       <c r="AA47" s="54"/>
       <c r="AB47" s="43"/>
@@ -6993,16 +6996,16 @@
       <c r="R48" s="86" t="s">
         <v>636</v>
       </c>
-      <c r="S48" s="108" t="s">
+      <c r="S48" s="107" t="s">
         <v>178</v>
       </c>
-      <c r="T48" s="108"/>
-      <c r="U48" s="108"/>
-      <c r="V48" s="108"/>
-      <c r="W48" s="108"/>
-      <c r="X48" s="108"/>
-      <c r="Y48" s="108"/>
-      <c r="Z48" s="108"/>
+      <c r="T48" s="107"/>
+      <c r="U48" s="107"/>
+      <c r="V48" s="107"/>
+      <c r="W48" s="107"/>
+      <c r="X48" s="107"/>
+      <c r="Y48" s="107"/>
+      <c r="Z48" s="107"/>
       <c r="AA48" s="54"/>
       <c r="AB48" s="43"/>
       <c r="AC48" s="43"/>
@@ -7074,17 +7077,17 @@
       <c r="R49" s="86" t="s">
         <v>730</v>
       </c>
-      <c r="S49" s="108" t="s">
+      <c r="S49" s="107" t="s">
         <v>268</v>
       </c>
-      <c r="T49" s="108"/>
-      <c r="U49" s="108"/>
-      <c r="V49" s="108"/>
-      <c r="W49" s="108"/>
-      <c r="X49" s="108"/>
-      <c r="Y49" s="108"/>
-      <c r="Z49" s="108"/>
-      <c r="AA49" s="108"/>
+      <c r="T49" s="107"/>
+      <c r="U49" s="107"/>
+      <c r="V49" s="107"/>
+      <c r="W49" s="107"/>
+      <c r="X49" s="107"/>
+      <c r="Y49" s="107"/>
+      <c r="Z49" s="107"/>
+      <c r="AA49" s="107"/>
       <c r="AB49" s="43"/>
       <c r="AC49" s="43"/>
       <c r="AD49" s="43"/>
@@ -7155,15 +7158,15 @@
       <c r="R50" s="86" t="s">
         <v>730</v>
       </c>
-      <c r="S50" s="108" t="s">
+      <c r="S50" s="107" t="s">
         <v>269</v>
       </c>
-      <c r="T50" s="108"/>
-      <c r="U50" s="108"/>
-      <c r="V50" s="108"/>
-      <c r="W50" s="108"/>
-      <c r="X50" s="108"/>
-      <c r="Y50" s="108"/>
+      <c r="T50" s="107"/>
+      <c r="U50" s="107"/>
+      <c r="V50" s="107"/>
+      <c r="W50" s="107"/>
+      <c r="X50" s="107"/>
+      <c r="Y50" s="107"/>
       <c r="Z50" s="54"/>
       <c r="AA50" s="54"/>
       <c r="AB50" s="43"/>
@@ -7232,16 +7235,16 @@
       <c r="R51" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S51" s="108" t="s">
+      <c r="S51" s="107" t="s">
         <v>170</v>
       </c>
-      <c r="T51" s="108"/>
-      <c r="U51" s="108"/>
-      <c r="V51" s="108"/>
-      <c r="W51" s="108"/>
-      <c r="X51" s="108"/>
-      <c r="Y51" s="108"/>
-      <c r="Z51" s="108"/>
+      <c r="T51" s="107"/>
+      <c r="U51" s="107"/>
+      <c r="V51" s="107"/>
+      <c r="W51" s="107"/>
+      <c r="X51" s="107"/>
+      <c r="Y51" s="107"/>
+      <c r="Z51" s="107"/>
       <c r="AA51" s="54"/>
       <c r="AB51" s="43"/>
       <c r="AC51" s="43"/>
@@ -7311,16 +7314,16 @@
       <c r="R52" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S52" s="102" t="s">
+      <c r="S52" s="104" t="s">
         <v>130</v>
       </c>
-      <c r="T52" s="102"/>
-      <c r="U52" s="102"/>
-      <c r="V52" s="102"/>
-      <c r="W52" s="102"/>
-      <c r="X52" s="102"/>
-      <c r="Y52" s="102"/>
-      <c r="Z52" s="102"/>
+      <c r="T52" s="104"/>
+      <c r="U52" s="104"/>
+      <c r="V52" s="104"/>
+      <c r="W52" s="104"/>
+      <c r="X52" s="104"/>
+      <c r="Y52" s="104"/>
+      <c r="Z52" s="104"/>
       <c r="AA52" s="43"/>
       <c r="AB52" s="43"/>
       <c r="AC52" s="43"/>
@@ -7390,16 +7393,16 @@
       <c r="R53" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S53" s="102" t="s">
+      <c r="S53" s="104" t="s">
         <v>272</v>
       </c>
-      <c r="T53" s="102"/>
-      <c r="U53" s="102"/>
-      <c r="V53" s="102"/>
-      <c r="W53" s="102"/>
-      <c r="X53" s="102"/>
-      <c r="Y53" s="102"/>
-      <c r="Z53" s="102"/>
+      <c r="T53" s="104"/>
+      <c r="U53" s="104"/>
+      <c r="V53" s="104"/>
+      <c r="W53" s="104"/>
+      <c r="X53" s="104"/>
+      <c r="Y53" s="104"/>
+      <c r="Z53" s="104"/>
       <c r="AA53" s="43"/>
       <c r="AB53" s="43"/>
       <c r="AC53" s="43"/>
@@ -7467,15 +7470,15 @@
       <c r="R54" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S54" s="102" t="s">
+      <c r="S54" s="104" t="s">
         <v>145</v>
       </c>
-      <c r="T54" s="102"/>
-      <c r="U54" s="102"/>
-      <c r="V54" s="102"/>
-      <c r="W54" s="102"/>
-      <c r="X54" s="102"/>
-      <c r="Y54" s="102"/>
+      <c r="T54" s="104"/>
+      <c r="U54" s="104"/>
+      <c r="V54" s="104"/>
+      <c r="W54" s="104"/>
+      <c r="X54" s="104"/>
+      <c r="Y54" s="104"/>
       <c r="Z54" s="43"/>
       <c r="AA54" s="43"/>
       <c r="AB54" s="43"/>
@@ -7548,16 +7551,16 @@
       <c r="R55" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S55" s="107" t="s">
+      <c r="S55" s="112" t="s">
         <v>260</v>
       </c>
-      <c r="T55" s="107"/>
-      <c r="U55" s="107"/>
-      <c r="V55" s="107"/>
-      <c r="W55" s="107"/>
-      <c r="X55" s="107"/>
-      <c r="Y55" s="107"/>
-      <c r="Z55" s="107"/>
+      <c r="T55" s="112"/>
+      <c r="U55" s="112"/>
+      <c r="V55" s="112"/>
+      <c r="W55" s="112"/>
+      <c r="X55" s="112"/>
+      <c r="Y55" s="112"/>
+      <c r="Z55" s="112"/>
       <c r="AA55" s="75"/>
       <c r="AB55" s="75"/>
       <c r="AC55" s="75"/>
@@ -7629,14 +7632,14 @@
       <c r="R56" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S56" s="107" t="s">
+      <c r="S56" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="T56" s="107"/>
-      <c r="U56" s="107"/>
-      <c r="V56" s="107"/>
-      <c r="W56" s="107"/>
-      <c r="X56" s="107"/>
+      <c r="T56" s="112"/>
+      <c r="U56" s="112"/>
+      <c r="V56" s="112"/>
+      <c r="W56" s="112"/>
+      <c r="X56" s="112"/>
       <c r="Y56" s="75"/>
       <c r="Z56" s="75"/>
       <c r="AA56" s="75"/>
@@ -7710,14 +7713,14 @@
       <c r="R57" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S57" s="107" t="s">
+      <c r="S57" s="112" t="s">
         <v>276</v>
       </c>
-      <c r="T57" s="107"/>
-      <c r="U57" s="107"/>
-      <c r="V57" s="107"/>
-      <c r="W57" s="107"/>
-      <c r="X57" s="107"/>
+      <c r="T57" s="112"/>
+      <c r="U57" s="112"/>
+      <c r="V57" s="112"/>
+      <c r="W57" s="112"/>
+      <c r="X57" s="112"/>
       <c r="Y57" s="75"/>
       <c r="Z57" s="75"/>
       <c r="AA57" s="75"/>
@@ -7791,14 +7794,14 @@
       <c r="R58" s="86" t="s">
         <v>753</v>
       </c>
-      <c r="S58" s="107" t="s">
+      <c r="S58" s="112" t="s">
         <v>278</v>
       </c>
-      <c r="T58" s="107"/>
-      <c r="U58" s="107"/>
-      <c r="V58" s="107"/>
-      <c r="W58" s="107"/>
-      <c r="X58" s="107"/>
+      <c r="T58" s="112"/>
+      <c r="U58" s="112"/>
+      <c r="V58" s="112"/>
+      <c r="W58" s="112"/>
+      <c r="X58" s="112"/>
       <c r="Y58" s="75"/>
       <c r="Z58" s="75"/>
       <c r="AA58" s="75"/>
@@ -7872,15 +7875,15 @@
       <c r="R59" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S59" s="107" t="s">
+      <c r="S59" s="112" t="s">
         <v>68</v>
       </c>
-      <c r="T59" s="107"/>
-      <c r="U59" s="107"/>
-      <c r="V59" s="107"/>
-      <c r="W59" s="107"/>
-      <c r="X59" s="107"/>
-      <c r="Y59" s="107"/>
+      <c r="T59" s="112"/>
+      <c r="U59" s="112"/>
+      <c r="V59" s="112"/>
+      <c r="W59" s="112"/>
+      <c r="X59" s="112"/>
+      <c r="Y59" s="112"/>
       <c r="Z59" s="75"/>
       <c r="AA59" s="75"/>
       <c r="AB59" s="75"/>
@@ -7953,14 +7956,14 @@
       <c r="R60" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S60" s="107" t="s">
+      <c r="S60" s="112" t="s">
         <v>126</v>
       </c>
-      <c r="T60" s="107"/>
-      <c r="U60" s="107"/>
-      <c r="V60" s="107"/>
-      <c r="W60" s="107"/>
-      <c r="X60" s="107"/>
+      <c r="T60" s="112"/>
+      <c r="U60" s="112"/>
+      <c r="V60" s="112"/>
+      <c r="W60" s="112"/>
+      <c r="X60" s="112"/>
       <c r="Y60" s="75"/>
       <c r="Z60" s="75"/>
       <c r="AA60" s="75"/>
@@ -8034,15 +8037,15 @@
       <c r="R61" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S61" s="102" t="s">
+      <c r="S61" s="104" t="s">
         <v>281</v>
       </c>
-      <c r="T61" s="102"/>
-      <c r="U61" s="102"/>
-      <c r="V61" s="102"/>
-      <c r="W61" s="102"/>
-      <c r="X61" s="102"/>
-      <c r="Y61" s="102"/>
+      <c r="T61" s="104"/>
+      <c r="U61" s="104"/>
+      <c r="V61" s="104"/>
+      <c r="W61" s="104"/>
+      <c r="X61" s="104"/>
+      <c r="Y61" s="104"/>
       <c r="Z61" s="43"/>
       <c r="AA61" s="43"/>
       <c r="AB61" s="43"/>
@@ -8115,16 +8118,16 @@
       <c r="R62" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S62" s="102" t="s">
+      <c r="S62" s="104" t="s">
         <v>282</v>
       </c>
-      <c r="T62" s="102"/>
-      <c r="U62" s="102"/>
-      <c r="V62" s="102"/>
-      <c r="W62" s="102"/>
-      <c r="X62" s="102"/>
-      <c r="Y62" s="102"/>
-      <c r="Z62" s="102"/>
+      <c r="T62" s="104"/>
+      <c r="U62" s="104"/>
+      <c r="V62" s="104"/>
+      <c r="W62" s="104"/>
+      <c r="X62" s="104"/>
+      <c r="Y62" s="104"/>
+      <c r="Z62" s="104"/>
       <c r="AA62" s="43"/>
       <c r="AB62" s="43"/>
       <c r="AC62" s="43"/>
@@ -8196,15 +8199,15 @@
       <c r="R63" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S63" s="102" t="s">
+      <c r="S63" s="104" t="s">
         <v>284</v>
       </c>
-      <c r="T63" s="102"/>
-      <c r="U63" s="102"/>
-      <c r="V63" s="102"/>
-      <c r="W63" s="102"/>
-      <c r="X63" s="102"/>
-      <c r="Y63" s="102"/>
+      <c r="T63" s="104"/>
+      <c r="U63" s="104"/>
+      <c r="V63" s="104"/>
+      <c r="W63" s="104"/>
+      <c r="X63" s="104"/>
+      <c r="Y63" s="104"/>
       <c r="Z63" s="43"/>
       <c r="AA63" s="43"/>
       <c r="AB63" s="43"/>
@@ -8277,15 +8280,15 @@
       <c r="R64" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S64" s="102" t="s">
+      <c r="S64" s="104" t="s">
         <v>70</v>
       </c>
-      <c r="T64" s="102"/>
-      <c r="U64" s="102"/>
-      <c r="V64" s="102"/>
-      <c r="W64" s="102"/>
-      <c r="X64" s="102"/>
-      <c r="Y64" s="102"/>
+      <c r="T64" s="104"/>
+      <c r="U64" s="104"/>
+      <c r="V64" s="104"/>
+      <c r="W64" s="104"/>
+      <c r="X64" s="104"/>
+      <c r="Y64" s="104"/>
       <c r="Z64" s="43"/>
       <c r="AA64" s="43"/>
       <c r="AB64" s="43"/>
@@ -8358,16 +8361,16 @@
       <c r="R65" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S65" s="102" t="s">
+      <c r="S65" s="104" t="s">
         <v>286</v>
       </c>
-      <c r="T65" s="102"/>
-      <c r="U65" s="102"/>
-      <c r="V65" s="102"/>
-      <c r="W65" s="102"/>
-      <c r="X65" s="102"/>
-      <c r="Y65" s="102"/>
-      <c r="Z65" s="102"/>
+      <c r="T65" s="104"/>
+      <c r="U65" s="104"/>
+      <c r="V65" s="104"/>
+      <c r="W65" s="104"/>
+      <c r="X65" s="104"/>
+      <c r="Y65" s="104"/>
+      <c r="Z65" s="104"/>
       <c r="AA65" s="43"/>
       <c r="AB65" s="43"/>
       <c r="AC65" s="43"/>
@@ -8439,16 +8442,16 @@
       <c r="R66" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S66" s="102" t="s">
+      <c r="S66" s="104" t="s">
         <v>287</v>
       </c>
-      <c r="T66" s="102"/>
-      <c r="U66" s="102"/>
-      <c r="V66" s="102"/>
-      <c r="W66" s="102"/>
-      <c r="X66" s="102"/>
-      <c r="Y66" s="102"/>
-      <c r="Z66" s="102"/>
+      <c r="T66" s="104"/>
+      <c r="U66" s="104"/>
+      <c r="V66" s="104"/>
+      <c r="W66" s="104"/>
+      <c r="X66" s="104"/>
+      <c r="Y66" s="104"/>
+      <c r="Z66" s="104"/>
       <c r="AA66" s="43"/>
       <c r="AB66" s="43"/>
       <c r="AC66" s="43"/>
@@ -8520,16 +8523,16 @@
       <c r="R67" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S67" s="103" t="s">
+      <c r="S67" s="113" t="s">
         <v>288</v>
       </c>
-      <c r="T67" s="103"/>
-      <c r="U67" s="103"/>
-      <c r="V67" s="103"/>
-      <c r="W67" s="103"/>
-      <c r="X67" s="103"/>
-      <c r="Y67" s="103"/>
-      <c r="Z67" s="103"/>
+      <c r="T67" s="113"/>
+      <c r="U67" s="113"/>
+      <c r="V67" s="113"/>
+      <c r="W67" s="113"/>
+      <c r="X67" s="113"/>
+      <c r="Y67" s="113"/>
+      <c r="Z67" s="113"/>
       <c r="AA67" s="82"/>
       <c r="AB67" s="82"/>
       <c r="AC67" s="82"/>
@@ -8601,16 +8604,16 @@
       <c r="R68" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S68" s="103" t="s">
+      <c r="S68" s="113" t="s">
         <v>288</v>
       </c>
-      <c r="T68" s="103"/>
-      <c r="U68" s="103"/>
-      <c r="V68" s="103"/>
-      <c r="W68" s="103"/>
-      <c r="X68" s="103"/>
-      <c r="Y68" s="103"/>
-      <c r="Z68" s="103"/>
+      <c r="T68" s="113"/>
+      <c r="U68" s="113"/>
+      <c r="V68" s="113"/>
+      <c r="W68" s="113"/>
+      <c r="X68" s="113"/>
+      <c r="Y68" s="113"/>
+      <c r="Z68" s="113"/>
       <c r="AA68" s="82"/>
       <c r="AB68" s="82"/>
       <c r="AC68" s="82"/>
@@ -8682,16 +8685,16 @@
       <c r="R69" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S69" s="103" t="s">
+      <c r="S69" s="113" t="s">
         <v>289</v>
       </c>
-      <c r="T69" s="103"/>
-      <c r="U69" s="103"/>
-      <c r="V69" s="103"/>
-      <c r="W69" s="103"/>
-      <c r="X69" s="103"/>
-      <c r="Y69" s="103"/>
-      <c r="Z69" s="103"/>
+      <c r="T69" s="113"/>
+      <c r="U69" s="113"/>
+      <c r="V69" s="113"/>
+      <c r="W69" s="113"/>
+      <c r="X69" s="113"/>
+      <c r="Y69" s="113"/>
+      <c r="Z69" s="113"/>
       <c r="AA69" s="82"/>
       <c r="AB69" s="82"/>
       <c r="AC69" s="82"/>
@@ -8755,15 +8758,15 @@
         <v>748</v>
       </c>
       <c r="R70" s="86"/>
-      <c r="S70" s="102" t="s">
+      <c r="S70" s="104" t="s">
         <v>75</v>
       </c>
-      <c r="T70" s="102"/>
-      <c r="U70" s="102"/>
-      <c r="V70" s="102"/>
-      <c r="W70" s="102"/>
-      <c r="X70" s="102"/>
-      <c r="Y70" s="102"/>
+      <c r="T70" s="104"/>
+      <c r="U70" s="104"/>
+      <c r="V70" s="104"/>
+      <c r="W70" s="104"/>
+      <c r="X70" s="104"/>
+      <c r="Y70" s="104"/>
       <c r="Z70" s="43"/>
       <c r="AA70" s="43"/>
       <c r="AB70" s="43"/>
@@ -8828,14 +8831,14 @@
         <v>748</v>
       </c>
       <c r="R71" s="86"/>
-      <c r="S71" s="102" t="s">
+      <c r="S71" s="104" t="s">
         <v>89</v>
       </c>
-      <c r="T71" s="102"/>
-      <c r="U71" s="102"/>
-      <c r="V71" s="102"/>
-      <c r="W71" s="102"/>
-      <c r="X71" s="102"/>
+      <c r="T71" s="104"/>
+      <c r="U71" s="104"/>
+      <c r="V71" s="104"/>
+      <c r="W71" s="104"/>
+      <c r="X71" s="104"/>
       <c r="Y71" s="43"/>
       <c r="Z71" s="43"/>
       <c r="AA71" s="43"/>
@@ -8905,16 +8908,16 @@
       <c r="R72" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S72" s="105" t="s">
+      <c r="S72" s="103" t="s">
         <v>91</v>
       </c>
-      <c r="T72" s="105"/>
-      <c r="U72" s="105"/>
-      <c r="V72" s="105"/>
-      <c r="W72" s="105"/>
-      <c r="X72" s="105"/>
-      <c r="Y72" s="105"/>
-      <c r="Z72" s="105"/>
+      <c r="T72" s="103"/>
+      <c r="U72" s="103"/>
+      <c r="V72" s="103"/>
+      <c r="W72" s="103"/>
+      <c r="X72" s="103"/>
+      <c r="Y72" s="103"/>
+      <c r="Z72" s="103"/>
       <c r="AA72" s="51"/>
       <c r="AB72" s="43"/>
       <c r="AC72" s="43"/>
@@ -8953,10 +8956,10 @@
       <c r="G73" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="H73" s="105" t="s">
+      <c r="H73" s="103" t="s">
         <v>10</v>
       </c>
-      <c r="I73" s="105"/>
+      <c r="I73" s="103"/>
       <c r="J73" s="51" t="s">
         <v>213</v>
       </c>
@@ -8984,15 +8987,15 @@
       <c r="R73" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S73" s="105" t="s">
+      <c r="S73" s="103" t="s">
         <v>293</v>
       </c>
-      <c r="T73" s="105"/>
-      <c r="U73" s="105"/>
-      <c r="V73" s="105"/>
-      <c r="W73" s="105"/>
-      <c r="X73" s="105"/>
-      <c r="Y73" s="105"/>
+      <c r="T73" s="103"/>
+      <c r="U73" s="103"/>
+      <c r="V73" s="103"/>
+      <c r="W73" s="103"/>
+      <c r="X73" s="103"/>
+      <c r="Y73" s="103"/>
       <c r="Z73" s="51"/>
       <c r="AA73" s="51"/>
       <c r="AB73" s="43"/>
@@ -9032,10 +9035,10 @@
       <c r="G74" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="H74" s="105" t="s">
+      <c r="H74" s="103" t="s">
         <v>10</v>
       </c>
-      <c r="I74" s="105"/>
+      <c r="I74" s="103"/>
       <c r="J74" s="51" t="s">
         <v>213</v>
       </c>
@@ -9063,16 +9066,16 @@
       <c r="R74" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S74" s="105" t="s">
+      <c r="S74" s="103" t="s">
         <v>106</v>
       </c>
-      <c r="T74" s="105"/>
-      <c r="U74" s="105"/>
-      <c r="V74" s="105"/>
-      <c r="W74" s="105"/>
-      <c r="X74" s="105"/>
-      <c r="Y74" s="105"/>
-      <c r="Z74" s="105"/>
+      <c r="T74" s="103"/>
+      <c r="U74" s="103"/>
+      <c r="V74" s="103"/>
+      <c r="W74" s="103"/>
+      <c r="X74" s="103"/>
+      <c r="Y74" s="103"/>
+      <c r="Z74" s="103"/>
       <c r="AA74" s="51"/>
       <c r="AB74" s="43"/>
       <c r="AC74" s="43"/>
@@ -9142,15 +9145,15 @@
       <c r="R75" s="86" t="s">
         <v>740</v>
       </c>
-      <c r="S75" s="105" t="s">
+      <c r="S75" s="103" t="s">
         <v>152</v>
       </c>
-      <c r="T75" s="105"/>
-      <c r="U75" s="105"/>
-      <c r="V75" s="105"/>
-      <c r="W75" s="105"/>
-      <c r="X75" s="105"/>
-      <c r="Y75" s="105"/>
+      <c r="T75" s="103"/>
+      <c r="U75" s="103"/>
+      <c r="V75" s="103"/>
+      <c r="W75" s="103"/>
+      <c r="X75" s="103"/>
+      <c r="Y75" s="103"/>
       <c r="Z75" s="51"/>
       <c r="AA75" s="51"/>
       <c r="AB75" s="43"/>
@@ -9190,10 +9193,10 @@
       <c r="G76" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="H76" s="105" t="s">
+      <c r="H76" s="103" t="s">
         <v>10</v>
       </c>
-      <c r="I76" s="105"/>
+      <c r="I76" s="103"/>
       <c r="J76" s="51" t="s">
         <v>213</v>
       </c>
@@ -9221,15 +9224,15 @@
       <c r="R76" s="86" t="s">
         <v>674</v>
       </c>
-      <c r="S76" s="105" t="s">
+      <c r="S76" s="103" t="s">
         <v>296</v>
       </c>
-      <c r="T76" s="105"/>
-      <c r="U76" s="105"/>
-      <c r="V76" s="105"/>
-      <c r="W76" s="105"/>
-      <c r="X76" s="105"/>
-      <c r="Y76" s="105"/>
+      <c r="T76" s="103"/>
+      <c r="U76" s="103"/>
+      <c r="V76" s="103"/>
+      <c r="W76" s="103"/>
+      <c r="X76" s="103"/>
+      <c r="Y76" s="103"/>
       <c r="Z76" s="51"/>
       <c r="AA76" s="51"/>
       <c r="AB76" s="43"/>
@@ -9302,16 +9305,16 @@
       <c r="R77" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S77" s="105" t="s">
+      <c r="S77" s="103" t="s">
         <v>297</v>
       </c>
-      <c r="T77" s="105"/>
-      <c r="U77" s="105"/>
-      <c r="V77" s="105"/>
-      <c r="W77" s="105"/>
-      <c r="X77" s="105"/>
-      <c r="Y77" s="105"/>
-      <c r="Z77" s="105"/>
+      <c r="T77" s="103"/>
+      <c r="U77" s="103"/>
+      <c r="V77" s="103"/>
+      <c r="W77" s="103"/>
+      <c r="X77" s="103"/>
+      <c r="Y77" s="103"/>
+      <c r="Z77" s="103"/>
       <c r="AA77" s="51"/>
       <c r="AB77" s="43"/>
       <c r="AC77" s="43"/>
@@ -9383,16 +9386,16 @@
       <c r="R78" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S78" s="106" t="s">
+      <c r="S78" s="111" t="s">
         <v>295</v>
       </c>
-      <c r="T78" s="106"/>
-      <c r="U78" s="106"/>
-      <c r="V78" s="106"/>
-      <c r="W78" s="106"/>
-      <c r="X78" s="106"/>
-      <c r="Y78" s="106"/>
-      <c r="Z78" s="106"/>
+      <c r="T78" s="111"/>
+      <c r="U78" s="111"/>
+      <c r="V78" s="111"/>
+      <c r="W78" s="111"/>
+      <c r="X78" s="111"/>
+      <c r="Y78" s="111"/>
+      <c r="Z78" s="111"/>
       <c r="AA78" s="44"/>
       <c r="AB78" s="43"/>
       <c r="AC78" s="43"/>
@@ -9464,14 +9467,14 @@
       <c r="R79" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S79" s="102" t="s">
+      <c r="S79" s="104" t="s">
         <v>301</v>
       </c>
-      <c r="T79" s="102"/>
-      <c r="U79" s="102"/>
-      <c r="V79" s="102"/>
-      <c r="W79" s="102"/>
-      <c r="X79" s="102"/>
+      <c r="T79" s="104"/>
+      <c r="U79" s="104"/>
+      <c r="V79" s="104"/>
+      <c r="W79" s="104"/>
+      <c r="X79" s="104"/>
       <c r="Y79" s="43"/>
       <c r="Z79" s="43"/>
       <c r="AA79" s="43"/>
@@ -9545,15 +9548,15 @@
       <c r="R80" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S80" s="102" t="s">
+      <c r="S80" s="104" t="s">
         <v>303</v>
       </c>
-      <c r="T80" s="102"/>
-      <c r="U80" s="102"/>
-      <c r="V80" s="102"/>
-      <c r="W80" s="102"/>
-      <c r="X80" s="102"/>
-      <c r="Y80" s="102"/>
+      <c r="T80" s="104"/>
+      <c r="U80" s="104"/>
+      <c r="V80" s="104"/>
+      <c r="W80" s="104"/>
+      <c r="X80" s="104"/>
+      <c r="Y80" s="104"/>
       <c r="Z80" s="43"/>
       <c r="AA80" s="43"/>
       <c r="AB80" s="43"/>
@@ -9626,13 +9629,13 @@
       <c r="R81" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S81" s="102" t="s">
+      <c r="S81" s="104" t="s">
         <v>305</v>
       </c>
-      <c r="T81" s="102"/>
-      <c r="U81" s="102"/>
-      <c r="V81" s="102"/>
-      <c r="W81" s="102"/>
+      <c r="T81" s="104"/>
+      <c r="U81" s="104"/>
+      <c r="V81" s="104"/>
+      <c r="W81" s="104"/>
       <c r="X81" s="43"/>
       <c r="Y81" s="43"/>
       <c r="Z81" s="43"/>
@@ -9707,17 +9710,17 @@
       <c r="R82" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S82" s="102" t="s">
+      <c r="S82" s="104" t="s">
         <v>307</v>
       </c>
-      <c r="T82" s="102"/>
-      <c r="U82" s="102"/>
-      <c r="V82" s="102"/>
-      <c r="W82" s="102"/>
-      <c r="X82" s="102"/>
-      <c r="Y82" s="102"/>
-      <c r="Z82" s="102"/>
-      <c r="AA82" s="102"/>
+      <c r="T82" s="104"/>
+      <c r="U82" s="104"/>
+      <c r="V82" s="104"/>
+      <c r="W82" s="104"/>
+      <c r="X82" s="104"/>
+      <c r="Y82" s="104"/>
+      <c r="Z82" s="104"/>
+      <c r="AA82" s="104"/>
       <c r="AB82" s="43"/>
       <c r="AC82" s="43"/>
       <c r="AD82" s="43"/>
@@ -9788,15 +9791,15 @@
       <c r="R83" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S83" s="102" t="s">
+      <c r="S83" s="104" t="s">
         <v>309</v>
       </c>
-      <c r="T83" s="102"/>
-      <c r="U83" s="102"/>
-      <c r="V83" s="102"/>
-      <c r="W83" s="102"/>
-      <c r="X83" s="102"/>
-      <c r="Y83" s="102"/>
+      <c r="T83" s="104"/>
+      <c r="U83" s="104"/>
+      <c r="V83" s="104"/>
+      <c r="W83" s="104"/>
+      <c r="X83" s="104"/>
+      <c r="Y83" s="104"/>
       <c r="Z83" s="43"/>
       <c r="AA83" s="43"/>
       <c r="AB83" s="43"/>
@@ -9869,14 +9872,14 @@
       <c r="R84" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S84" s="102" t="s">
+      <c r="S84" s="104" t="s">
         <v>311</v>
       </c>
-      <c r="T84" s="102"/>
-      <c r="U84" s="102"/>
-      <c r="V84" s="102"/>
-      <c r="W84" s="102"/>
-      <c r="X84" s="102"/>
+      <c r="T84" s="104"/>
+      <c r="U84" s="104"/>
+      <c r="V84" s="104"/>
+      <c r="W84" s="104"/>
+      <c r="X84" s="104"/>
       <c r="Y84" s="43"/>
       <c r="Z84" s="43"/>
       <c r="AA84" s="43"/>
@@ -9950,14 +9953,14 @@
       <c r="R85" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S85" s="102" t="s">
+      <c r="S85" s="104" t="s">
         <v>313</v>
       </c>
-      <c r="T85" s="102"/>
-      <c r="U85" s="102"/>
-      <c r="V85" s="102"/>
-      <c r="W85" s="102"/>
-      <c r="X85" s="102"/>
+      <c r="T85" s="104"/>
+      <c r="U85" s="104"/>
+      <c r="V85" s="104"/>
+      <c r="W85" s="104"/>
+      <c r="X85" s="104"/>
       <c r="Y85" s="43"/>
       <c r="Z85" s="43"/>
       <c r="AA85" s="43"/>
@@ -10031,14 +10034,14 @@
       <c r="R86" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S86" s="102" t="s">
+      <c r="S86" s="104" t="s">
         <v>315</v>
       </c>
-      <c r="T86" s="102"/>
-      <c r="U86" s="102"/>
-      <c r="V86" s="102"/>
-      <c r="W86" s="102"/>
-      <c r="X86" s="102"/>
+      <c r="T86" s="104"/>
+      <c r="U86" s="104"/>
+      <c r="V86" s="104"/>
+      <c r="W86" s="104"/>
+      <c r="X86" s="104"/>
       <c r="Y86" s="43"/>
       <c r="Z86" s="43"/>
       <c r="AA86" s="43"/>
@@ -10112,14 +10115,14 @@
       <c r="R87" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S87" s="102" t="s">
+      <c r="S87" s="104" t="s">
         <v>317</v>
       </c>
-      <c r="T87" s="102"/>
-      <c r="U87" s="102"/>
-      <c r="V87" s="102"/>
-      <c r="W87" s="102"/>
-      <c r="X87" s="102"/>
+      <c r="T87" s="104"/>
+      <c r="U87" s="104"/>
+      <c r="V87" s="104"/>
+      <c r="W87" s="104"/>
+      <c r="X87" s="104"/>
       <c r="Y87" s="43"/>
       <c r="Z87" s="43"/>
       <c r="AA87" s="43"/>
@@ -10191,15 +10194,15 @@
       <c r="R88" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S88" s="102" t="s">
+      <c r="S88" s="104" t="s">
         <v>321</v>
       </c>
-      <c r="T88" s="102"/>
-      <c r="U88" s="102"/>
-      <c r="V88" s="102"/>
-      <c r="W88" s="102"/>
-      <c r="X88" s="102"/>
-      <c r="Y88" s="102"/>
+      <c r="T88" s="104"/>
+      <c r="U88" s="104"/>
+      <c r="V88" s="104"/>
+      <c r="W88" s="104"/>
+      <c r="X88" s="104"/>
+      <c r="Y88" s="104"/>
       <c r="Z88" s="43"/>
       <c r="AA88" s="43"/>
       <c r="AB88" s="43"/>
@@ -10237,10 +10240,10 @@
       <c r="G89" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="H89" s="102" t="s">
+      <c r="H89" s="104" t="s">
         <v>17</v>
       </c>
-      <c r="I89" s="102"/>
+      <c r="I89" s="104"/>
       <c r="J89" s="43" t="s">
         <v>213</v>
       </c>
@@ -10268,15 +10271,15 @@
       <c r="R89" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S89" s="102" t="s">
+      <c r="S89" s="104" t="s">
         <v>323</v>
       </c>
-      <c r="T89" s="102"/>
-      <c r="U89" s="102"/>
-      <c r="V89" s="102"/>
-      <c r="W89" s="102"/>
-      <c r="X89" s="102"/>
-      <c r="Y89" s="102"/>
+      <c r="T89" s="104"/>
+      <c r="U89" s="104"/>
+      <c r="V89" s="104"/>
+      <c r="W89" s="104"/>
+      <c r="X89" s="104"/>
+      <c r="Y89" s="104"/>
       <c r="Z89" s="43"/>
       <c r="AA89" s="43"/>
       <c r="AB89" s="43"/>
@@ -10347,15 +10350,15 @@
       <c r="R90" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S90" s="102" t="s">
+      <c r="S90" s="104" t="s">
         <v>325</v>
       </c>
-      <c r="T90" s="102"/>
-      <c r="U90" s="102"/>
-      <c r="V90" s="102"/>
-      <c r="W90" s="102"/>
-      <c r="X90" s="102"/>
-      <c r="Y90" s="102"/>
+      <c r="T90" s="104"/>
+      <c r="U90" s="104"/>
+      <c r="V90" s="104"/>
+      <c r="W90" s="104"/>
+      <c r="X90" s="104"/>
+      <c r="Y90" s="104"/>
       <c r="Z90" s="43"/>
       <c r="AA90" s="43"/>
       <c r="AB90" s="43"/>
@@ -10386,10 +10389,10 @@
       <c r="D91" s="51" t="s">
         <v>326</v>
       </c>
-      <c r="E91" s="105" t="s">
+      <c r="E91" s="103" t="s">
         <v>327</v>
       </c>
-      <c r="F91" s="105"/>
+      <c r="F91" s="103"/>
       <c r="G91" s="51" t="s">
         <v>604</v>
       </c>
@@ -10426,16 +10429,16 @@
       <c r="R91" s="86" t="s">
         <v>689</v>
       </c>
-      <c r="S91" s="105" t="s">
+      <c r="S91" s="103" t="s">
         <v>80</v>
       </c>
-      <c r="T91" s="105"/>
-      <c r="U91" s="105"/>
-      <c r="V91" s="105"/>
-      <c r="W91" s="105"/>
-      <c r="X91" s="105"/>
-      <c r="Y91" s="105"/>
-      <c r="Z91" s="105"/>
+      <c r="T91" s="103"/>
+      <c r="U91" s="103"/>
+      <c r="V91" s="103"/>
+      <c r="W91" s="103"/>
+      <c r="X91" s="103"/>
+      <c r="Y91" s="103"/>
+      <c r="Z91" s="103"/>
       <c r="AA91" s="51"/>
       <c r="AB91" s="51"/>
       <c r="AC91" s="51"/>
@@ -10465,10 +10468,10 @@
       <c r="D92" s="51" t="s">
         <v>326</v>
       </c>
-      <c r="E92" s="105" t="s">
+      <c r="E92" s="103" t="s">
         <v>327</v>
       </c>
-      <c r="F92" s="105"/>
+      <c r="F92" s="103"/>
       <c r="G92" s="51" t="s">
         <v>604</v>
       </c>
@@ -10505,16 +10508,16 @@
       <c r="R92" s="86" t="s">
         <v>610</v>
       </c>
-      <c r="S92" s="105" t="s">
+      <c r="S92" s="103" t="s">
         <v>328</v>
       </c>
-      <c r="T92" s="105"/>
-      <c r="U92" s="105"/>
-      <c r="V92" s="105"/>
-      <c r="W92" s="105"/>
-      <c r="X92" s="105"/>
-      <c r="Y92" s="105"/>
-      <c r="Z92" s="105"/>
+      <c r="T92" s="103"/>
+      <c r="U92" s="103"/>
+      <c r="V92" s="103"/>
+      <c r="W92" s="103"/>
+      <c r="X92" s="103"/>
+      <c r="Y92" s="103"/>
+      <c r="Z92" s="103"/>
       <c r="AA92" s="51"/>
       <c r="AB92" s="51"/>
       <c r="AC92" s="51"/>
@@ -10544,10 +10547,10 @@
       <c r="D93" s="51" t="s">
         <v>326</v>
       </c>
-      <c r="E93" s="105" t="s">
+      <c r="E93" s="103" t="s">
         <v>327</v>
       </c>
-      <c r="F93" s="105"/>
+      <c r="F93" s="103"/>
       <c r="G93" s="51" t="s">
         <v>604</v>
       </c>
@@ -10580,16 +10583,16 @@
         <v>628</v>
       </c>
       <c r="R93" s="86"/>
-      <c r="S93" s="105" t="s">
+      <c r="S93" s="103" t="s">
         <v>329</v>
       </c>
-      <c r="T93" s="105"/>
-      <c r="U93" s="105"/>
-      <c r="V93" s="105"/>
-      <c r="W93" s="105"/>
-      <c r="X93" s="105"/>
-      <c r="Y93" s="105"/>
-      <c r="Z93" s="105"/>
+      <c r="T93" s="103"/>
+      <c r="U93" s="103"/>
+      <c r="V93" s="103"/>
+      <c r="W93" s="103"/>
+      <c r="X93" s="103"/>
+      <c r="Y93" s="103"/>
+      <c r="Z93" s="103"/>
       <c r="AA93" s="51"/>
       <c r="AB93" s="51"/>
       <c r="AC93" s="51"/>
@@ -10661,17 +10664,17 @@
       <c r="R94" s="86" t="s">
         <v>662</v>
       </c>
-      <c r="S94" s="102" t="s">
+      <c r="S94" s="104" t="s">
         <v>174</v>
       </c>
-      <c r="T94" s="102"/>
-      <c r="U94" s="102"/>
-      <c r="V94" s="102"/>
-      <c r="W94" s="102"/>
-      <c r="X94" s="102"/>
-      <c r="Y94" s="102"/>
-      <c r="Z94" s="102"/>
-      <c r="AA94" s="102"/>
+      <c r="T94" s="104"/>
+      <c r="U94" s="104"/>
+      <c r="V94" s="104"/>
+      <c r="W94" s="104"/>
+      <c r="X94" s="104"/>
+      <c r="Y94" s="104"/>
+      <c r="Z94" s="104"/>
+      <c r="AA94" s="104"/>
       <c r="AB94" s="43"/>
       <c r="AC94" s="43"/>
       <c r="AD94" s="43"/>
@@ -10700,10 +10703,10 @@
       <c r="D95" s="43" t="s">
         <v>601</v>
       </c>
-      <c r="E95" s="102" t="s">
+      <c r="E95" s="104" t="s">
         <v>331</v>
       </c>
-      <c r="F95" s="102"/>
+      <c r="F95" s="104"/>
       <c r="G95" s="43" t="s">
         <v>7</v>
       </c>
@@ -10736,15 +10739,15 @@
         <v>682</v>
       </c>
       <c r="R95" s="86"/>
-      <c r="S95" s="102" t="s">
+      <c r="S95" s="104" t="s">
         <v>150</v>
       </c>
-      <c r="T95" s="102"/>
-      <c r="U95" s="102"/>
-      <c r="V95" s="102"/>
-      <c r="W95" s="102"/>
-      <c r="X95" s="102"/>
-      <c r="Y95" s="102"/>
+      <c r="T95" s="104"/>
+      <c r="U95" s="104"/>
+      <c r="V95" s="104"/>
+      <c r="W95" s="104"/>
+      <c r="X95" s="104"/>
+      <c r="Y95" s="104"/>
       <c r="Z95" s="43"/>
       <c r="AA95" s="43"/>
       <c r="AB95" s="43"/>
@@ -10775,10 +10778,10 @@
       <c r="D96" s="43" t="s">
         <v>601</v>
       </c>
-      <c r="E96" s="102" t="s">
+      <c r="E96" s="104" t="s">
         <v>331</v>
       </c>
-      <c r="F96" s="102"/>
+      <c r="F96" s="104"/>
       <c r="G96" s="43" t="s">
         <v>7</v>
       </c>
@@ -10809,16 +10812,16 @@
         <v>680</v>
       </c>
       <c r="R96" s="86"/>
-      <c r="S96" s="102" t="s">
+      <c r="S96" s="104" t="s">
         <v>172</v>
       </c>
-      <c r="T96" s="102"/>
-      <c r="U96" s="102"/>
-      <c r="V96" s="102"/>
-      <c r="W96" s="102"/>
-      <c r="X96" s="102"/>
-      <c r="Y96" s="102"/>
-      <c r="Z96" s="102"/>
+      <c r="T96" s="104"/>
+      <c r="U96" s="104"/>
+      <c r="V96" s="104"/>
+      <c r="W96" s="104"/>
+      <c r="X96" s="104"/>
+      <c r="Y96" s="104"/>
+      <c r="Z96" s="104"/>
       <c r="AA96" s="43"/>
       <c r="AB96" s="43"/>
       <c r="AC96" s="43"/>
@@ -10848,10 +10851,10 @@
       <c r="D97" s="43" t="s">
         <v>601</v>
       </c>
-      <c r="E97" s="102" t="s">
+      <c r="E97" s="104" t="s">
         <v>331</v>
       </c>
-      <c r="F97" s="102"/>
+      <c r="F97" s="104"/>
       <c r="G97" s="43" t="s">
         <v>7</v>
       </c>
@@ -10886,16 +10889,16 @@
         <v>679</v>
       </c>
       <c r="R97" s="86"/>
-      <c r="S97" s="102" t="s">
+      <c r="S97" s="104" t="s">
         <v>182</v>
       </c>
-      <c r="T97" s="102"/>
-      <c r="U97" s="102"/>
-      <c r="V97" s="102"/>
-      <c r="W97" s="102"/>
-      <c r="X97" s="102"/>
-      <c r="Y97" s="102"/>
-      <c r="Z97" s="102"/>
+      <c r="T97" s="104"/>
+      <c r="U97" s="104"/>
+      <c r="V97" s="104"/>
+      <c r="W97" s="104"/>
+      <c r="X97" s="104"/>
+      <c r="Y97" s="104"/>
+      <c r="Z97" s="104"/>
       <c r="AA97" s="43"/>
       <c r="AB97" s="43"/>
       <c r="AC97" s="43"/>
@@ -10963,16 +10966,16 @@
       <c r="R98" s="86" t="s">
         <v>612</v>
       </c>
-      <c r="S98" s="104" t="s">
+      <c r="S98" s="105" t="s">
         <v>102</v>
       </c>
-      <c r="T98" s="104"/>
-      <c r="U98" s="104"/>
-      <c r="V98" s="104"/>
-      <c r="W98" s="104"/>
-      <c r="X98" s="104"/>
-      <c r="Y98" s="104"/>
-      <c r="Z98" s="104"/>
+      <c r="T98" s="105"/>
+      <c r="U98" s="105"/>
+      <c r="V98" s="105"/>
+      <c r="W98" s="105"/>
+      <c r="X98" s="105"/>
+      <c r="Y98" s="105"/>
+      <c r="Z98" s="105"/>
       <c r="AA98" s="65"/>
       <c r="AB98" s="65"/>
       <c r="AC98" s="65"/>
@@ -11040,16 +11043,16 @@
       <c r="R99" s="86" t="s">
         <v>674</v>
       </c>
-      <c r="S99" s="104" t="s">
+      <c r="S99" s="105" t="s">
         <v>259</v>
       </c>
-      <c r="T99" s="104"/>
-      <c r="U99" s="104"/>
-      <c r="V99" s="104"/>
-      <c r="W99" s="104"/>
-      <c r="X99" s="104"/>
-      <c r="Y99" s="104"/>
-      <c r="Z99" s="104"/>
+      <c r="T99" s="105"/>
+      <c r="U99" s="105"/>
+      <c r="V99" s="105"/>
+      <c r="W99" s="105"/>
+      <c r="X99" s="105"/>
+      <c r="Y99" s="105"/>
+      <c r="Z99" s="105"/>
       <c r="AA99" s="65"/>
       <c r="AB99" s="65"/>
       <c r="AC99" s="65"/>
@@ -11117,16 +11120,16 @@
       <c r="R100" s="86" t="s">
         <v>672</v>
       </c>
-      <c r="S100" s="104" t="s">
+      <c r="S100" s="105" t="s">
         <v>187</v>
       </c>
-      <c r="T100" s="104"/>
-      <c r="U100" s="104"/>
-      <c r="V100" s="104"/>
-      <c r="W100" s="104"/>
-      <c r="X100" s="104"/>
-      <c r="Y100" s="104"/>
-      <c r="Z100" s="104"/>
+      <c r="T100" s="105"/>
+      <c r="U100" s="105"/>
+      <c r="V100" s="105"/>
+      <c r="W100" s="105"/>
+      <c r="X100" s="105"/>
+      <c r="Y100" s="105"/>
+      <c r="Z100" s="105"/>
       <c r="AA100" s="65"/>
       <c r="AB100" s="65"/>
       <c r="AC100" s="65"/>
@@ -11790,24 +11793,24 @@
     </row>
     <row r="116" spans="1:41" ht="12.75">
       <c r="A116" s="80"/>
-      <c r="B116" s="113"/>
-      <c r="C116" s="113"/>
-      <c r="D116" s="113"/>
-      <c r="E116" s="113"/>
-      <c r="F116" s="113"/>
-      <c r="G116" s="113"/>
-      <c r="H116" s="113"/>
-      <c r="I116" s="113"/>
-      <c r="J116" s="113"/>
-      <c r="K116" s="113"/>
-      <c r="L116" s="113"/>
-      <c r="M116" s="113"/>
-      <c r="N116" s="113"/>
-      <c r="O116" s="113"/>
-      <c r="P116" s="113"/>
-      <c r="Q116" s="113"/>
-      <c r="R116" s="113"/>
-      <c r="S116" s="113"/>
+      <c r="B116" s="102"/>
+      <c r="C116" s="102"/>
+      <c r="D116" s="102"/>
+      <c r="E116" s="102"/>
+      <c r="F116" s="102"/>
+      <c r="G116" s="102"/>
+      <c r="H116" s="102"/>
+      <c r="I116" s="102"/>
+      <c r="J116" s="102"/>
+      <c r="K116" s="102"/>
+      <c r="L116" s="102"/>
+      <c r="M116" s="102"/>
+      <c r="N116" s="102"/>
+      <c r="O116" s="102"/>
+      <c r="P116" s="102"/>
+      <c r="Q116" s="102"/>
+      <c r="R116" s="102"/>
+      <c r="S116" s="102"/>
       <c r="T116" s="80"/>
       <c r="U116" s="80"/>
       <c r="V116" s="80"/>
@@ -12134,24 +12137,24 @@
     </row>
     <row r="124" spans="1:41" ht="12.75">
       <c r="A124" s="80"/>
-      <c r="B124" s="113"/>
-      <c r="C124" s="113"/>
-      <c r="D124" s="113"/>
-      <c r="E124" s="113"/>
-      <c r="F124" s="113"/>
-      <c r="G124" s="113"/>
-      <c r="H124" s="113"/>
-      <c r="I124" s="113"/>
-      <c r="J124" s="113"/>
-      <c r="K124" s="113"/>
-      <c r="L124" s="113"/>
-      <c r="M124" s="113"/>
-      <c r="N124" s="113"/>
-      <c r="O124" s="113"/>
-      <c r="P124" s="113"/>
-      <c r="Q124" s="113"/>
-      <c r="R124" s="113"/>
-      <c r="S124" s="113"/>
+      <c r="B124" s="102"/>
+      <c r="C124" s="102"/>
+      <c r="D124" s="102"/>
+      <c r="E124" s="102"/>
+      <c r="F124" s="102"/>
+      <c r="G124" s="102"/>
+      <c r="H124" s="102"/>
+      <c r="I124" s="102"/>
+      <c r="J124" s="102"/>
+      <c r="K124" s="102"/>
+      <c r="L124" s="102"/>
+      <c r="M124" s="102"/>
+      <c r="N124" s="102"/>
+      <c r="O124" s="102"/>
+      <c r="P124" s="102"/>
+      <c r="Q124" s="102"/>
+      <c r="R124" s="102"/>
+      <c r="S124" s="102"/>
       <c r="T124" s="80"/>
       <c r="U124" s="80"/>
       <c r="V124" s="80"/>
@@ -12392,24 +12395,24 @@
     </row>
     <row r="130" spans="1:41" ht="12.75">
       <c r="A130" s="80"/>
-      <c r="B130" s="113"/>
-      <c r="C130" s="113"/>
-      <c r="D130" s="113"/>
-      <c r="E130" s="113"/>
-      <c r="F130" s="113"/>
-      <c r="G130" s="113"/>
-      <c r="H130" s="113"/>
-      <c r="I130" s="113"/>
-      <c r="J130" s="113"/>
-      <c r="K130" s="113"/>
-      <c r="L130" s="113"/>
-      <c r="M130" s="113"/>
-      <c r="N130" s="113"/>
-      <c r="O130" s="113"/>
-      <c r="P130" s="113"/>
-      <c r="Q130" s="113"/>
-      <c r="R130" s="113"/>
-      <c r="S130" s="113"/>
+      <c r="B130" s="102"/>
+      <c r="C130" s="102"/>
+      <c r="D130" s="102"/>
+      <c r="E130" s="102"/>
+      <c r="F130" s="102"/>
+      <c r="G130" s="102"/>
+      <c r="H130" s="102"/>
+      <c r="I130" s="102"/>
+      <c r="J130" s="102"/>
+      <c r="K130" s="102"/>
+      <c r="L130" s="102"/>
+      <c r="M130" s="102"/>
+      <c r="N130" s="102"/>
+      <c r="O130" s="102"/>
+      <c r="P130" s="102"/>
+      <c r="Q130" s="102"/>
+      <c r="R130" s="102"/>
+      <c r="S130" s="102"/>
       <c r="T130" s="80"/>
       <c r="U130" s="80"/>
       <c r="V130" s="80"/>
@@ -12779,20 +12782,20 @@
     </row>
     <row r="139" spans="1:41" ht="12.75">
       <c r="A139" s="80"/>
-      <c r="B139" s="113"/>
-      <c r="C139" s="113"/>
-      <c r="D139" s="113"/>
-      <c r="E139" s="113"/>
-      <c r="F139" s="113"/>
-      <c r="G139" s="113"/>
-      <c r="H139" s="113"/>
-      <c r="I139" s="113"/>
-      <c r="J139" s="113"/>
-      <c r="K139" s="113"/>
-      <c r="L139" s="113"/>
-      <c r="M139" s="113"/>
-      <c r="N139" s="113"/>
-      <c r="O139" s="113"/>
+      <c r="B139" s="102"/>
+      <c r="C139" s="102"/>
+      <c r="D139" s="102"/>
+      <c r="E139" s="102"/>
+      <c r="F139" s="102"/>
+      <c r="G139" s="102"/>
+      <c r="H139" s="102"/>
+      <c r="I139" s="102"/>
+      <c r="J139" s="102"/>
+      <c r="K139" s="102"/>
+      <c r="L139" s="102"/>
+      <c r="M139" s="102"/>
+      <c r="N139" s="102"/>
+      <c r="O139" s="102"/>
       <c r="P139" s="93"/>
       <c r="Q139" s="93"/>
       <c r="R139" s="93"/>
@@ -49502,98 +49505,6 @@
   </sheetData>
   <autoFilter ref="A1:AI895" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <mergeCells count="116">
-    <mergeCell ref="B116:S116"/>
-    <mergeCell ref="B124:S124"/>
-    <mergeCell ref="B130:S130"/>
-    <mergeCell ref="B139:O139"/>
-    <mergeCell ref="E91:F91"/>
-    <mergeCell ref="S91:Z91"/>
-    <mergeCell ref="E92:F92"/>
-    <mergeCell ref="S92:Z92"/>
-    <mergeCell ref="E93:F93"/>
-    <mergeCell ref="S93:Z93"/>
-    <mergeCell ref="S94:AA94"/>
-    <mergeCell ref="E95:F95"/>
-    <mergeCell ref="E96:F96"/>
-    <mergeCell ref="S96:Z96"/>
-    <mergeCell ref="S95:Y95"/>
-    <mergeCell ref="S100:Z100"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="S2:X2"/>
-    <mergeCell ref="S3:Y3"/>
-    <mergeCell ref="S7:Z7"/>
-    <mergeCell ref="S9:Z9"/>
-    <mergeCell ref="S10:Y10"/>
-    <mergeCell ref="S14:Y14"/>
-    <mergeCell ref="S16:AA16"/>
-    <mergeCell ref="S18:X18"/>
-    <mergeCell ref="S1:T1"/>
-    <mergeCell ref="S4:X4"/>
-    <mergeCell ref="S5:Y5"/>
-    <mergeCell ref="S6:Y6"/>
-    <mergeCell ref="S8:Y8"/>
-    <mergeCell ref="S11:Y11"/>
-    <mergeCell ref="S17:Z17"/>
-    <mergeCell ref="S21:Y21"/>
-    <mergeCell ref="S12:Z12"/>
-    <mergeCell ref="S13:Z13"/>
-    <mergeCell ref="S15:Z15"/>
-    <mergeCell ref="S29:Z29"/>
-    <mergeCell ref="S31:Z31"/>
-    <mergeCell ref="S22:Z22"/>
-    <mergeCell ref="S23:Y23"/>
-    <mergeCell ref="S25:Y25"/>
-    <mergeCell ref="S26:Y26"/>
-    <mergeCell ref="S19:Y19"/>
-    <mergeCell ref="S20:Z20"/>
-    <mergeCell ref="S24:Y24"/>
-    <mergeCell ref="S27:Z27"/>
-    <mergeCell ref="S28:Z28"/>
-    <mergeCell ref="S30:Y30"/>
-    <mergeCell ref="S32:Y32"/>
-    <mergeCell ref="S33:Z33"/>
-    <mergeCell ref="S34:Y34"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="S35:Y35"/>
-    <mergeCell ref="S36:X36"/>
-    <mergeCell ref="S37:Z37"/>
-    <mergeCell ref="S38:AA38"/>
-    <mergeCell ref="S39:X39"/>
-    <mergeCell ref="S40:X40"/>
-    <mergeCell ref="S41:Z41"/>
-    <mergeCell ref="S42:AA42"/>
-    <mergeCell ref="S43:Z43"/>
-    <mergeCell ref="S44:Y44"/>
-    <mergeCell ref="S45:Z45"/>
-    <mergeCell ref="S46:X46"/>
-    <mergeCell ref="S47:Y47"/>
-    <mergeCell ref="S53:Z53"/>
-    <mergeCell ref="S48:Z48"/>
-    <mergeCell ref="S49:AA49"/>
-    <mergeCell ref="S50:Y50"/>
-    <mergeCell ref="S51:Z51"/>
-    <mergeCell ref="S52:Z52"/>
-    <mergeCell ref="S73:Y73"/>
-    <mergeCell ref="S75:Y75"/>
-    <mergeCell ref="S76:Y76"/>
-    <mergeCell ref="S77:Z77"/>
-    <mergeCell ref="S78:Z78"/>
-    <mergeCell ref="S79:X79"/>
-    <mergeCell ref="S54:Y54"/>
-    <mergeCell ref="S55:Z55"/>
-    <mergeCell ref="S56:X56"/>
-    <mergeCell ref="S57:X57"/>
-    <mergeCell ref="S64:Y64"/>
-    <mergeCell ref="S69:Z69"/>
-    <mergeCell ref="S58:X58"/>
-    <mergeCell ref="S59:Y59"/>
-    <mergeCell ref="S60:X60"/>
-    <mergeCell ref="S61:Y61"/>
-    <mergeCell ref="S62:Z62"/>
-    <mergeCell ref="S63:Y63"/>
-    <mergeCell ref="S65:Z65"/>
-    <mergeCell ref="S66:Z66"/>
-    <mergeCell ref="S67:Z67"/>
     <mergeCell ref="S90:Y90"/>
     <mergeCell ref="S87:X87"/>
     <mergeCell ref="S88:Y88"/>
@@ -49618,6 +49529,98 @@
     <mergeCell ref="S82:AA82"/>
     <mergeCell ref="S84:X84"/>
     <mergeCell ref="S85:X85"/>
+    <mergeCell ref="S73:Y73"/>
+    <mergeCell ref="S75:Y75"/>
+    <mergeCell ref="S76:Y76"/>
+    <mergeCell ref="S77:Z77"/>
+    <mergeCell ref="S78:Z78"/>
+    <mergeCell ref="S79:X79"/>
+    <mergeCell ref="S54:Y54"/>
+    <mergeCell ref="S55:Z55"/>
+    <mergeCell ref="S56:X56"/>
+    <mergeCell ref="S57:X57"/>
+    <mergeCell ref="S64:Y64"/>
+    <mergeCell ref="S69:Z69"/>
+    <mergeCell ref="S58:X58"/>
+    <mergeCell ref="S59:Y59"/>
+    <mergeCell ref="S60:X60"/>
+    <mergeCell ref="S61:Y61"/>
+    <mergeCell ref="S62:Z62"/>
+    <mergeCell ref="S63:Y63"/>
+    <mergeCell ref="S65:Z65"/>
+    <mergeCell ref="S66:Z66"/>
+    <mergeCell ref="S67:Z67"/>
+    <mergeCell ref="S40:X40"/>
+    <mergeCell ref="S41:Z41"/>
+    <mergeCell ref="S42:AA42"/>
+    <mergeCell ref="S43:Z43"/>
+    <mergeCell ref="S44:Y44"/>
+    <mergeCell ref="S45:Z45"/>
+    <mergeCell ref="S46:X46"/>
+    <mergeCell ref="S47:Y47"/>
+    <mergeCell ref="S53:Z53"/>
+    <mergeCell ref="S48:Z48"/>
+    <mergeCell ref="S49:AA49"/>
+    <mergeCell ref="S50:Y50"/>
+    <mergeCell ref="S51:Z51"/>
+    <mergeCell ref="S52:Z52"/>
+    <mergeCell ref="S32:Y32"/>
+    <mergeCell ref="S33:Z33"/>
+    <mergeCell ref="S34:Y34"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="S35:Y35"/>
+    <mergeCell ref="S36:X36"/>
+    <mergeCell ref="S37:Z37"/>
+    <mergeCell ref="S38:AA38"/>
+    <mergeCell ref="S39:X39"/>
+    <mergeCell ref="S29:Z29"/>
+    <mergeCell ref="S31:Z31"/>
+    <mergeCell ref="S22:Z22"/>
+    <mergeCell ref="S23:Y23"/>
+    <mergeCell ref="S25:Y25"/>
+    <mergeCell ref="S26:Y26"/>
+    <mergeCell ref="S19:Y19"/>
+    <mergeCell ref="S20:Z20"/>
+    <mergeCell ref="S24:Y24"/>
+    <mergeCell ref="S27:Z27"/>
+    <mergeCell ref="S28:Z28"/>
+    <mergeCell ref="S30:Y30"/>
+    <mergeCell ref="S1:T1"/>
+    <mergeCell ref="S4:X4"/>
+    <mergeCell ref="S5:Y5"/>
+    <mergeCell ref="S6:Y6"/>
+    <mergeCell ref="S8:Y8"/>
+    <mergeCell ref="S11:Y11"/>
+    <mergeCell ref="S17:Z17"/>
+    <mergeCell ref="S21:Y21"/>
+    <mergeCell ref="S12:Z12"/>
+    <mergeCell ref="S13:Z13"/>
+    <mergeCell ref="S15:Z15"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="S2:X2"/>
+    <mergeCell ref="S3:Y3"/>
+    <mergeCell ref="S7:Z7"/>
+    <mergeCell ref="S9:Z9"/>
+    <mergeCell ref="S10:Y10"/>
+    <mergeCell ref="S14:Y14"/>
+    <mergeCell ref="S16:AA16"/>
+    <mergeCell ref="S18:X18"/>
+    <mergeCell ref="B116:S116"/>
+    <mergeCell ref="B124:S124"/>
+    <mergeCell ref="B130:S130"/>
+    <mergeCell ref="B139:O139"/>
+    <mergeCell ref="E91:F91"/>
+    <mergeCell ref="S91:Z91"/>
+    <mergeCell ref="E92:F92"/>
+    <mergeCell ref="S92:Z92"/>
+    <mergeCell ref="E93:F93"/>
+    <mergeCell ref="S93:Z93"/>
+    <mergeCell ref="S94:AA94"/>
+    <mergeCell ref="E95:F95"/>
+    <mergeCell ref="E96:F96"/>
+    <mergeCell ref="S96:Z96"/>
+    <mergeCell ref="S95:Y95"/>
+    <mergeCell ref="S100:Z100"/>
   </mergeCells>
   <phoneticPr fontId="21" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
Crocodile "Encounter" to "Experience"
</commit_message>
<xml_diff>
--- a/CDT AITP Go Live (2).xlsx
+++ b/CDT AITP Go Live (2).xlsx
@@ -2911,30 +2911,15 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2943,8 +2928,23 @@
     <xf numFmtId="0" fontId="18" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3245,10 +3245,10 @@
       <c r="R1" s="85" t="s">
         <v>607</v>
       </c>
-      <c r="S1" s="108" t="s">
+      <c r="S1" s="112" t="s">
         <v>210</v>
       </c>
-      <c r="T1" s="108"/>
+      <c r="T1" s="112"/>
       <c r="U1" s="43"/>
       <c r="V1" s="43"/>
       <c r="W1" s="43"/>
@@ -3291,10 +3291,10 @@
       <c r="G2" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="H2" s="104" t="s">
+      <c r="H2" s="102" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="104"/>
+      <c r="I2" s="102"/>
       <c r="J2" s="43" t="s">
         <v>213</v>
       </c>
@@ -3322,14 +3322,14 @@
       <c r="R2" s="86" t="s">
         <v>609</v>
       </c>
-      <c r="S2" s="104" t="s">
+      <c r="S2" s="102" t="s">
         <v>184</v>
       </c>
-      <c r="T2" s="104"/>
-      <c r="U2" s="104"/>
-      <c r="V2" s="104"/>
-      <c r="W2" s="104"/>
-      <c r="X2" s="104"/>
+      <c r="T2" s="102"/>
+      <c r="U2" s="102"/>
+      <c r="V2" s="102"/>
+      <c r="W2" s="102"/>
+      <c r="X2" s="102"/>
       <c r="Y2" s="43"/>
       <c r="Z2" s="43"/>
       <c r="AA2" s="43"/>
@@ -3401,15 +3401,15 @@
       <c r="R3" s="86" t="s">
         <v>611</v>
       </c>
-      <c r="S3" s="104" t="s">
+      <c r="S3" s="102" t="s">
         <v>194</v>
       </c>
-      <c r="T3" s="104"/>
-      <c r="U3" s="104"/>
-      <c r="V3" s="104"/>
-      <c r="W3" s="104"/>
-      <c r="X3" s="104"/>
-      <c r="Y3" s="104"/>
+      <c r="T3" s="102"/>
+      <c r="U3" s="102"/>
+      <c r="V3" s="102"/>
+      <c r="W3" s="102"/>
+      <c r="X3" s="102"/>
+      <c r="Y3" s="102"/>
       <c r="Z3" s="43"/>
       <c r="AA3" s="43"/>
       <c r="AB3" s="43"/>
@@ -3480,14 +3480,14 @@
       <c r="R4" s="86" t="s">
         <v>612</v>
       </c>
-      <c r="S4" s="104" t="s">
+      <c r="S4" s="102" t="s">
         <v>214</v>
       </c>
-      <c r="T4" s="104"/>
-      <c r="U4" s="104"/>
-      <c r="V4" s="104"/>
-      <c r="W4" s="104"/>
-      <c r="X4" s="104"/>
+      <c r="T4" s="102"/>
+      <c r="U4" s="102"/>
+      <c r="V4" s="102"/>
+      <c r="W4" s="102"/>
+      <c r="X4" s="102"/>
       <c r="Y4" s="43"/>
       <c r="Z4" s="43"/>
       <c r="AA4" s="43"/>
@@ -3561,15 +3561,15 @@
       <c r="R5" s="86" t="s">
         <v>614</v>
       </c>
-      <c r="S5" s="104" t="s">
+      <c r="S5" s="102" t="s">
         <v>219</v>
       </c>
-      <c r="T5" s="104"/>
-      <c r="U5" s="104"/>
-      <c r="V5" s="104"/>
-      <c r="W5" s="104"/>
-      <c r="X5" s="104"/>
-      <c r="Y5" s="104"/>
+      <c r="T5" s="102"/>
+      <c r="U5" s="102"/>
+      <c r="V5" s="102"/>
+      <c r="W5" s="102"/>
+      <c r="X5" s="102"/>
+      <c r="Y5" s="102"/>
       <c r="Z5" s="43"/>
       <c r="AA5" s="43"/>
       <c r="AB5" s="43"/>
@@ -3638,15 +3638,15 @@
       <c r="R6" s="86" t="s">
         <v>616</v>
       </c>
-      <c r="S6" s="106" t="s">
+      <c r="S6" s="110" t="s">
         <v>72</v>
       </c>
-      <c r="T6" s="106"/>
-      <c r="U6" s="106"/>
-      <c r="V6" s="106"/>
-      <c r="W6" s="106"/>
-      <c r="X6" s="106"/>
-      <c r="Y6" s="106"/>
+      <c r="T6" s="110"/>
+      <c r="U6" s="110"/>
+      <c r="V6" s="110"/>
+      <c r="W6" s="110"/>
+      <c r="X6" s="110"/>
+      <c r="Y6" s="110"/>
       <c r="Z6" s="50"/>
       <c r="AA6" s="50"/>
       <c r="AB6" s="50"/>
@@ -3715,16 +3715,16 @@
       <c r="R7" s="86" t="s">
         <v>618</v>
       </c>
-      <c r="S7" s="106" t="s">
+      <c r="S7" s="110" t="s">
         <v>77</v>
       </c>
-      <c r="T7" s="106"/>
-      <c r="U7" s="106"/>
-      <c r="V7" s="106"/>
-      <c r="W7" s="106"/>
-      <c r="X7" s="106"/>
-      <c r="Y7" s="106"/>
-      <c r="Z7" s="106"/>
+      <c r="T7" s="110"/>
+      <c r="U7" s="110"/>
+      <c r="V7" s="110"/>
+      <c r="W7" s="110"/>
+      <c r="X7" s="110"/>
+      <c r="Y7" s="110"/>
+      <c r="Z7" s="110"/>
       <c r="AA7" s="50"/>
       <c r="AB7" s="50"/>
       <c r="AC7" s="50"/>
@@ -3794,15 +3794,15 @@
       <c r="R8" s="86" t="s">
         <v>619</v>
       </c>
-      <c r="S8" s="106" t="s">
+      <c r="S8" s="110" t="s">
         <v>190</v>
       </c>
-      <c r="T8" s="106"/>
-      <c r="U8" s="106"/>
-      <c r="V8" s="106"/>
-      <c r="W8" s="106"/>
-      <c r="X8" s="106"/>
-      <c r="Y8" s="106"/>
+      <c r="T8" s="110"/>
+      <c r="U8" s="110"/>
+      <c r="V8" s="110"/>
+      <c r="W8" s="110"/>
+      <c r="X8" s="110"/>
+      <c r="Y8" s="110"/>
       <c r="Z8" s="50"/>
       <c r="AA8" s="50"/>
       <c r="AB8" s="50"/>
@@ -3875,16 +3875,16 @@
       <c r="R9" s="86" t="s">
         <v>615</v>
       </c>
-      <c r="S9" s="107" t="s">
+      <c r="S9" s="108" t="s">
         <v>224</v>
       </c>
-      <c r="T9" s="107"/>
-      <c r="U9" s="107"/>
-      <c r="V9" s="107"/>
-      <c r="W9" s="107"/>
-      <c r="X9" s="107"/>
-      <c r="Y9" s="107"/>
-      <c r="Z9" s="107"/>
+      <c r="T9" s="108"/>
+      <c r="U9" s="108"/>
+      <c r="V9" s="108"/>
+      <c r="W9" s="108"/>
+      <c r="X9" s="108"/>
+      <c r="Y9" s="108"/>
+      <c r="Z9" s="108"/>
       <c r="AA9" s="54"/>
       <c r="AB9" s="54"/>
       <c r="AC9" s="54"/>
@@ -3956,15 +3956,15 @@
       <c r="R10" s="86" t="s">
         <v>610</v>
       </c>
-      <c r="S10" s="105" t="s">
+      <c r="S10" s="104" t="s">
         <v>221</v>
       </c>
-      <c r="T10" s="105"/>
-      <c r="U10" s="105"/>
-      <c r="V10" s="105"/>
-      <c r="W10" s="105"/>
-      <c r="X10" s="105"/>
-      <c r="Y10" s="105"/>
+      <c r="T10" s="104"/>
+      <c r="U10" s="104"/>
+      <c r="V10" s="104"/>
+      <c r="W10" s="104"/>
+      <c r="X10" s="104"/>
+      <c r="Y10" s="104"/>
       <c r="Z10" s="65"/>
       <c r="AA10" s="65"/>
       <c r="AB10" s="65"/>
@@ -4037,15 +4037,15 @@
       <c r="R11" s="86" t="s">
         <v>623</v>
       </c>
-      <c r="S11" s="105" t="s">
+      <c r="S11" s="104" t="s">
         <v>222</v>
       </c>
-      <c r="T11" s="105"/>
-      <c r="U11" s="105"/>
-      <c r="V11" s="105"/>
-      <c r="W11" s="105"/>
-      <c r="X11" s="105"/>
-      <c r="Y11" s="105"/>
+      <c r="T11" s="104"/>
+      <c r="U11" s="104"/>
+      <c r="V11" s="104"/>
+      <c r="W11" s="104"/>
+      <c r="X11" s="104"/>
+      <c r="Y11" s="104"/>
       <c r="Z11" s="65"/>
       <c r="AA11" s="65"/>
       <c r="AB11" s="65"/>
@@ -4118,16 +4118,16 @@
       <c r="R12" s="86" t="s">
         <v>612</v>
       </c>
-      <c r="S12" s="105" t="s">
+      <c r="S12" s="104" t="s">
         <v>226</v>
       </c>
-      <c r="T12" s="105"/>
-      <c r="U12" s="105"/>
-      <c r="V12" s="105"/>
-      <c r="W12" s="105"/>
-      <c r="X12" s="105"/>
-      <c r="Y12" s="105"/>
-      <c r="Z12" s="105"/>
+      <c r="T12" s="104"/>
+      <c r="U12" s="104"/>
+      <c r="V12" s="104"/>
+      <c r="W12" s="104"/>
+      <c r="X12" s="104"/>
+      <c r="Y12" s="104"/>
+      <c r="Z12" s="104"/>
       <c r="AA12" s="65"/>
       <c r="AB12" s="65"/>
       <c r="AC12" s="65"/>
@@ -4197,16 +4197,16 @@
       <c r="R13" s="86" t="s">
         <v>625</v>
       </c>
-      <c r="S13" s="104" t="s">
+      <c r="S13" s="102" t="s">
         <v>231</v>
       </c>
-      <c r="T13" s="104"/>
-      <c r="U13" s="104"/>
-      <c r="V13" s="104"/>
-      <c r="W13" s="104"/>
-      <c r="X13" s="104"/>
-      <c r="Y13" s="104"/>
-      <c r="Z13" s="104"/>
+      <c r="T13" s="102"/>
+      <c r="U13" s="102"/>
+      <c r="V13" s="102"/>
+      <c r="W13" s="102"/>
+      <c r="X13" s="102"/>
+      <c r="Y13" s="102"/>
+      <c r="Z13" s="102"/>
       <c r="AA13" s="43"/>
       <c r="AB13" s="43"/>
       <c r="AC13" s="43"/>
@@ -4274,15 +4274,15 @@
       <c r="R14" s="86" t="s">
         <v>627</v>
       </c>
-      <c r="S14" s="104" t="s">
+      <c r="S14" s="102" t="s">
         <v>148</v>
       </c>
-      <c r="T14" s="104"/>
-      <c r="U14" s="104"/>
-      <c r="V14" s="104"/>
-      <c r="W14" s="104"/>
-      <c r="X14" s="104"/>
-      <c r="Y14" s="104"/>
+      <c r="T14" s="102"/>
+      <c r="U14" s="102"/>
+      <c r="V14" s="102"/>
+      <c r="W14" s="102"/>
+      <c r="X14" s="102"/>
+      <c r="Y14" s="102"/>
       <c r="Z14" s="43"/>
       <c r="AA14" s="43"/>
       <c r="AB14" s="43"/>
@@ -4355,16 +4355,16 @@
       <c r="R15" s="86" t="s">
         <v>629</v>
       </c>
-      <c r="S15" s="103" t="s">
+      <c r="S15" s="105" t="s">
         <v>86</v>
       </c>
-      <c r="T15" s="103"/>
-      <c r="U15" s="103"/>
-      <c r="V15" s="103"/>
-      <c r="W15" s="103"/>
-      <c r="X15" s="103"/>
-      <c r="Y15" s="103"/>
-      <c r="Z15" s="103"/>
+      <c r="T15" s="105"/>
+      <c r="U15" s="105"/>
+      <c r="V15" s="105"/>
+      <c r="W15" s="105"/>
+      <c r="X15" s="105"/>
+      <c r="Y15" s="105"/>
+      <c r="Z15" s="105"/>
       <c r="AA15" s="51"/>
       <c r="AB15" s="43"/>
       <c r="AC15" s="43"/>
@@ -4436,17 +4436,17 @@
       <c r="R16" s="86" t="s">
         <v>630</v>
       </c>
-      <c r="S16" s="103" t="s">
+      <c r="S16" s="105" t="s">
         <v>234</v>
       </c>
-      <c r="T16" s="103"/>
-      <c r="U16" s="103"/>
-      <c r="V16" s="103"/>
-      <c r="W16" s="103"/>
-      <c r="X16" s="103"/>
-      <c r="Y16" s="103"/>
-      <c r="Z16" s="103"/>
-      <c r="AA16" s="103"/>
+      <c r="T16" s="105"/>
+      <c r="U16" s="105"/>
+      <c r="V16" s="105"/>
+      <c r="W16" s="105"/>
+      <c r="X16" s="105"/>
+      <c r="Y16" s="105"/>
+      <c r="Z16" s="105"/>
+      <c r="AA16" s="105"/>
       <c r="AB16" s="43"/>
       <c r="AC16" s="43"/>
       <c r="AD16" s="43"/>
@@ -4517,16 +4517,16 @@
       <c r="R17" s="86" t="s">
         <v>632</v>
       </c>
-      <c r="S17" s="103" t="s">
+      <c r="S17" s="105" t="s">
         <v>84</v>
       </c>
-      <c r="T17" s="103"/>
-      <c r="U17" s="103"/>
-      <c r="V17" s="103"/>
-      <c r="W17" s="103"/>
-      <c r="X17" s="103"/>
-      <c r="Y17" s="103"/>
-      <c r="Z17" s="103"/>
+      <c r="T17" s="105"/>
+      <c r="U17" s="105"/>
+      <c r="V17" s="105"/>
+      <c r="W17" s="105"/>
+      <c r="X17" s="105"/>
+      <c r="Y17" s="105"/>
+      <c r="Z17" s="105"/>
       <c r="AA17" s="51"/>
       <c r="AB17" s="43"/>
       <c r="AC17" s="43"/>
@@ -4598,14 +4598,14 @@
       <c r="R18" s="86" t="s">
         <v>632</v>
       </c>
-      <c r="S18" s="103" t="s">
+      <c r="S18" s="105" t="s">
         <v>82</v>
       </c>
-      <c r="T18" s="103"/>
-      <c r="U18" s="103"/>
-      <c r="V18" s="103"/>
-      <c r="W18" s="103"/>
-      <c r="X18" s="103"/>
+      <c r="T18" s="105"/>
+      <c r="U18" s="105"/>
+      <c r="V18" s="105"/>
+      <c r="W18" s="105"/>
+      <c r="X18" s="105"/>
       <c r="Y18" s="51"/>
       <c r="Z18" s="51"/>
       <c r="AA18" s="51"/>
@@ -4679,15 +4679,15 @@
       <c r="R19" s="86" t="s">
         <v>634</v>
       </c>
-      <c r="S19" s="103" t="s">
+      <c r="S19" s="105" t="s">
         <v>96</v>
       </c>
-      <c r="T19" s="103"/>
-      <c r="U19" s="103"/>
-      <c r="V19" s="103"/>
-      <c r="W19" s="103"/>
-      <c r="X19" s="103"/>
-      <c r="Y19" s="103"/>
+      <c r="T19" s="105"/>
+      <c r="U19" s="105"/>
+      <c r="V19" s="105"/>
+      <c r="W19" s="105"/>
+      <c r="X19" s="105"/>
+      <c r="Y19" s="105"/>
       <c r="Z19" s="51"/>
       <c r="AA19" s="51"/>
       <c r="AB19" s="43"/>
@@ -4760,16 +4760,16 @@
       <c r="R20" s="86" t="s">
         <v>636</v>
       </c>
-      <c r="S20" s="103" t="s">
+      <c r="S20" s="105" t="s">
         <v>235</v>
       </c>
-      <c r="T20" s="103"/>
-      <c r="U20" s="103"/>
-      <c r="V20" s="103"/>
-      <c r="W20" s="103"/>
-      <c r="X20" s="103"/>
-      <c r="Y20" s="103"/>
-      <c r="Z20" s="103"/>
+      <c r="T20" s="105"/>
+      <c r="U20" s="105"/>
+      <c r="V20" s="105"/>
+      <c r="W20" s="105"/>
+      <c r="X20" s="105"/>
+      <c r="Y20" s="105"/>
+      <c r="Z20" s="105"/>
       <c r="AA20" s="51"/>
       <c r="AB20" s="43"/>
       <c r="AC20" s="43"/>
@@ -4841,15 +4841,15 @@
       <c r="R21" s="86" t="s">
         <v>610</v>
       </c>
-      <c r="S21" s="103" t="s">
+      <c r="S21" s="105" t="s">
         <v>236</v>
       </c>
-      <c r="T21" s="103"/>
-      <c r="U21" s="103"/>
-      <c r="V21" s="103"/>
-      <c r="W21" s="103"/>
-      <c r="X21" s="103"/>
-      <c r="Y21" s="103"/>
+      <c r="T21" s="105"/>
+      <c r="U21" s="105"/>
+      <c r="V21" s="105"/>
+      <c r="W21" s="105"/>
+      <c r="X21" s="105"/>
+      <c r="Y21" s="105"/>
       <c r="Z21" s="51"/>
       <c r="AA21" s="51"/>
       <c r="AB21" s="43"/>
@@ -4922,16 +4922,16 @@
       <c r="R22" s="86" t="s">
         <v>639</v>
       </c>
-      <c r="S22" s="103" t="s">
+      <c r="S22" s="105" t="s">
         <v>238</v>
       </c>
-      <c r="T22" s="103"/>
-      <c r="U22" s="103"/>
-      <c r="V22" s="103"/>
-      <c r="W22" s="103"/>
-      <c r="X22" s="103"/>
-      <c r="Y22" s="103"/>
-      <c r="Z22" s="103"/>
+      <c r="T22" s="105"/>
+      <c r="U22" s="105"/>
+      <c r="V22" s="105"/>
+      <c r="W22" s="105"/>
+      <c r="X22" s="105"/>
+      <c r="Y22" s="105"/>
+      <c r="Z22" s="105"/>
       <c r="AA22" s="51"/>
       <c r="AB22" s="43"/>
       <c r="AC22" s="43"/>
@@ -5003,15 +5003,15 @@
       <c r="R23" s="86" t="s">
         <v>632</v>
       </c>
-      <c r="S23" s="103" t="s">
+      <c r="S23" s="105" t="s">
         <v>98</v>
       </c>
-      <c r="T23" s="103"/>
-      <c r="U23" s="103"/>
-      <c r="V23" s="103"/>
-      <c r="W23" s="103"/>
-      <c r="X23" s="103"/>
-      <c r="Y23" s="103"/>
+      <c r="T23" s="105"/>
+      <c r="U23" s="105"/>
+      <c r="V23" s="105"/>
+      <c r="W23" s="105"/>
+      <c r="X23" s="105"/>
+      <c r="Y23" s="105"/>
       <c r="Z23" s="51"/>
       <c r="AA23" s="51"/>
       <c r="AB23" s="43"/>
@@ -5084,15 +5084,15 @@
       <c r="R24" s="86" t="s">
         <v>641</v>
       </c>
-      <c r="S24" s="106" t="s">
+      <c r="S24" s="110" t="s">
         <v>240</v>
       </c>
-      <c r="T24" s="106"/>
-      <c r="U24" s="106"/>
-      <c r="V24" s="106"/>
-      <c r="W24" s="106"/>
-      <c r="X24" s="106"/>
-      <c r="Y24" s="106"/>
+      <c r="T24" s="110"/>
+      <c r="U24" s="110"/>
+      <c r="V24" s="110"/>
+      <c r="W24" s="110"/>
+      <c r="X24" s="110"/>
+      <c r="Y24" s="110"/>
       <c r="Z24" s="50"/>
       <c r="AA24" s="50"/>
       <c r="AB24" s="43"/>
@@ -5165,15 +5165,15 @@
       <c r="R25" s="86" t="s">
         <v>668</v>
       </c>
-      <c r="S25" s="106" t="s">
+      <c r="S25" s="110" t="s">
         <v>112</v>
       </c>
-      <c r="T25" s="106"/>
-      <c r="U25" s="106"/>
-      <c r="V25" s="106"/>
-      <c r="W25" s="106"/>
-      <c r="X25" s="106"/>
-      <c r="Y25" s="106"/>
+      <c r="T25" s="110"/>
+      <c r="U25" s="110"/>
+      <c r="V25" s="110"/>
+      <c r="W25" s="110"/>
+      <c r="X25" s="110"/>
+      <c r="Y25" s="110"/>
       <c r="Z25" s="50"/>
       <c r="AA25" s="50"/>
       <c r="AB25" s="43"/>
@@ -5246,15 +5246,15 @@
       <c r="R26" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S26" s="106" t="s">
+      <c r="S26" s="110" t="s">
         <v>108</v>
       </c>
-      <c r="T26" s="106"/>
-      <c r="U26" s="106"/>
-      <c r="V26" s="106"/>
-      <c r="W26" s="106"/>
-      <c r="X26" s="106"/>
-      <c r="Y26" s="106"/>
+      <c r="T26" s="110"/>
+      <c r="U26" s="110"/>
+      <c r="V26" s="110"/>
+      <c r="W26" s="110"/>
+      <c r="X26" s="110"/>
+      <c r="Y26" s="110"/>
       <c r="Z26" s="50"/>
       <c r="AA26" s="50"/>
       <c r="AB26" s="43"/>
@@ -5327,16 +5327,16 @@
       <c r="R27" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S27" s="106" t="s">
+      <c r="S27" s="110" t="s">
         <v>243</v>
       </c>
-      <c r="T27" s="106"/>
-      <c r="U27" s="106"/>
-      <c r="V27" s="106"/>
-      <c r="W27" s="106"/>
-      <c r="X27" s="106"/>
-      <c r="Y27" s="106"/>
-      <c r="Z27" s="106"/>
+      <c r="T27" s="110"/>
+      <c r="U27" s="110"/>
+      <c r="V27" s="110"/>
+      <c r="W27" s="110"/>
+      <c r="X27" s="110"/>
+      <c r="Y27" s="110"/>
+      <c r="Z27" s="110"/>
       <c r="AA27" s="50"/>
       <c r="AB27" s="43"/>
       <c r="AC27" s="43"/>
@@ -5408,16 +5408,16 @@
       <c r="R28" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S28" s="106" t="s">
+      <c r="S28" s="110" t="s">
         <v>245</v>
       </c>
-      <c r="T28" s="106"/>
-      <c r="U28" s="106"/>
-      <c r="V28" s="106"/>
-      <c r="W28" s="106"/>
-      <c r="X28" s="106"/>
-      <c r="Y28" s="106"/>
-      <c r="Z28" s="106"/>
+      <c r="T28" s="110"/>
+      <c r="U28" s="110"/>
+      <c r="V28" s="110"/>
+      <c r="W28" s="110"/>
+      <c r="X28" s="110"/>
+      <c r="Y28" s="110"/>
+      <c r="Z28" s="110"/>
       <c r="AA28" s="50"/>
       <c r="AB28" s="43"/>
       <c r="AC28" s="43"/>
@@ -5489,16 +5489,16 @@
       <c r="R29" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S29" s="106" t="s">
+      <c r="S29" s="110" t="s">
         <v>247</v>
       </c>
-      <c r="T29" s="106"/>
-      <c r="U29" s="106"/>
-      <c r="V29" s="106"/>
-      <c r="W29" s="106"/>
-      <c r="X29" s="106"/>
-      <c r="Y29" s="106"/>
-      <c r="Z29" s="106"/>
+      <c r="T29" s="110"/>
+      <c r="U29" s="110"/>
+      <c r="V29" s="110"/>
+      <c r="W29" s="110"/>
+      <c r="X29" s="110"/>
+      <c r="Y29" s="110"/>
+      <c r="Z29" s="110"/>
       <c r="AA29" s="50"/>
       <c r="AB29" s="43"/>
       <c r="AC29" s="43"/>
@@ -5570,15 +5570,15 @@
       <c r="R30" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S30" s="106" t="s">
+      <c r="S30" s="110" t="s">
         <v>249</v>
       </c>
-      <c r="T30" s="106"/>
-      <c r="U30" s="106"/>
-      <c r="V30" s="106"/>
-      <c r="W30" s="106"/>
-      <c r="X30" s="106"/>
-      <c r="Y30" s="106"/>
+      <c r="T30" s="110"/>
+      <c r="U30" s="110"/>
+      <c r="V30" s="110"/>
+      <c r="W30" s="110"/>
+      <c r="X30" s="110"/>
+      <c r="Y30" s="110"/>
       <c r="Z30" s="50"/>
       <c r="AA30" s="50"/>
       <c r="AB30" s="43"/>
@@ -5651,16 +5651,16 @@
       <c r="R31" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S31" s="109" t="s">
+      <c r="S31" s="111" t="s">
         <v>115</v>
       </c>
-      <c r="T31" s="109"/>
-      <c r="U31" s="109"/>
-      <c r="V31" s="109"/>
-      <c r="W31" s="109"/>
-      <c r="X31" s="109"/>
-      <c r="Y31" s="109"/>
-      <c r="Z31" s="109"/>
+      <c r="T31" s="111"/>
+      <c r="U31" s="111"/>
+      <c r="V31" s="111"/>
+      <c r="W31" s="111"/>
+      <c r="X31" s="111"/>
+      <c r="Y31" s="111"/>
+      <c r="Z31" s="111"/>
       <c r="AA31" s="52"/>
       <c r="AB31" s="43"/>
       <c r="AC31" s="43"/>
@@ -5728,15 +5728,15 @@
         <v>706</v>
       </c>
       <c r="R32" s="86"/>
-      <c r="S32" s="110" t="s">
+      <c r="S32" s="109" t="s">
         <v>252</v>
       </c>
-      <c r="T32" s="110"/>
-      <c r="U32" s="110"/>
-      <c r="V32" s="110"/>
-      <c r="W32" s="110"/>
-      <c r="X32" s="110"/>
-      <c r="Y32" s="110"/>
+      <c r="T32" s="109"/>
+      <c r="U32" s="109"/>
+      <c r="V32" s="109"/>
+      <c r="W32" s="109"/>
+      <c r="X32" s="109"/>
+      <c r="Y32" s="109"/>
       <c r="Z32" s="53"/>
       <c r="AA32" s="53"/>
       <c r="AB32" s="43"/>
@@ -5774,10 +5774,10 @@
       <c r="G33" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="H33" s="110" t="s">
+      <c r="H33" s="109" t="s">
         <v>7</v>
       </c>
-      <c r="I33" s="110"/>
+      <c r="I33" s="109"/>
       <c r="J33" s="53" t="s">
         <v>213</v>
       </c>
@@ -5805,16 +5805,16 @@
       <c r="R33" s="86" t="s">
         <v>708</v>
       </c>
-      <c r="S33" s="110" t="s">
+      <c r="S33" s="109" t="s">
         <v>253</v>
       </c>
-      <c r="T33" s="110"/>
-      <c r="U33" s="110"/>
-      <c r="V33" s="110"/>
-      <c r="W33" s="110"/>
-      <c r="X33" s="110"/>
-      <c r="Y33" s="110"/>
-      <c r="Z33" s="110"/>
+      <c r="T33" s="109"/>
+      <c r="U33" s="109"/>
+      <c r="V33" s="109"/>
+      <c r="W33" s="109"/>
+      <c r="X33" s="109"/>
+      <c r="Y33" s="109"/>
+      <c r="Z33" s="109"/>
       <c r="AA33" s="53"/>
       <c r="AB33" s="43"/>
       <c r="AC33" s="43"/>
@@ -5884,15 +5884,15 @@
       <c r="R34" s="86" t="s">
         <v>708</v>
       </c>
-      <c r="S34" s="110" t="s">
+      <c r="S34" s="109" t="s">
         <v>254</v>
       </c>
-      <c r="T34" s="110"/>
-      <c r="U34" s="110"/>
-      <c r="V34" s="110"/>
-      <c r="W34" s="110"/>
-      <c r="X34" s="110"/>
-      <c r="Y34" s="110"/>
+      <c r="T34" s="109"/>
+      <c r="U34" s="109"/>
+      <c r="V34" s="109"/>
+      <c r="W34" s="109"/>
+      <c r="X34" s="109"/>
+      <c r="Y34" s="109"/>
       <c r="Z34" s="53"/>
       <c r="AA34" s="53"/>
       <c r="AB34" s="43"/>
@@ -5961,15 +5961,15 @@
         <v>709</v>
       </c>
       <c r="R35" s="86"/>
-      <c r="S35" s="110" t="s">
+      <c r="S35" s="109" t="s">
         <v>255</v>
       </c>
-      <c r="T35" s="110"/>
-      <c r="U35" s="110"/>
-      <c r="V35" s="110"/>
-      <c r="W35" s="110"/>
-      <c r="X35" s="110"/>
-      <c r="Y35" s="110"/>
+      <c r="T35" s="109"/>
+      <c r="U35" s="109"/>
+      <c r="V35" s="109"/>
+      <c r="W35" s="109"/>
+      <c r="X35" s="109"/>
+      <c r="Y35" s="109"/>
       <c r="Z35" s="53"/>
       <c r="AA35" s="53"/>
       <c r="AB35" s="43"/>
@@ -6040,14 +6040,14 @@
       <c r="R36" s="86" t="s">
         <v>712</v>
       </c>
-      <c r="S36" s="110" t="s">
+      <c r="S36" s="109" t="s">
         <v>256</v>
       </c>
-      <c r="T36" s="110"/>
-      <c r="U36" s="110"/>
-      <c r="V36" s="110"/>
-      <c r="W36" s="110"/>
-      <c r="X36" s="110"/>
+      <c r="T36" s="109"/>
+      <c r="U36" s="109"/>
+      <c r="V36" s="109"/>
+      <c r="W36" s="109"/>
+      <c r="X36" s="109"/>
       <c r="Y36" s="53"/>
       <c r="Z36" s="53"/>
       <c r="AA36" s="53"/>
@@ -6117,16 +6117,16 @@
         <v>689</v>
       </c>
       <c r="R37" s="86"/>
-      <c r="S37" s="110" t="s">
+      <c r="S37" s="109" t="s">
         <v>257</v>
       </c>
-      <c r="T37" s="110"/>
-      <c r="U37" s="110"/>
-      <c r="V37" s="110"/>
-      <c r="W37" s="110"/>
-      <c r="X37" s="110"/>
-      <c r="Y37" s="110"/>
-      <c r="Z37" s="110"/>
+      <c r="T37" s="109"/>
+      <c r="U37" s="109"/>
+      <c r="V37" s="109"/>
+      <c r="W37" s="109"/>
+      <c r="X37" s="109"/>
+      <c r="Y37" s="109"/>
+      <c r="Z37" s="109"/>
       <c r="AA37" s="53"/>
       <c r="AB37" s="43"/>
       <c r="AC37" s="43"/>
@@ -6194,17 +6194,17 @@
         <v>689</v>
       </c>
       <c r="R38" s="86"/>
-      <c r="S38" s="110" t="s">
+      <c r="S38" s="109" t="s">
         <v>258</v>
       </c>
-      <c r="T38" s="110"/>
-      <c r="U38" s="110"/>
-      <c r="V38" s="110"/>
-      <c r="W38" s="110"/>
-      <c r="X38" s="110"/>
-      <c r="Y38" s="110"/>
-      <c r="Z38" s="110"/>
-      <c r="AA38" s="110"/>
+      <c r="T38" s="109"/>
+      <c r="U38" s="109"/>
+      <c r="V38" s="109"/>
+      <c r="W38" s="109"/>
+      <c r="X38" s="109"/>
+      <c r="Y38" s="109"/>
+      <c r="Z38" s="109"/>
+      <c r="AA38" s="109"/>
       <c r="AB38" s="43"/>
       <c r="AC38" s="43"/>
       <c r="AD38" s="43"/>
@@ -6275,14 +6275,14 @@
       <c r="R39" s="86" t="s">
         <v>715</v>
       </c>
-      <c r="S39" s="107" t="s">
+      <c r="S39" s="108" t="s">
         <v>166</v>
       </c>
-      <c r="T39" s="107"/>
-      <c r="U39" s="107"/>
-      <c r="V39" s="107"/>
-      <c r="W39" s="107"/>
-      <c r="X39" s="107"/>
+      <c r="T39" s="108"/>
+      <c r="U39" s="108"/>
+      <c r="V39" s="108"/>
+      <c r="W39" s="108"/>
+      <c r="X39" s="108"/>
       <c r="Y39" s="54"/>
       <c r="Z39" s="54"/>
       <c r="AA39" s="54"/>
@@ -6356,14 +6356,14 @@
       <c r="R40" s="86" t="s">
         <v>624</v>
       </c>
-      <c r="S40" s="107" t="s">
+      <c r="S40" s="108" t="s">
         <v>263</v>
       </c>
-      <c r="T40" s="107"/>
-      <c r="U40" s="107"/>
-      <c r="V40" s="107"/>
-      <c r="W40" s="107"/>
-      <c r="X40" s="107"/>
+      <c r="T40" s="108"/>
+      <c r="U40" s="108"/>
+      <c r="V40" s="108"/>
+      <c r="W40" s="108"/>
+      <c r="X40" s="108"/>
       <c r="Y40" s="54"/>
       <c r="Z40" s="54"/>
       <c r="AA40" s="54"/>
@@ -6435,16 +6435,16 @@
       <c r="R41" s="86" t="s">
         <v>719</v>
       </c>
-      <c r="S41" s="107" t="s">
+      <c r="S41" s="108" t="s">
         <v>264</v>
       </c>
-      <c r="T41" s="107"/>
-      <c r="U41" s="107"/>
-      <c r="V41" s="107"/>
-      <c r="W41" s="107"/>
-      <c r="X41" s="107"/>
-      <c r="Y41" s="107"/>
-      <c r="Z41" s="107"/>
+      <c r="T41" s="108"/>
+      <c r="U41" s="108"/>
+      <c r="V41" s="108"/>
+      <c r="W41" s="108"/>
+      <c r="X41" s="108"/>
+      <c r="Y41" s="108"/>
+      <c r="Z41" s="108"/>
       <c r="AA41" s="54"/>
       <c r="AB41" s="43"/>
       <c r="AC41" s="43"/>
@@ -6516,17 +6516,17 @@
       <c r="R42" s="86" t="s">
         <v>719</v>
       </c>
-      <c r="S42" s="107" t="s">
+      <c r="S42" s="108" t="s">
         <v>161</v>
       </c>
-      <c r="T42" s="107"/>
-      <c r="U42" s="107"/>
-      <c r="V42" s="107"/>
-      <c r="W42" s="107"/>
-      <c r="X42" s="107"/>
-      <c r="Y42" s="107"/>
-      <c r="Z42" s="107"/>
-      <c r="AA42" s="107"/>
+      <c r="T42" s="108"/>
+      <c r="U42" s="108"/>
+      <c r="V42" s="108"/>
+      <c r="W42" s="108"/>
+      <c r="X42" s="108"/>
+      <c r="Y42" s="108"/>
+      <c r="Z42" s="108"/>
+      <c r="AA42" s="108"/>
       <c r="AB42" s="43"/>
       <c r="AC42" s="43"/>
       <c r="AD42" s="43"/>
@@ -6597,16 +6597,16 @@
       <c r="R43" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S43" s="107" t="s">
+      <c r="S43" s="108" t="s">
         <v>265</v>
       </c>
-      <c r="T43" s="107"/>
-      <c r="U43" s="107"/>
-      <c r="V43" s="107"/>
-      <c r="W43" s="107"/>
-      <c r="X43" s="107"/>
-      <c r="Y43" s="107"/>
-      <c r="Z43" s="107"/>
+      <c r="T43" s="108"/>
+      <c r="U43" s="108"/>
+      <c r="V43" s="108"/>
+      <c r="W43" s="108"/>
+      <c r="X43" s="108"/>
+      <c r="Y43" s="108"/>
+      <c r="Z43" s="108"/>
       <c r="AA43" s="54"/>
       <c r="AB43" s="43"/>
       <c r="AC43" s="43"/>
@@ -6678,15 +6678,15 @@
       <c r="R44" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S44" s="107" t="s">
+      <c r="S44" s="108" t="s">
         <v>158</v>
       </c>
-      <c r="T44" s="107"/>
-      <c r="U44" s="107"/>
-      <c r="V44" s="107"/>
-      <c r="W44" s="107"/>
-      <c r="X44" s="107"/>
-      <c r="Y44" s="107"/>
+      <c r="T44" s="108"/>
+      <c r="U44" s="108"/>
+      <c r="V44" s="108"/>
+      <c r="W44" s="108"/>
+      <c r="X44" s="108"/>
+      <c r="Y44" s="108"/>
       <c r="Z44" s="54"/>
       <c r="AA44" s="54"/>
       <c r="AB44" s="43"/>
@@ -6757,16 +6757,16 @@
       <c r="R45" s="86" t="s">
         <v>719</v>
       </c>
-      <c r="S45" s="107" t="s">
+      <c r="S45" s="108" t="s">
         <v>266</v>
       </c>
-      <c r="T45" s="107"/>
-      <c r="U45" s="107"/>
-      <c r="V45" s="107"/>
-      <c r="W45" s="107"/>
-      <c r="X45" s="107"/>
-      <c r="Y45" s="107"/>
-      <c r="Z45" s="107"/>
+      <c r="T45" s="108"/>
+      <c r="U45" s="108"/>
+      <c r="V45" s="108"/>
+      <c r="W45" s="108"/>
+      <c r="X45" s="108"/>
+      <c r="Y45" s="108"/>
+      <c r="Z45" s="108"/>
       <c r="AA45" s="54"/>
       <c r="AB45" s="43"/>
       <c r="AC45" s="43"/>
@@ -6834,14 +6834,14 @@
       <c r="R46" s="86" t="s">
         <v>632</v>
       </c>
-      <c r="S46" s="107" t="s">
+      <c r="S46" s="108" t="s">
         <v>132</v>
       </c>
-      <c r="T46" s="107"/>
-      <c r="U46" s="107"/>
-      <c r="V46" s="107"/>
-      <c r="W46" s="107"/>
-      <c r="X46" s="107"/>
+      <c r="T46" s="108"/>
+      <c r="U46" s="108"/>
+      <c r="V46" s="108"/>
+      <c r="W46" s="108"/>
+      <c r="X46" s="108"/>
       <c r="Y46" s="54"/>
       <c r="Z46" s="54"/>
       <c r="AA46" s="54"/>
@@ -6915,15 +6915,15 @@
       <c r="R47" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S47" s="107" t="s">
+      <c r="S47" s="108" t="s">
         <v>136</v>
       </c>
-      <c r="T47" s="107"/>
-      <c r="U47" s="107"/>
-      <c r="V47" s="107"/>
-      <c r="W47" s="107"/>
-      <c r="X47" s="107"/>
-      <c r="Y47" s="107"/>
+      <c r="T47" s="108"/>
+      <c r="U47" s="108"/>
+      <c r="V47" s="108"/>
+      <c r="W47" s="108"/>
+      <c r="X47" s="108"/>
+      <c r="Y47" s="108"/>
       <c r="Z47" s="54"/>
       <c r="AA47" s="54"/>
       <c r="AB47" s="43"/>
@@ -6996,16 +6996,16 @@
       <c r="R48" s="86" t="s">
         <v>636</v>
       </c>
-      <c r="S48" s="107" t="s">
+      <c r="S48" s="108" t="s">
         <v>178</v>
       </c>
-      <c r="T48" s="107"/>
-      <c r="U48" s="107"/>
-      <c r="V48" s="107"/>
-      <c r="W48" s="107"/>
-      <c r="X48" s="107"/>
-      <c r="Y48" s="107"/>
-      <c r="Z48" s="107"/>
+      <c r="T48" s="108"/>
+      <c r="U48" s="108"/>
+      <c r="V48" s="108"/>
+      <c r="W48" s="108"/>
+      <c r="X48" s="108"/>
+      <c r="Y48" s="108"/>
+      <c r="Z48" s="108"/>
       <c r="AA48" s="54"/>
       <c r="AB48" s="43"/>
       <c r="AC48" s="43"/>
@@ -7077,17 +7077,17 @@
       <c r="R49" s="86" t="s">
         <v>730</v>
       </c>
-      <c r="S49" s="107" t="s">
+      <c r="S49" s="108" t="s">
         <v>268</v>
       </c>
-      <c r="T49" s="107"/>
-      <c r="U49" s="107"/>
-      <c r="V49" s="107"/>
-      <c r="W49" s="107"/>
-      <c r="X49" s="107"/>
-      <c r="Y49" s="107"/>
-      <c r="Z49" s="107"/>
-      <c r="AA49" s="107"/>
+      <c r="T49" s="108"/>
+      <c r="U49" s="108"/>
+      <c r="V49" s="108"/>
+      <c r="W49" s="108"/>
+      <c r="X49" s="108"/>
+      <c r="Y49" s="108"/>
+      <c r="Z49" s="108"/>
+      <c r="AA49" s="108"/>
       <c r="AB49" s="43"/>
       <c r="AC49" s="43"/>
       <c r="AD49" s="43"/>
@@ -7158,15 +7158,15 @@
       <c r="R50" s="86" t="s">
         <v>730</v>
       </c>
-      <c r="S50" s="107" t="s">
+      <c r="S50" s="108" t="s">
         <v>269</v>
       </c>
-      <c r="T50" s="107"/>
-      <c r="U50" s="107"/>
-      <c r="V50" s="107"/>
-      <c r="W50" s="107"/>
-      <c r="X50" s="107"/>
-      <c r="Y50" s="107"/>
+      <c r="T50" s="108"/>
+      <c r="U50" s="108"/>
+      <c r="V50" s="108"/>
+      <c r="W50" s="108"/>
+      <c r="X50" s="108"/>
+      <c r="Y50" s="108"/>
       <c r="Z50" s="54"/>
       <c r="AA50" s="54"/>
       <c r="AB50" s="43"/>
@@ -7235,16 +7235,16 @@
       <c r="R51" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S51" s="107" t="s">
+      <c r="S51" s="108" t="s">
         <v>170</v>
       </c>
-      <c r="T51" s="107"/>
-      <c r="U51" s="107"/>
-      <c r="V51" s="107"/>
-      <c r="W51" s="107"/>
-      <c r="X51" s="107"/>
-      <c r="Y51" s="107"/>
-      <c r="Z51" s="107"/>
+      <c r="T51" s="108"/>
+      <c r="U51" s="108"/>
+      <c r="V51" s="108"/>
+      <c r="W51" s="108"/>
+      <c r="X51" s="108"/>
+      <c r="Y51" s="108"/>
+      <c r="Z51" s="108"/>
       <c r="AA51" s="54"/>
       <c r="AB51" s="43"/>
       <c r="AC51" s="43"/>
@@ -7314,16 +7314,16 @@
       <c r="R52" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S52" s="104" t="s">
+      <c r="S52" s="102" t="s">
         <v>130</v>
       </c>
-      <c r="T52" s="104"/>
-      <c r="U52" s="104"/>
-      <c r="V52" s="104"/>
-      <c r="W52" s="104"/>
-      <c r="X52" s="104"/>
-      <c r="Y52" s="104"/>
-      <c r="Z52" s="104"/>
+      <c r="T52" s="102"/>
+      <c r="U52" s="102"/>
+      <c r="V52" s="102"/>
+      <c r="W52" s="102"/>
+      <c r="X52" s="102"/>
+      <c r="Y52" s="102"/>
+      <c r="Z52" s="102"/>
       <c r="AA52" s="43"/>
       <c r="AB52" s="43"/>
       <c r="AC52" s="43"/>
@@ -7393,16 +7393,16 @@
       <c r="R53" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S53" s="104" t="s">
+      <c r="S53" s="102" t="s">
         <v>272</v>
       </c>
-      <c r="T53" s="104"/>
-      <c r="U53" s="104"/>
-      <c r="V53" s="104"/>
-      <c r="W53" s="104"/>
-      <c r="X53" s="104"/>
-      <c r="Y53" s="104"/>
-      <c r="Z53" s="104"/>
+      <c r="T53" s="102"/>
+      <c r="U53" s="102"/>
+      <c r="V53" s="102"/>
+      <c r="W53" s="102"/>
+      <c r="X53" s="102"/>
+      <c r="Y53" s="102"/>
+      <c r="Z53" s="102"/>
       <c r="AA53" s="43"/>
       <c r="AB53" s="43"/>
       <c r="AC53" s="43"/>
@@ -7470,15 +7470,15 @@
       <c r="R54" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S54" s="104" t="s">
+      <c r="S54" s="102" t="s">
         <v>145</v>
       </c>
-      <c r="T54" s="104"/>
-      <c r="U54" s="104"/>
-      <c r="V54" s="104"/>
-      <c r="W54" s="104"/>
-      <c r="X54" s="104"/>
-      <c r="Y54" s="104"/>
+      <c r="T54" s="102"/>
+      <c r="U54" s="102"/>
+      <c r="V54" s="102"/>
+      <c r="W54" s="102"/>
+      <c r="X54" s="102"/>
+      <c r="Y54" s="102"/>
       <c r="Z54" s="43"/>
       <c r="AA54" s="43"/>
       <c r="AB54" s="43"/>
@@ -7551,16 +7551,16 @@
       <c r="R55" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S55" s="112" t="s">
+      <c r="S55" s="107" t="s">
         <v>260</v>
       </c>
-      <c r="T55" s="112"/>
-      <c r="U55" s="112"/>
-      <c r="V55" s="112"/>
-      <c r="W55" s="112"/>
-      <c r="X55" s="112"/>
-      <c r="Y55" s="112"/>
-      <c r="Z55" s="112"/>
+      <c r="T55" s="107"/>
+      <c r="U55" s="107"/>
+      <c r="V55" s="107"/>
+      <c r="W55" s="107"/>
+      <c r="X55" s="107"/>
+      <c r="Y55" s="107"/>
+      <c r="Z55" s="107"/>
       <c r="AA55" s="75"/>
       <c r="AB55" s="75"/>
       <c r="AC55" s="75"/>
@@ -7632,14 +7632,14 @@
       <c r="R56" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S56" s="112" t="s">
+      <c r="S56" s="107" t="s">
         <v>64</v>
       </c>
-      <c r="T56" s="112"/>
-      <c r="U56" s="112"/>
-      <c r="V56" s="112"/>
-      <c r="W56" s="112"/>
-      <c r="X56" s="112"/>
+      <c r="T56" s="107"/>
+      <c r="U56" s="107"/>
+      <c r="V56" s="107"/>
+      <c r="W56" s="107"/>
+      <c r="X56" s="107"/>
       <c r="Y56" s="75"/>
       <c r="Z56" s="75"/>
       <c r="AA56" s="75"/>
@@ -7713,14 +7713,14 @@
       <c r="R57" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S57" s="112" t="s">
+      <c r="S57" s="107" t="s">
         <v>276</v>
       </c>
-      <c r="T57" s="112"/>
-      <c r="U57" s="112"/>
-      <c r="V57" s="112"/>
-      <c r="W57" s="112"/>
-      <c r="X57" s="112"/>
+      <c r="T57" s="107"/>
+      <c r="U57" s="107"/>
+      <c r="V57" s="107"/>
+      <c r="W57" s="107"/>
+      <c r="X57" s="107"/>
       <c r="Y57" s="75"/>
       <c r="Z57" s="75"/>
       <c r="AA57" s="75"/>
@@ -7794,14 +7794,14 @@
       <c r="R58" s="86" t="s">
         <v>753</v>
       </c>
-      <c r="S58" s="112" t="s">
+      <c r="S58" s="107" t="s">
         <v>278</v>
       </c>
-      <c r="T58" s="112"/>
-      <c r="U58" s="112"/>
-      <c r="V58" s="112"/>
-      <c r="W58" s="112"/>
-      <c r="X58" s="112"/>
+      <c r="T58" s="107"/>
+      <c r="U58" s="107"/>
+      <c r="V58" s="107"/>
+      <c r="W58" s="107"/>
+      <c r="X58" s="107"/>
       <c r="Y58" s="75"/>
       <c r="Z58" s="75"/>
       <c r="AA58" s="75"/>
@@ -7875,15 +7875,15 @@
       <c r="R59" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S59" s="112" t="s">
+      <c r="S59" s="107" t="s">
         <v>68</v>
       </c>
-      <c r="T59" s="112"/>
-      <c r="U59" s="112"/>
-      <c r="V59" s="112"/>
-      <c r="W59" s="112"/>
-      <c r="X59" s="112"/>
-      <c r="Y59" s="112"/>
+      <c r="T59" s="107"/>
+      <c r="U59" s="107"/>
+      <c r="V59" s="107"/>
+      <c r="W59" s="107"/>
+      <c r="X59" s="107"/>
+      <c r="Y59" s="107"/>
       <c r="Z59" s="75"/>
       <c r="AA59" s="75"/>
       <c r="AB59" s="75"/>
@@ -7956,14 +7956,14 @@
       <c r="R60" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S60" s="112" t="s">
+      <c r="S60" s="107" t="s">
         <v>126</v>
       </c>
-      <c r="T60" s="112"/>
-      <c r="U60" s="112"/>
-      <c r="V60" s="112"/>
-      <c r="W60" s="112"/>
-      <c r="X60" s="112"/>
+      <c r="T60" s="107"/>
+      <c r="U60" s="107"/>
+      <c r="V60" s="107"/>
+      <c r="W60" s="107"/>
+      <c r="X60" s="107"/>
       <c r="Y60" s="75"/>
       <c r="Z60" s="75"/>
       <c r="AA60" s="75"/>
@@ -8037,15 +8037,15 @@
       <c r="R61" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S61" s="104" t="s">
+      <c r="S61" s="102" t="s">
         <v>281</v>
       </c>
-      <c r="T61" s="104"/>
-      <c r="U61" s="104"/>
-      <c r="V61" s="104"/>
-      <c r="W61" s="104"/>
-      <c r="X61" s="104"/>
-      <c r="Y61" s="104"/>
+      <c r="T61" s="102"/>
+      <c r="U61" s="102"/>
+      <c r="V61" s="102"/>
+      <c r="W61" s="102"/>
+      <c r="X61" s="102"/>
+      <c r="Y61" s="102"/>
       <c r="Z61" s="43"/>
       <c r="AA61" s="43"/>
       <c r="AB61" s="43"/>
@@ -8118,16 +8118,16 @@
       <c r="R62" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S62" s="104" t="s">
+      <c r="S62" s="102" t="s">
         <v>282</v>
       </c>
-      <c r="T62" s="104"/>
-      <c r="U62" s="104"/>
-      <c r="V62" s="104"/>
-      <c r="W62" s="104"/>
-      <c r="X62" s="104"/>
-      <c r="Y62" s="104"/>
-      <c r="Z62" s="104"/>
+      <c r="T62" s="102"/>
+      <c r="U62" s="102"/>
+      <c r="V62" s="102"/>
+      <c r="W62" s="102"/>
+      <c r="X62" s="102"/>
+      <c r="Y62" s="102"/>
+      <c r="Z62" s="102"/>
       <c r="AA62" s="43"/>
       <c r="AB62" s="43"/>
       <c r="AC62" s="43"/>
@@ -8199,15 +8199,15 @@
       <c r="R63" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S63" s="104" t="s">
+      <c r="S63" s="102" t="s">
         <v>284</v>
       </c>
-      <c r="T63" s="104"/>
-      <c r="U63" s="104"/>
-      <c r="V63" s="104"/>
-      <c r="W63" s="104"/>
-      <c r="X63" s="104"/>
-      <c r="Y63" s="104"/>
+      <c r="T63" s="102"/>
+      <c r="U63" s="102"/>
+      <c r="V63" s="102"/>
+      <c r="W63" s="102"/>
+      <c r="X63" s="102"/>
+      <c r="Y63" s="102"/>
       <c r="Z63" s="43"/>
       <c r="AA63" s="43"/>
       <c r="AB63" s="43"/>
@@ -8280,15 +8280,15 @@
       <c r="R64" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S64" s="104" t="s">
+      <c r="S64" s="102" t="s">
         <v>70</v>
       </c>
-      <c r="T64" s="104"/>
-      <c r="U64" s="104"/>
-      <c r="V64" s="104"/>
-      <c r="W64" s="104"/>
-      <c r="X64" s="104"/>
-      <c r="Y64" s="104"/>
+      <c r="T64" s="102"/>
+      <c r="U64" s="102"/>
+      <c r="V64" s="102"/>
+      <c r="W64" s="102"/>
+      <c r="X64" s="102"/>
+      <c r="Y64" s="102"/>
       <c r="Z64" s="43"/>
       <c r="AA64" s="43"/>
       <c r="AB64" s="43"/>
@@ -8361,16 +8361,16 @@
       <c r="R65" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S65" s="104" t="s">
+      <c r="S65" s="102" t="s">
         <v>286</v>
       </c>
-      <c r="T65" s="104"/>
-      <c r="U65" s="104"/>
-      <c r="V65" s="104"/>
-      <c r="W65" s="104"/>
-      <c r="X65" s="104"/>
-      <c r="Y65" s="104"/>
-      <c r="Z65" s="104"/>
+      <c r="T65" s="102"/>
+      <c r="U65" s="102"/>
+      <c r="V65" s="102"/>
+      <c r="W65" s="102"/>
+      <c r="X65" s="102"/>
+      <c r="Y65" s="102"/>
+      <c r="Z65" s="102"/>
       <c r="AA65" s="43"/>
       <c r="AB65" s="43"/>
       <c r="AC65" s="43"/>
@@ -8442,16 +8442,16 @@
       <c r="R66" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S66" s="104" t="s">
+      <c r="S66" s="102" t="s">
         <v>287</v>
       </c>
-      <c r="T66" s="104"/>
-      <c r="U66" s="104"/>
-      <c r="V66" s="104"/>
-      <c r="W66" s="104"/>
-      <c r="X66" s="104"/>
-      <c r="Y66" s="104"/>
-      <c r="Z66" s="104"/>
+      <c r="T66" s="102"/>
+      <c r="U66" s="102"/>
+      <c r="V66" s="102"/>
+      <c r="W66" s="102"/>
+      <c r="X66" s="102"/>
+      <c r="Y66" s="102"/>
+      <c r="Z66" s="102"/>
       <c r="AA66" s="43"/>
       <c r="AB66" s="43"/>
       <c r="AC66" s="43"/>
@@ -8523,16 +8523,16 @@
       <c r="R67" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S67" s="113" t="s">
+      <c r="S67" s="103" t="s">
         <v>288</v>
       </c>
-      <c r="T67" s="113"/>
-      <c r="U67" s="113"/>
-      <c r="V67" s="113"/>
-      <c r="W67" s="113"/>
-      <c r="X67" s="113"/>
-      <c r="Y67" s="113"/>
-      <c r="Z67" s="113"/>
+      <c r="T67" s="103"/>
+      <c r="U67" s="103"/>
+      <c r="V67" s="103"/>
+      <c r="W67" s="103"/>
+      <c r="X67" s="103"/>
+      <c r="Y67" s="103"/>
+      <c r="Z67" s="103"/>
       <c r="AA67" s="82"/>
       <c r="AB67" s="82"/>
       <c r="AC67" s="82"/>
@@ -8604,16 +8604,16 @@
       <c r="R68" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S68" s="113" t="s">
+      <c r="S68" s="103" t="s">
         <v>288</v>
       </c>
-      <c r="T68" s="113"/>
-      <c r="U68" s="113"/>
-      <c r="V68" s="113"/>
-      <c r="W68" s="113"/>
-      <c r="X68" s="113"/>
-      <c r="Y68" s="113"/>
-      <c r="Z68" s="113"/>
+      <c r="T68" s="103"/>
+      <c r="U68" s="103"/>
+      <c r="V68" s="103"/>
+      <c r="W68" s="103"/>
+      <c r="X68" s="103"/>
+      <c r="Y68" s="103"/>
+      <c r="Z68" s="103"/>
       <c r="AA68" s="82"/>
       <c r="AB68" s="82"/>
       <c r="AC68" s="82"/>
@@ -8685,16 +8685,16 @@
       <c r="R69" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S69" s="113" t="s">
+      <c r="S69" s="103" t="s">
         <v>289</v>
       </c>
-      <c r="T69" s="113"/>
-      <c r="U69" s="113"/>
-      <c r="V69" s="113"/>
-      <c r="W69" s="113"/>
-      <c r="X69" s="113"/>
-      <c r="Y69" s="113"/>
-      <c r="Z69" s="113"/>
+      <c r="T69" s="103"/>
+      <c r="U69" s="103"/>
+      <c r="V69" s="103"/>
+      <c r="W69" s="103"/>
+      <c r="X69" s="103"/>
+      <c r="Y69" s="103"/>
+      <c r="Z69" s="103"/>
       <c r="AA69" s="82"/>
       <c r="AB69" s="82"/>
       <c r="AC69" s="82"/>
@@ -8758,15 +8758,15 @@
         <v>748</v>
       </c>
       <c r="R70" s="86"/>
-      <c r="S70" s="104" t="s">
+      <c r="S70" s="102" t="s">
         <v>75</v>
       </c>
-      <c r="T70" s="104"/>
-      <c r="U70" s="104"/>
-      <c r="V70" s="104"/>
-      <c r="W70" s="104"/>
-      <c r="X70" s="104"/>
-      <c r="Y70" s="104"/>
+      <c r="T70" s="102"/>
+      <c r="U70" s="102"/>
+      <c r="V70" s="102"/>
+      <c r="W70" s="102"/>
+      <c r="X70" s="102"/>
+      <c r="Y70" s="102"/>
       <c r="Z70" s="43"/>
       <c r="AA70" s="43"/>
       <c r="AB70" s="43"/>
@@ -8831,14 +8831,14 @@
         <v>748</v>
       </c>
       <c r="R71" s="86"/>
-      <c r="S71" s="104" t="s">
+      <c r="S71" s="102" t="s">
         <v>89</v>
       </c>
-      <c r="T71" s="104"/>
-      <c r="U71" s="104"/>
-      <c r="V71" s="104"/>
-      <c r="W71" s="104"/>
-      <c r="X71" s="104"/>
+      <c r="T71" s="102"/>
+      <c r="U71" s="102"/>
+      <c r="V71" s="102"/>
+      <c r="W71" s="102"/>
+      <c r="X71" s="102"/>
       <c r="Y71" s="43"/>
       <c r="Z71" s="43"/>
       <c r="AA71" s="43"/>
@@ -8908,16 +8908,16 @@
       <c r="R72" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S72" s="103" t="s">
+      <c r="S72" s="105" t="s">
         <v>91</v>
       </c>
-      <c r="T72" s="103"/>
-      <c r="U72" s="103"/>
-      <c r="V72" s="103"/>
-      <c r="W72" s="103"/>
-      <c r="X72" s="103"/>
-      <c r="Y72" s="103"/>
-      <c r="Z72" s="103"/>
+      <c r="T72" s="105"/>
+      <c r="U72" s="105"/>
+      <c r="V72" s="105"/>
+      <c r="W72" s="105"/>
+      <c r="X72" s="105"/>
+      <c r="Y72" s="105"/>
+      <c r="Z72" s="105"/>
       <c r="AA72" s="51"/>
       <c r="AB72" s="43"/>
       <c r="AC72" s="43"/>
@@ -8956,10 +8956,10 @@
       <c r="G73" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="H73" s="103" t="s">
+      <c r="H73" s="105" t="s">
         <v>10</v>
       </c>
-      <c r="I73" s="103"/>
+      <c r="I73" s="105"/>
       <c r="J73" s="51" t="s">
         <v>213</v>
       </c>
@@ -8987,15 +8987,15 @@
       <c r="R73" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S73" s="103" t="s">
+      <c r="S73" s="105" t="s">
         <v>293</v>
       </c>
-      <c r="T73" s="103"/>
-      <c r="U73" s="103"/>
-      <c r="V73" s="103"/>
-      <c r="W73" s="103"/>
-      <c r="X73" s="103"/>
-      <c r="Y73" s="103"/>
+      <c r="T73" s="105"/>
+      <c r="U73" s="105"/>
+      <c r="V73" s="105"/>
+      <c r="W73" s="105"/>
+      <c r="X73" s="105"/>
+      <c r="Y73" s="105"/>
       <c r="Z73" s="51"/>
       <c r="AA73" s="51"/>
       <c r="AB73" s="43"/>
@@ -9035,10 +9035,10 @@
       <c r="G74" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="H74" s="103" t="s">
+      <c r="H74" s="105" t="s">
         <v>10</v>
       </c>
-      <c r="I74" s="103"/>
+      <c r="I74" s="105"/>
       <c r="J74" s="51" t="s">
         <v>213</v>
       </c>
@@ -9066,16 +9066,16 @@
       <c r="R74" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S74" s="103" t="s">
+      <c r="S74" s="105" t="s">
         <v>106</v>
       </c>
-      <c r="T74" s="103"/>
-      <c r="U74" s="103"/>
-      <c r="V74" s="103"/>
-      <c r="W74" s="103"/>
-      <c r="X74" s="103"/>
-      <c r="Y74" s="103"/>
-      <c r="Z74" s="103"/>
+      <c r="T74" s="105"/>
+      <c r="U74" s="105"/>
+      <c r="V74" s="105"/>
+      <c r="W74" s="105"/>
+      <c r="X74" s="105"/>
+      <c r="Y74" s="105"/>
+      <c r="Z74" s="105"/>
       <c r="AA74" s="51"/>
       <c r="AB74" s="43"/>
       <c r="AC74" s="43"/>
@@ -9145,15 +9145,15 @@
       <c r="R75" s="86" t="s">
         <v>740</v>
       </c>
-      <c r="S75" s="103" t="s">
+      <c r="S75" s="105" t="s">
         <v>152</v>
       </c>
-      <c r="T75" s="103"/>
-      <c r="U75" s="103"/>
-      <c r="V75" s="103"/>
-      <c r="W75" s="103"/>
-      <c r="X75" s="103"/>
-      <c r="Y75" s="103"/>
+      <c r="T75" s="105"/>
+      <c r="U75" s="105"/>
+      <c r="V75" s="105"/>
+      <c r="W75" s="105"/>
+      <c r="X75" s="105"/>
+      <c r="Y75" s="105"/>
       <c r="Z75" s="51"/>
       <c r="AA75" s="51"/>
       <c r="AB75" s="43"/>
@@ -9193,10 +9193,10 @@
       <c r="G76" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="H76" s="103" t="s">
+      <c r="H76" s="105" t="s">
         <v>10</v>
       </c>
-      <c r="I76" s="103"/>
+      <c r="I76" s="105"/>
       <c r="J76" s="51" t="s">
         <v>213</v>
       </c>
@@ -9224,15 +9224,15 @@
       <c r="R76" s="86" t="s">
         <v>674</v>
       </c>
-      <c r="S76" s="103" t="s">
+      <c r="S76" s="105" t="s">
         <v>296</v>
       </c>
-      <c r="T76" s="103"/>
-      <c r="U76" s="103"/>
-      <c r="V76" s="103"/>
-      <c r="W76" s="103"/>
-      <c r="X76" s="103"/>
-      <c r="Y76" s="103"/>
+      <c r="T76" s="105"/>
+      <c r="U76" s="105"/>
+      <c r="V76" s="105"/>
+      <c r="W76" s="105"/>
+      <c r="X76" s="105"/>
+      <c r="Y76" s="105"/>
       <c r="Z76" s="51"/>
       <c r="AA76" s="51"/>
       <c r="AB76" s="43"/>
@@ -9305,16 +9305,16 @@
       <c r="R77" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S77" s="103" t="s">
+      <c r="S77" s="105" t="s">
         <v>297</v>
       </c>
-      <c r="T77" s="103"/>
-      <c r="U77" s="103"/>
-      <c r="V77" s="103"/>
-      <c r="W77" s="103"/>
-      <c r="X77" s="103"/>
-      <c r="Y77" s="103"/>
-      <c r="Z77" s="103"/>
+      <c r="T77" s="105"/>
+      <c r="U77" s="105"/>
+      <c r="V77" s="105"/>
+      <c r="W77" s="105"/>
+      <c r="X77" s="105"/>
+      <c r="Y77" s="105"/>
+      <c r="Z77" s="105"/>
       <c r="AA77" s="51"/>
       <c r="AB77" s="43"/>
       <c r="AC77" s="43"/>
@@ -9386,16 +9386,16 @@
       <c r="R78" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S78" s="111" t="s">
+      <c r="S78" s="106" t="s">
         <v>295</v>
       </c>
-      <c r="T78" s="111"/>
-      <c r="U78" s="111"/>
-      <c r="V78" s="111"/>
-      <c r="W78" s="111"/>
-      <c r="X78" s="111"/>
-      <c r="Y78" s="111"/>
-      <c r="Z78" s="111"/>
+      <c r="T78" s="106"/>
+      <c r="U78" s="106"/>
+      <c r="V78" s="106"/>
+      <c r="W78" s="106"/>
+      <c r="X78" s="106"/>
+      <c r="Y78" s="106"/>
+      <c r="Z78" s="106"/>
       <c r="AA78" s="44"/>
       <c r="AB78" s="43"/>
       <c r="AC78" s="43"/>
@@ -9467,14 +9467,14 @@
       <c r="R79" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S79" s="104" t="s">
+      <c r="S79" s="102" t="s">
         <v>301</v>
       </c>
-      <c r="T79" s="104"/>
-      <c r="U79" s="104"/>
-      <c r="V79" s="104"/>
-      <c r="W79" s="104"/>
-      <c r="X79" s="104"/>
+      <c r="T79" s="102"/>
+      <c r="U79" s="102"/>
+      <c r="V79" s="102"/>
+      <c r="W79" s="102"/>
+      <c r="X79" s="102"/>
       <c r="Y79" s="43"/>
       <c r="Z79" s="43"/>
       <c r="AA79" s="43"/>
@@ -9548,15 +9548,15 @@
       <c r="R80" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S80" s="104" t="s">
+      <c r="S80" s="102" t="s">
         <v>303</v>
       </c>
-      <c r="T80" s="104"/>
-      <c r="U80" s="104"/>
-      <c r="V80" s="104"/>
-      <c r="W80" s="104"/>
-      <c r="X80" s="104"/>
-      <c r="Y80" s="104"/>
+      <c r="T80" s="102"/>
+      <c r="U80" s="102"/>
+      <c r="V80" s="102"/>
+      <c r="W80" s="102"/>
+      <c r="X80" s="102"/>
+      <c r="Y80" s="102"/>
       <c r="Z80" s="43"/>
       <c r="AA80" s="43"/>
       <c r="AB80" s="43"/>
@@ -9629,13 +9629,13 @@
       <c r="R81" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S81" s="104" t="s">
+      <c r="S81" s="102" t="s">
         <v>305</v>
       </c>
-      <c r="T81" s="104"/>
-      <c r="U81" s="104"/>
-      <c r="V81" s="104"/>
-      <c r="W81" s="104"/>
+      <c r="T81" s="102"/>
+      <c r="U81" s="102"/>
+      <c r="V81" s="102"/>
+      <c r="W81" s="102"/>
       <c r="X81" s="43"/>
       <c r="Y81" s="43"/>
       <c r="Z81" s="43"/>
@@ -9710,17 +9710,17 @@
       <c r="R82" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S82" s="104" t="s">
+      <c r="S82" s="102" t="s">
         <v>307</v>
       </c>
-      <c r="T82" s="104"/>
-      <c r="U82" s="104"/>
-      <c r="V82" s="104"/>
-      <c r="W82" s="104"/>
-      <c r="X82" s="104"/>
-      <c r="Y82" s="104"/>
-      <c r="Z82" s="104"/>
-      <c r="AA82" s="104"/>
+      <c r="T82" s="102"/>
+      <c r="U82" s="102"/>
+      <c r="V82" s="102"/>
+      <c r="W82" s="102"/>
+      <c r="X82" s="102"/>
+      <c r="Y82" s="102"/>
+      <c r="Z82" s="102"/>
+      <c r="AA82" s="102"/>
       <c r="AB82" s="43"/>
       <c r="AC82" s="43"/>
       <c r="AD82" s="43"/>
@@ -9791,15 +9791,15 @@
       <c r="R83" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S83" s="104" t="s">
+      <c r="S83" s="102" t="s">
         <v>309</v>
       </c>
-      <c r="T83" s="104"/>
-      <c r="U83" s="104"/>
-      <c r="V83" s="104"/>
-      <c r="W83" s="104"/>
-      <c r="X83" s="104"/>
-      <c r="Y83" s="104"/>
+      <c r="T83" s="102"/>
+      <c r="U83" s="102"/>
+      <c r="V83" s="102"/>
+      <c r="W83" s="102"/>
+      <c r="X83" s="102"/>
+      <c r="Y83" s="102"/>
       <c r="Z83" s="43"/>
       <c r="AA83" s="43"/>
       <c r="AB83" s="43"/>
@@ -9872,14 +9872,14 @@
       <c r="R84" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S84" s="104" t="s">
+      <c r="S84" s="102" t="s">
         <v>311</v>
       </c>
-      <c r="T84" s="104"/>
-      <c r="U84" s="104"/>
-      <c r="V84" s="104"/>
-      <c r="W84" s="104"/>
-      <c r="X84" s="104"/>
+      <c r="T84" s="102"/>
+      <c r="U84" s="102"/>
+      <c r="V84" s="102"/>
+      <c r="W84" s="102"/>
+      <c r="X84" s="102"/>
       <c r="Y84" s="43"/>
       <c r="Z84" s="43"/>
       <c r="AA84" s="43"/>
@@ -9953,14 +9953,14 @@
       <c r="R85" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S85" s="104" t="s">
+      <c r="S85" s="102" t="s">
         <v>313</v>
       </c>
-      <c r="T85" s="104"/>
-      <c r="U85" s="104"/>
-      <c r="V85" s="104"/>
-      <c r="W85" s="104"/>
-      <c r="X85" s="104"/>
+      <c r="T85" s="102"/>
+      <c r="U85" s="102"/>
+      <c r="V85" s="102"/>
+      <c r="W85" s="102"/>
+      <c r="X85" s="102"/>
       <c r="Y85" s="43"/>
       <c r="Z85" s="43"/>
       <c r="AA85" s="43"/>
@@ -10034,14 +10034,14 @@
       <c r="R86" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S86" s="104" t="s">
+      <c r="S86" s="102" t="s">
         <v>315</v>
       </c>
-      <c r="T86" s="104"/>
-      <c r="U86" s="104"/>
-      <c r="V86" s="104"/>
-      <c r="W86" s="104"/>
-      <c r="X86" s="104"/>
+      <c r="T86" s="102"/>
+      <c r="U86" s="102"/>
+      <c r="V86" s="102"/>
+      <c r="W86" s="102"/>
+      <c r="X86" s="102"/>
       <c r="Y86" s="43"/>
       <c r="Z86" s="43"/>
       <c r="AA86" s="43"/>
@@ -10115,14 +10115,14 @@
       <c r="R87" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S87" s="104" t="s">
+      <c r="S87" s="102" t="s">
         <v>317</v>
       </c>
-      <c r="T87" s="104"/>
-      <c r="U87" s="104"/>
-      <c r="V87" s="104"/>
-      <c r="W87" s="104"/>
-      <c r="X87" s="104"/>
+      <c r="T87" s="102"/>
+      <c r="U87" s="102"/>
+      <c r="V87" s="102"/>
+      <c r="W87" s="102"/>
+      <c r="X87" s="102"/>
       <c r="Y87" s="43"/>
       <c r="Z87" s="43"/>
       <c r="AA87" s="43"/>
@@ -10194,15 +10194,15 @@
       <c r="R88" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S88" s="104" t="s">
+      <c r="S88" s="102" t="s">
         <v>321</v>
       </c>
-      <c r="T88" s="104"/>
-      <c r="U88" s="104"/>
-      <c r="V88" s="104"/>
-      <c r="W88" s="104"/>
-      <c r="X88" s="104"/>
-      <c r="Y88" s="104"/>
+      <c r="T88" s="102"/>
+      <c r="U88" s="102"/>
+      <c r="V88" s="102"/>
+      <c r="W88" s="102"/>
+      <c r="X88" s="102"/>
+      <c r="Y88" s="102"/>
       <c r="Z88" s="43"/>
       <c r="AA88" s="43"/>
       <c r="AB88" s="43"/>
@@ -10240,10 +10240,10 @@
       <c r="G89" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="H89" s="104" t="s">
+      <c r="H89" s="102" t="s">
         <v>17</v>
       </c>
-      <c r="I89" s="104"/>
+      <c r="I89" s="102"/>
       <c r="J89" s="43" t="s">
         <v>213</v>
       </c>
@@ -10271,15 +10271,15 @@
       <c r="R89" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S89" s="104" t="s">
+      <c r="S89" s="102" t="s">
         <v>323</v>
       </c>
-      <c r="T89" s="104"/>
-      <c r="U89" s="104"/>
-      <c r="V89" s="104"/>
-      <c r="W89" s="104"/>
-      <c r="X89" s="104"/>
-      <c r="Y89" s="104"/>
+      <c r="T89" s="102"/>
+      <c r="U89" s="102"/>
+      <c r="V89" s="102"/>
+      <c r="W89" s="102"/>
+      <c r="X89" s="102"/>
+      <c r="Y89" s="102"/>
       <c r="Z89" s="43"/>
       <c r="AA89" s="43"/>
       <c r="AB89" s="43"/>
@@ -10350,15 +10350,15 @@
       <c r="R90" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S90" s="104" t="s">
+      <c r="S90" s="102" t="s">
         <v>325</v>
       </c>
-      <c r="T90" s="104"/>
-      <c r="U90" s="104"/>
-      <c r="V90" s="104"/>
-      <c r="W90" s="104"/>
-      <c r="X90" s="104"/>
-      <c r="Y90" s="104"/>
+      <c r="T90" s="102"/>
+      <c r="U90" s="102"/>
+      <c r="V90" s="102"/>
+      <c r="W90" s="102"/>
+      <c r="X90" s="102"/>
+      <c r="Y90" s="102"/>
       <c r="Z90" s="43"/>
       <c r="AA90" s="43"/>
       <c r="AB90" s="43"/>
@@ -10389,10 +10389,10 @@
       <c r="D91" s="51" t="s">
         <v>326</v>
       </c>
-      <c r="E91" s="103" t="s">
+      <c r="E91" s="105" t="s">
         <v>327</v>
       </c>
-      <c r="F91" s="103"/>
+      <c r="F91" s="105"/>
       <c r="G91" s="51" t="s">
         <v>604</v>
       </c>
@@ -10429,16 +10429,16 @@
       <c r="R91" s="86" t="s">
         <v>689</v>
       </c>
-      <c r="S91" s="103" t="s">
+      <c r="S91" s="105" t="s">
         <v>80</v>
       </c>
-      <c r="T91" s="103"/>
-      <c r="U91" s="103"/>
-      <c r="V91" s="103"/>
-      <c r="W91" s="103"/>
-      <c r="X91" s="103"/>
-      <c r="Y91" s="103"/>
-      <c r="Z91" s="103"/>
+      <c r="T91" s="105"/>
+      <c r="U91" s="105"/>
+      <c r="V91" s="105"/>
+      <c r="W91" s="105"/>
+      <c r="X91" s="105"/>
+      <c r="Y91" s="105"/>
+      <c r="Z91" s="105"/>
       <c r="AA91" s="51"/>
       <c r="AB91" s="51"/>
       <c r="AC91" s="51"/>
@@ -10468,10 +10468,10 @@
       <c r="D92" s="51" t="s">
         <v>326</v>
       </c>
-      <c r="E92" s="103" t="s">
+      <c r="E92" s="105" t="s">
         <v>327</v>
       </c>
-      <c r="F92" s="103"/>
+      <c r="F92" s="105"/>
       <c r="G92" s="51" t="s">
         <v>604</v>
       </c>
@@ -10508,16 +10508,16 @@
       <c r="R92" s="86" t="s">
         <v>610</v>
       </c>
-      <c r="S92" s="103" t="s">
+      <c r="S92" s="105" t="s">
         <v>328</v>
       </c>
-      <c r="T92" s="103"/>
-      <c r="U92" s="103"/>
-      <c r="V92" s="103"/>
-      <c r="W92" s="103"/>
-      <c r="X92" s="103"/>
-      <c r="Y92" s="103"/>
-      <c r="Z92" s="103"/>
+      <c r="T92" s="105"/>
+      <c r="U92" s="105"/>
+      <c r="V92" s="105"/>
+      <c r="W92" s="105"/>
+      <c r="X92" s="105"/>
+      <c r="Y92" s="105"/>
+      <c r="Z92" s="105"/>
       <c r="AA92" s="51"/>
       <c r="AB92" s="51"/>
       <c r="AC92" s="51"/>
@@ -10547,10 +10547,10 @@
       <c r="D93" s="51" t="s">
         <v>326</v>
       </c>
-      <c r="E93" s="103" t="s">
+      <c r="E93" s="105" t="s">
         <v>327</v>
       </c>
-      <c r="F93" s="103"/>
+      <c r="F93" s="105"/>
       <c r="G93" s="51" t="s">
         <v>604</v>
       </c>
@@ -10583,16 +10583,16 @@
         <v>628</v>
       </c>
       <c r="R93" s="86"/>
-      <c r="S93" s="103" t="s">
+      <c r="S93" s="105" t="s">
         <v>329</v>
       </c>
-      <c r="T93" s="103"/>
-      <c r="U93" s="103"/>
-      <c r="V93" s="103"/>
-      <c r="W93" s="103"/>
-      <c r="X93" s="103"/>
-      <c r="Y93" s="103"/>
-      <c r="Z93" s="103"/>
+      <c r="T93" s="105"/>
+      <c r="U93" s="105"/>
+      <c r="V93" s="105"/>
+      <c r="W93" s="105"/>
+      <c r="X93" s="105"/>
+      <c r="Y93" s="105"/>
+      <c r="Z93" s="105"/>
       <c r="AA93" s="51"/>
       <c r="AB93" s="51"/>
       <c r="AC93" s="51"/>
@@ -10664,17 +10664,17 @@
       <c r="R94" s="86" t="s">
         <v>662</v>
       </c>
-      <c r="S94" s="104" t="s">
+      <c r="S94" s="102" t="s">
         <v>174</v>
       </c>
-      <c r="T94" s="104"/>
-      <c r="U94" s="104"/>
-      <c r="V94" s="104"/>
-      <c r="W94" s="104"/>
-      <c r="X94" s="104"/>
-      <c r="Y94" s="104"/>
-      <c r="Z94" s="104"/>
-      <c r="AA94" s="104"/>
+      <c r="T94" s="102"/>
+      <c r="U94" s="102"/>
+      <c r="V94" s="102"/>
+      <c r="W94" s="102"/>
+      <c r="X94" s="102"/>
+      <c r="Y94" s="102"/>
+      <c r="Z94" s="102"/>
+      <c r="AA94" s="102"/>
       <c r="AB94" s="43"/>
       <c r="AC94" s="43"/>
       <c r="AD94" s="43"/>
@@ -10703,10 +10703,10 @@
       <c r="D95" s="43" t="s">
         <v>601</v>
       </c>
-      <c r="E95" s="104" t="s">
+      <c r="E95" s="102" t="s">
         <v>331</v>
       </c>
-      <c r="F95" s="104"/>
+      <c r="F95" s="102"/>
       <c r="G95" s="43" t="s">
         <v>7</v>
       </c>
@@ -10739,15 +10739,15 @@
         <v>682</v>
       </c>
       <c r="R95" s="86"/>
-      <c r="S95" s="104" t="s">
+      <c r="S95" s="102" t="s">
         <v>150</v>
       </c>
-      <c r="T95" s="104"/>
-      <c r="U95" s="104"/>
-      <c r="V95" s="104"/>
-      <c r="W95" s="104"/>
-      <c r="X95" s="104"/>
-      <c r="Y95" s="104"/>
+      <c r="T95" s="102"/>
+      <c r="U95" s="102"/>
+      <c r="V95" s="102"/>
+      <c r="W95" s="102"/>
+      <c r="X95" s="102"/>
+      <c r="Y95" s="102"/>
       <c r="Z95" s="43"/>
       <c r="AA95" s="43"/>
       <c r="AB95" s="43"/>
@@ -10778,10 +10778,10 @@
       <c r="D96" s="43" t="s">
         <v>601</v>
       </c>
-      <c r="E96" s="104" t="s">
+      <c r="E96" s="102" t="s">
         <v>331</v>
       </c>
-      <c r="F96" s="104"/>
+      <c r="F96" s="102"/>
       <c r="G96" s="43" t="s">
         <v>7</v>
       </c>
@@ -10812,16 +10812,16 @@
         <v>680</v>
       </c>
       <c r="R96" s="86"/>
-      <c r="S96" s="104" t="s">
+      <c r="S96" s="102" t="s">
         <v>172</v>
       </c>
-      <c r="T96" s="104"/>
-      <c r="U96" s="104"/>
-      <c r="V96" s="104"/>
-      <c r="W96" s="104"/>
-      <c r="X96" s="104"/>
-      <c r="Y96" s="104"/>
-      <c r="Z96" s="104"/>
+      <c r="T96" s="102"/>
+      <c r="U96" s="102"/>
+      <c r="V96" s="102"/>
+      <c r="W96" s="102"/>
+      <c r="X96" s="102"/>
+      <c r="Y96" s="102"/>
+      <c r="Z96" s="102"/>
       <c r="AA96" s="43"/>
       <c r="AB96" s="43"/>
       <c r="AC96" s="43"/>
@@ -10851,10 +10851,10 @@
       <c r="D97" s="43" t="s">
         <v>601</v>
       </c>
-      <c r="E97" s="104" t="s">
+      <c r="E97" s="102" t="s">
         <v>331</v>
       </c>
-      <c r="F97" s="104"/>
+      <c r="F97" s="102"/>
       <c r="G97" s="43" t="s">
         <v>7</v>
       </c>
@@ -10889,16 +10889,16 @@
         <v>679</v>
       </c>
       <c r="R97" s="86"/>
-      <c r="S97" s="104" t="s">
+      <c r="S97" s="102" t="s">
         <v>182</v>
       </c>
-      <c r="T97" s="104"/>
-      <c r="U97" s="104"/>
-      <c r="V97" s="104"/>
-      <c r="W97" s="104"/>
-      <c r="X97" s="104"/>
-      <c r="Y97" s="104"/>
-      <c r="Z97" s="104"/>
+      <c r="T97" s="102"/>
+      <c r="U97" s="102"/>
+      <c r="V97" s="102"/>
+      <c r="W97" s="102"/>
+      <c r="X97" s="102"/>
+      <c r="Y97" s="102"/>
+      <c r="Z97" s="102"/>
       <c r="AA97" s="43"/>
       <c r="AB97" s="43"/>
       <c r="AC97" s="43"/>
@@ -10966,16 +10966,16 @@
       <c r="R98" s="86" t="s">
         <v>612</v>
       </c>
-      <c r="S98" s="105" t="s">
+      <c r="S98" s="104" t="s">
         <v>102</v>
       </c>
-      <c r="T98" s="105"/>
-      <c r="U98" s="105"/>
-      <c r="V98" s="105"/>
-      <c r="W98" s="105"/>
-      <c r="X98" s="105"/>
-      <c r="Y98" s="105"/>
-      <c r="Z98" s="105"/>
+      <c r="T98" s="104"/>
+      <c r="U98" s="104"/>
+      <c r="V98" s="104"/>
+      <c r="W98" s="104"/>
+      <c r="X98" s="104"/>
+      <c r="Y98" s="104"/>
+      <c r="Z98" s="104"/>
       <c r="AA98" s="65"/>
       <c r="AB98" s="65"/>
       <c r="AC98" s="65"/>
@@ -11043,16 +11043,16 @@
       <c r="R99" s="86" t="s">
         <v>674</v>
       </c>
-      <c r="S99" s="105" t="s">
+      <c r="S99" s="104" t="s">
         <v>259</v>
       </c>
-      <c r="T99" s="105"/>
-      <c r="U99" s="105"/>
-      <c r="V99" s="105"/>
-      <c r="W99" s="105"/>
-      <c r="X99" s="105"/>
-      <c r="Y99" s="105"/>
-      <c r="Z99" s="105"/>
+      <c r="T99" s="104"/>
+      <c r="U99" s="104"/>
+      <c r="V99" s="104"/>
+      <c r="W99" s="104"/>
+      <c r="X99" s="104"/>
+      <c r="Y99" s="104"/>
+      <c r="Z99" s="104"/>
       <c r="AA99" s="65"/>
       <c r="AB99" s="65"/>
       <c r="AC99" s="65"/>
@@ -11120,16 +11120,16 @@
       <c r="R100" s="86" t="s">
         <v>672</v>
       </c>
-      <c r="S100" s="105" t="s">
+      <c r="S100" s="104" t="s">
         <v>187</v>
       </c>
-      <c r="T100" s="105"/>
-      <c r="U100" s="105"/>
-      <c r="V100" s="105"/>
-      <c r="W100" s="105"/>
-      <c r="X100" s="105"/>
-      <c r="Y100" s="105"/>
-      <c r="Z100" s="105"/>
+      <c r="T100" s="104"/>
+      <c r="U100" s="104"/>
+      <c r="V100" s="104"/>
+      <c r="W100" s="104"/>
+      <c r="X100" s="104"/>
+      <c r="Y100" s="104"/>
+      <c r="Z100" s="104"/>
       <c r="AA100" s="65"/>
       <c r="AB100" s="65"/>
       <c r="AC100" s="65"/>
@@ -11793,24 +11793,24 @@
     </row>
     <row r="116" spans="1:41" ht="12.75">
       <c r="A116" s="80"/>
-      <c r="B116" s="102"/>
-      <c r="C116" s="102"/>
-      <c r="D116" s="102"/>
-      <c r="E116" s="102"/>
-      <c r="F116" s="102"/>
-      <c r="G116" s="102"/>
-      <c r="H116" s="102"/>
-      <c r="I116" s="102"/>
-      <c r="J116" s="102"/>
-      <c r="K116" s="102"/>
-      <c r="L116" s="102"/>
-      <c r="M116" s="102"/>
-      <c r="N116" s="102"/>
-      <c r="O116" s="102"/>
-      <c r="P116" s="102"/>
-      <c r="Q116" s="102"/>
-      <c r="R116" s="102"/>
-      <c r="S116" s="102"/>
+      <c r="B116" s="113"/>
+      <c r="C116" s="113"/>
+      <c r="D116" s="113"/>
+      <c r="E116" s="113"/>
+      <c r="F116" s="113"/>
+      <c r="G116" s="113"/>
+      <c r="H116" s="113"/>
+      <c r="I116" s="113"/>
+      <c r="J116" s="113"/>
+      <c r="K116" s="113"/>
+      <c r="L116" s="113"/>
+      <c r="M116" s="113"/>
+      <c r="N116" s="113"/>
+      <c r="O116" s="113"/>
+      <c r="P116" s="113"/>
+      <c r="Q116" s="113"/>
+      <c r="R116" s="113"/>
+      <c r="S116" s="113"/>
       <c r="T116" s="80"/>
       <c r="U116" s="80"/>
       <c r="V116" s="80"/>
@@ -12137,24 +12137,24 @@
     </row>
     <row r="124" spans="1:41" ht="12.75">
       <c r="A124" s="80"/>
-      <c r="B124" s="102"/>
-      <c r="C124" s="102"/>
-      <c r="D124" s="102"/>
-      <c r="E124" s="102"/>
-      <c r="F124" s="102"/>
-      <c r="G124" s="102"/>
-      <c r="H124" s="102"/>
-      <c r="I124" s="102"/>
-      <c r="J124" s="102"/>
-      <c r="K124" s="102"/>
-      <c r="L124" s="102"/>
-      <c r="M124" s="102"/>
-      <c r="N124" s="102"/>
-      <c r="O124" s="102"/>
-      <c r="P124" s="102"/>
-      <c r="Q124" s="102"/>
-      <c r="R124" s="102"/>
-      <c r="S124" s="102"/>
+      <c r="B124" s="113"/>
+      <c r="C124" s="113"/>
+      <c r="D124" s="113"/>
+      <c r="E124" s="113"/>
+      <c r="F124" s="113"/>
+      <c r="G124" s="113"/>
+      <c r="H124" s="113"/>
+      <c r="I124" s="113"/>
+      <c r="J124" s="113"/>
+      <c r="K124" s="113"/>
+      <c r="L124" s="113"/>
+      <c r="M124" s="113"/>
+      <c r="N124" s="113"/>
+      <c r="O124" s="113"/>
+      <c r="P124" s="113"/>
+      <c r="Q124" s="113"/>
+      <c r="R124" s="113"/>
+      <c r="S124" s="113"/>
       <c r="T124" s="80"/>
       <c r="U124" s="80"/>
       <c r="V124" s="80"/>
@@ -12395,24 +12395,24 @@
     </row>
     <row r="130" spans="1:41" ht="12.75">
       <c r="A130" s="80"/>
-      <c r="B130" s="102"/>
-      <c r="C130" s="102"/>
-      <c r="D130" s="102"/>
-      <c r="E130" s="102"/>
-      <c r="F130" s="102"/>
-      <c r="G130" s="102"/>
-      <c r="H130" s="102"/>
-      <c r="I130" s="102"/>
-      <c r="J130" s="102"/>
-      <c r="K130" s="102"/>
-      <c r="L130" s="102"/>
-      <c r="M130" s="102"/>
-      <c r="N130" s="102"/>
-      <c r="O130" s="102"/>
-      <c r="P130" s="102"/>
-      <c r="Q130" s="102"/>
-      <c r="R130" s="102"/>
-      <c r="S130" s="102"/>
+      <c r="B130" s="113"/>
+      <c r="C130" s="113"/>
+      <c r="D130" s="113"/>
+      <c r="E130" s="113"/>
+      <c r="F130" s="113"/>
+      <c r="G130" s="113"/>
+      <c r="H130" s="113"/>
+      <c r="I130" s="113"/>
+      <c r="J130" s="113"/>
+      <c r="K130" s="113"/>
+      <c r="L130" s="113"/>
+      <c r="M130" s="113"/>
+      <c r="N130" s="113"/>
+      <c r="O130" s="113"/>
+      <c r="P130" s="113"/>
+      <c r="Q130" s="113"/>
+      <c r="R130" s="113"/>
+      <c r="S130" s="113"/>
       <c r="T130" s="80"/>
       <c r="U130" s="80"/>
       <c r="V130" s="80"/>
@@ -12782,20 +12782,20 @@
     </row>
     <row r="139" spans="1:41" ht="12.75">
       <c r="A139" s="80"/>
-      <c r="B139" s="102"/>
-      <c r="C139" s="102"/>
-      <c r="D139" s="102"/>
-      <c r="E139" s="102"/>
-      <c r="F139" s="102"/>
-      <c r="G139" s="102"/>
-      <c r="H139" s="102"/>
-      <c r="I139" s="102"/>
-      <c r="J139" s="102"/>
-      <c r="K139" s="102"/>
-      <c r="L139" s="102"/>
-      <c r="M139" s="102"/>
-      <c r="N139" s="102"/>
-      <c r="O139" s="102"/>
+      <c r="B139" s="113"/>
+      <c r="C139" s="113"/>
+      <c r="D139" s="113"/>
+      <c r="E139" s="113"/>
+      <c r="F139" s="113"/>
+      <c r="G139" s="113"/>
+      <c r="H139" s="113"/>
+      <c r="I139" s="113"/>
+      <c r="J139" s="113"/>
+      <c r="K139" s="113"/>
+      <c r="L139" s="113"/>
+      <c r="M139" s="113"/>
+      <c r="N139" s="113"/>
+      <c r="O139" s="113"/>
       <c r="P139" s="93"/>
       <c r="Q139" s="93"/>
       <c r="R139" s="93"/>
@@ -49505,6 +49505,98 @@
   </sheetData>
   <autoFilter ref="A1:AI895" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <mergeCells count="116">
+    <mergeCell ref="B116:S116"/>
+    <mergeCell ref="B124:S124"/>
+    <mergeCell ref="B130:S130"/>
+    <mergeCell ref="B139:O139"/>
+    <mergeCell ref="E91:F91"/>
+    <mergeCell ref="S91:Z91"/>
+    <mergeCell ref="E92:F92"/>
+    <mergeCell ref="S92:Z92"/>
+    <mergeCell ref="E93:F93"/>
+    <mergeCell ref="S93:Z93"/>
+    <mergeCell ref="S94:AA94"/>
+    <mergeCell ref="E95:F95"/>
+    <mergeCell ref="E96:F96"/>
+    <mergeCell ref="S96:Z96"/>
+    <mergeCell ref="S95:Y95"/>
+    <mergeCell ref="S100:Z100"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="S2:X2"/>
+    <mergeCell ref="S3:Y3"/>
+    <mergeCell ref="S7:Z7"/>
+    <mergeCell ref="S9:Z9"/>
+    <mergeCell ref="S10:Y10"/>
+    <mergeCell ref="S14:Y14"/>
+    <mergeCell ref="S16:AA16"/>
+    <mergeCell ref="S18:X18"/>
+    <mergeCell ref="S1:T1"/>
+    <mergeCell ref="S4:X4"/>
+    <mergeCell ref="S5:Y5"/>
+    <mergeCell ref="S6:Y6"/>
+    <mergeCell ref="S8:Y8"/>
+    <mergeCell ref="S11:Y11"/>
+    <mergeCell ref="S17:Z17"/>
+    <mergeCell ref="S21:Y21"/>
+    <mergeCell ref="S12:Z12"/>
+    <mergeCell ref="S13:Z13"/>
+    <mergeCell ref="S15:Z15"/>
+    <mergeCell ref="S29:Z29"/>
+    <mergeCell ref="S31:Z31"/>
+    <mergeCell ref="S22:Z22"/>
+    <mergeCell ref="S23:Y23"/>
+    <mergeCell ref="S25:Y25"/>
+    <mergeCell ref="S26:Y26"/>
+    <mergeCell ref="S19:Y19"/>
+    <mergeCell ref="S20:Z20"/>
+    <mergeCell ref="S24:Y24"/>
+    <mergeCell ref="S27:Z27"/>
+    <mergeCell ref="S28:Z28"/>
+    <mergeCell ref="S30:Y30"/>
+    <mergeCell ref="S32:Y32"/>
+    <mergeCell ref="S33:Z33"/>
+    <mergeCell ref="S34:Y34"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="S35:Y35"/>
+    <mergeCell ref="S36:X36"/>
+    <mergeCell ref="S37:Z37"/>
+    <mergeCell ref="S38:AA38"/>
+    <mergeCell ref="S39:X39"/>
+    <mergeCell ref="S40:X40"/>
+    <mergeCell ref="S41:Z41"/>
+    <mergeCell ref="S42:AA42"/>
+    <mergeCell ref="S43:Z43"/>
+    <mergeCell ref="S44:Y44"/>
+    <mergeCell ref="S45:Z45"/>
+    <mergeCell ref="S46:X46"/>
+    <mergeCell ref="S47:Y47"/>
+    <mergeCell ref="S53:Z53"/>
+    <mergeCell ref="S48:Z48"/>
+    <mergeCell ref="S49:AA49"/>
+    <mergeCell ref="S50:Y50"/>
+    <mergeCell ref="S51:Z51"/>
+    <mergeCell ref="S52:Z52"/>
+    <mergeCell ref="S73:Y73"/>
+    <mergeCell ref="S75:Y75"/>
+    <mergeCell ref="S76:Y76"/>
+    <mergeCell ref="S77:Z77"/>
+    <mergeCell ref="S78:Z78"/>
+    <mergeCell ref="S79:X79"/>
+    <mergeCell ref="S54:Y54"/>
+    <mergeCell ref="S55:Z55"/>
+    <mergeCell ref="S56:X56"/>
+    <mergeCell ref="S57:X57"/>
+    <mergeCell ref="S64:Y64"/>
+    <mergeCell ref="S69:Z69"/>
+    <mergeCell ref="S58:X58"/>
+    <mergeCell ref="S59:Y59"/>
+    <mergeCell ref="S60:X60"/>
+    <mergeCell ref="S61:Y61"/>
+    <mergeCell ref="S62:Z62"/>
+    <mergeCell ref="S63:Y63"/>
+    <mergeCell ref="S65:Z65"/>
+    <mergeCell ref="S66:Z66"/>
+    <mergeCell ref="S67:Z67"/>
     <mergeCell ref="S90:Y90"/>
     <mergeCell ref="S87:X87"/>
     <mergeCell ref="S88:Y88"/>
@@ -49529,98 +49621,6 @@
     <mergeCell ref="S82:AA82"/>
     <mergeCell ref="S84:X84"/>
     <mergeCell ref="S85:X85"/>
-    <mergeCell ref="S73:Y73"/>
-    <mergeCell ref="S75:Y75"/>
-    <mergeCell ref="S76:Y76"/>
-    <mergeCell ref="S77:Z77"/>
-    <mergeCell ref="S78:Z78"/>
-    <mergeCell ref="S79:X79"/>
-    <mergeCell ref="S54:Y54"/>
-    <mergeCell ref="S55:Z55"/>
-    <mergeCell ref="S56:X56"/>
-    <mergeCell ref="S57:X57"/>
-    <mergeCell ref="S64:Y64"/>
-    <mergeCell ref="S69:Z69"/>
-    <mergeCell ref="S58:X58"/>
-    <mergeCell ref="S59:Y59"/>
-    <mergeCell ref="S60:X60"/>
-    <mergeCell ref="S61:Y61"/>
-    <mergeCell ref="S62:Z62"/>
-    <mergeCell ref="S63:Y63"/>
-    <mergeCell ref="S65:Z65"/>
-    <mergeCell ref="S66:Z66"/>
-    <mergeCell ref="S67:Z67"/>
-    <mergeCell ref="S40:X40"/>
-    <mergeCell ref="S41:Z41"/>
-    <mergeCell ref="S42:AA42"/>
-    <mergeCell ref="S43:Z43"/>
-    <mergeCell ref="S44:Y44"/>
-    <mergeCell ref="S45:Z45"/>
-    <mergeCell ref="S46:X46"/>
-    <mergeCell ref="S47:Y47"/>
-    <mergeCell ref="S53:Z53"/>
-    <mergeCell ref="S48:Z48"/>
-    <mergeCell ref="S49:AA49"/>
-    <mergeCell ref="S50:Y50"/>
-    <mergeCell ref="S51:Z51"/>
-    <mergeCell ref="S52:Z52"/>
-    <mergeCell ref="S32:Y32"/>
-    <mergeCell ref="S33:Z33"/>
-    <mergeCell ref="S34:Y34"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="S35:Y35"/>
-    <mergeCell ref="S36:X36"/>
-    <mergeCell ref="S37:Z37"/>
-    <mergeCell ref="S38:AA38"/>
-    <mergeCell ref="S39:X39"/>
-    <mergeCell ref="S29:Z29"/>
-    <mergeCell ref="S31:Z31"/>
-    <mergeCell ref="S22:Z22"/>
-    <mergeCell ref="S23:Y23"/>
-    <mergeCell ref="S25:Y25"/>
-    <mergeCell ref="S26:Y26"/>
-    <mergeCell ref="S19:Y19"/>
-    <mergeCell ref="S20:Z20"/>
-    <mergeCell ref="S24:Y24"/>
-    <mergeCell ref="S27:Z27"/>
-    <mergeCell ref="S28:Z28"/>
-    <mergeCell ref="S30:Y30"/>
-    <mergeCell ref="S1:T1"/>
-    <mergeCell ref="S4:X4"/>
-    <mergeCell ref="S5:Y5"/>
-    <mergeCell ref="S6:Y6"/>
-    <mergeCell ref="S8:Y8"/>
-    <mergeCell ref="S11:Y11"/>
-    <mergeCell ref="S17:Z17"/>
-    <mergeCell ref="S21:Y21"/>
-    <mergeCell ref="S12:Z12"/>
-    <mergeCell ref="S13:Z13"/>
-    <mergeCell ref="S15:Z15"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="S2:X2"/>
-    <mergeCell ref="S3:Y3"/>
-    <mergeCell ref="S7:Z7"/>
-    <mergeCell ref="S9:Z9"/>
-    <mergeCell ref="S10:Y10"/>
-    <mergeCell ref="S14:Y14"/>
-    <mergeCell ref="S16:AA16"/>
-    <mergeCell ref="S18:X18"/>
-    <mergeCell ref="B116:S116"/>
-    <mergeCell ref="B124:S124"/>
-    <mergeCell ref="B130:S130"/>
-    <mergeCell ref="B139:O139"/>
-    <mergeCell ref="E91:F91"/>
-    <mergeCell ref="S91:Z91"/>
-    <mergeCell ref="E92:F92"/>
-    <mergeCell ref="S92:Z92"/>
-    <mergeCell ref="E93:F93"/>
-    <mergeCell ref="S93:Z93"/>
-    <mergeCell ref="S94:AA94"/>
-    <mergeCell ref="E95:F95"/>
-    <mergeCell ref="E96:F96"/>
-    <mergeCell ref="S96:Z96"/>
-    <mergeCell ref="S95:Y95"/>
-    <mergeCell ref="S100:Z100"/>
   </mergeCells>
   <phoneticPr fontId="21" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
"Encounter" changed to "Experience"
</commit_message>
<xml_diff>
--- a/CDT AITP Go Live (2).xlsx
+++ b/CDT AITP Go Live (2).xlsx
@@ -2911,15 +2911,30 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2928,23 +2943,8 @@
     <xf numFmtId="0" fontId="18" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3245,10 +3245,10 @@
       <c r="R1" s="85" t="s">
         <v>607</v>
       </c>
-      <c r="S1" s="112" t="s">
+      <c r="S1" s="108" t="s">
         <v>210</v>
       </c>
-      <c r="T1" s="112"/>
+      <c r="T1" s="108"/>
       <c r="U1" s="43"/>
       <c r="V1" s="43"/>
       <c r="W1" s="43"/>
@@ -3291,10 +3291,10 @@
       <c r="G2" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="H2" s="102" t="s">
+      <c r="H2" s="104" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="102"/>
+      <c r="I2" s="104"/>
       <c r="J2" s="43" t="s">
         <v>213</v>
       </c>
@@ -3322,14 +3322,14 @@
       <c r="R2" s="86" t="s">
         <v>609</v>
       </c>
-      <c r="S2" s="102" t="s">
+      <c r="S2" s="104" t="s">
         <v>184</v>
       </c>
-      <c r="T2" s="102"/>
-      <c r="U2" s="102"/>
-      <c r="V2" s="102"/>
-      <c r="W2" s="102"/>
-      <c r="X2" s="102"/>
+      <c r="T2" s="104"/>
+      <c r="U2" s="104"/>
+      <c r="V2" s="104"/>
+      <c r="W2" s="104"/>
+      <c r="X2" s="104"/>
       <c r="Y2" s="43"/>
       <c r="Z2" s="43"/>
       <c r="AA2" s="43"/>
@@ -3401,15 +3401,15 @@
       <c r="R3" s="86" t="s">
         <v>611</v>
       </c>
-      <c r="S3" s="102" t="s">
+      <c r="S3" s="104" t="s">
         <v>194</v>
       </c>
-      <c r="T3" s="102"/>
-      <c r="U3" s="102"/>
-      <c r="V3" s="102"/>
-      <c r="W3" s="102"/>
-      <c r="X3" s="102"/>
-      <c r="Y3" s="102"/>
+      <c r="T3" s="104"/>
+      <c r="U3" s="104"/>
+      <c r="V3" s="104"/>
+      <c r="W3" s="104"/>
+      <c r="X3" s="104"/>
+      <c r="Y3" s="104"/>
       <c r="Z3" s="43"/>
       <c r="AA3" s="43"/>
       <c r="AB3" s="43"/>
@@ -3480,14 +3480,14 @@
       <c r="R4" s="86" t="s">
         <v>612</v>
       </c>
-      <c r="S4" s="102" t="s">
+      <c r="S4" s="104" t="s">
         <v>214</v>
       </c>
-      <c r="T4" s="102"/>
-      <c r="U4" s="102"/>
-      <c r="V4" s="102"/>
-      <c r="W4" s="102"/>
-      <c r="X4" s="102"/>
+      <c r="T4" s="104"/>
+      <c r="U4" s="104"/>
+      <c r="V4" s="104"/>
+      <c r="W4" s="104"/>
+      <c r="X4" s="104"/>
       <c r="Y4" s="43"/>
       <c r="Z4" s="43"/>
       <c r="AA4" s="43"/>
@@ -3561,15 +3561,15 @@
       <c r="R5" s="86" t="s">
         <v>614</v>
       </c>
-      <c r="S5" s="102" t="s">
+      <c r="S5" s="104" t="s">
         <v>219</v>
       </c>
-      <c r="T5" s="102"/>
-      <c r="U5" s="102"/>
-      <c r="V5" s="102"/>
-      <c r="W5" s="102"/>
-      <c r="X5" s="102"/>
-      <c r="Y5" s="102"/>
+      <c r="T5" s="104"/>
+      <c r="U5" s="104"/>
+      <c r="V5" s="104"/>
+      <c r="W5" s="104"/>
+      <c r="X5" s="104"/>
+      <c r="Y5" s="104"/>
       <c r="Z5" s="43"/>
       <c r="AA5" s="43"/>
       <c r="AB5" s="43"/>
@@ -3638,15 +3638,15 @@
       <c r="R6" s="86" t="s">
         <v>616</v>
       </c>
-      <c r="S6" s="110" t="s">
+      <c r="S6" s="106" t="s">
         <v>72</v>
       </c>
-      <c r="T6" s="110"/>
-      <c r="U6" s="110"/>
-      <c r="V6" s="110"/>
-      <c r="W6" s="110"/>
-      <c r="X6" s="110"/>
-      <c r="Y6" s="110"/>
+      <c r="T6" s="106"/>
+      <c r="U6" s="106"/>
+      <c r="V6" s="106"/>
+      <c r="W6" s="106"/>
+      <c r="X6" s="106"/>
+      <c r="Y6" s="106"/>
       <c r="Z6" s="50"/>
       <c r="AA6" s="50"/>
       <c r="AB6" s="50"/>
@@ -3715,16 +3715,16 @@
       <c r="R7" s="86" t="s">
         <v>618</v>
       </c>
-      <c r="S7" s="110" t="s">
+      <c r="S7" s="106" t="s">
         <v>77</v>
       </c>
-      <c r="T7" s="110"/>
-      <c r="U7" s="110"/>
-      <c r="V7" s="110"/>
-      <c r="W7" s="110"/>
-      <c r="X7" s="110"/>
-      <c r="Y7" s="110"/>
-      <c r="Z7" s="110"/>
+      <c r="T7" s="106"/>
+      <c r="U7" s="106"/>
+      <c r="V7" s="106"/>
+      <c r="W7" s="106"/>
+      <c r="X7" s="106"/>
+      <c r="Y7" s="106"/>
+      <c r="Z7" s="106"/>
       <c r="AA7" s="50"/>
       <c r="AB7" s="50"/>
       <c r="AC7" s="50"/>
@@ -3794,15 +3794,15 @@
       <c r="R8" s="86" t="s">
         <v>619</v>
       </c>
-      <c r="S8" s="110" t="s">
+      <c r="S8" s="106" t="s">
         <v>190</v>
       </c>
-      <c r="T8" s="110"/>
-      <c r="U8" s="110"/>
-      <c r="V8" s="110"/>
-      <c r="W8" s="110"/>
-      <c r="X8" s="110"/>
-      <c r="Y8" s="110"/>
+      <c r="T8" s="106"/>
+      <c r="U8" s="106"/>
+      <c r="V8" s="106"/>
+      <c r="W8" s="106"/>
+      <c r="X8" s="106"/>
+      <c r="Y8" s="106"/>
       <c r="Z8" s="50"/>
       <c r="AA8" s="50"/>
       <c r="AB8" s="50"/>
@@ -3875,16 +3875,16 @@
       <c r="R9" s="86" t="s">
         <v>615</v>
       </c>
-      <c r="S9" s="108" t="s">
+      <c r="S9" s="107" t="s">
         <v>224</v>
       </c>
-      <c r="T9" s="108"/>
-      <c r="U9" s="108"/>
-      <c r="V9" s="108"/>
-      <c r="W9" s="108"/>
-      <c r="X9" s="108"/>
-      <c r="Y9" s="108"/>
-      <c r="Z9" s="108"/>
+      <c r="T9" s="107"/>
+      <c r="U9" s="107"/>
+      <c r="V9" s="107"/>
+      <c r="W9" s="107"/>
+      <c r="X9" s="107"/>
+      <c r="Y9" s="107"/>
+      <c r="Z9" s="107"/>
       <c r="AA9" s="54"/>
       <c r="AB9" s="54"/>
       <c r="AC9" s="54"/>
@@ -3956,15 +3956,15 @@
       <c r="R10" s="86" t="s">
         <v>610</v>
       </c>
-      <c r="S10" s="104" t="s">
+      <c r="S10" s="105" t="s">
         <v>221</v>
       </c>
-      <c r="T10" s="104"/>
-      <c r="U10" s="104"/>
-      <c r="V10" s="104"/>
-      <c r="W10" s="104"/>
-      <c r="X10" s="104"/>
-      <c r="Y10" s="104"/>
+      <c r="T10" s="105"/>
+      <c r="U10" s="105"/>
+      <c r="V10" s="105"/>
+      <c r="W10" s="105"/>
+      <c r="X10" s="105"/>
+      <c r="Y10" s="105"/>
       <c r="Z10" s="65"/>
       <c r="AA10" s="65"/>
       <c r="AB10" s="65"/>
@@ -4037,15 +4037,15 @@
       <c r="R11" s="86" t="s">
         <v>623</v>
       </c>
-      <c r="S11" s="104" t="s">
+      <c r="S11" s="105" t="s">
         <v>222</v>
       </c>
-      <c r="T11" s="104"/>
-      <c r="U11" s="104"/>
-      <c r="V11" s="104"/>
-      <c r="W11" s="104"/>
-      <c r="X11" s="104"/>
-      <c r="Y11" s="104"/>
+      <c r="T11" s="105"/>
+      <c r="U11" s="105"/>
+      <c r="V11" s="105"/>
+      <c r="W11" s="105"/>
+      <c r="X11" s="105"/>
+      <c r="Y11" s="105"/>
       <c r="Z11" s="65"/>
       <c r="AA11" s="65"/>
       <c r="AB11" s="65"/>
@@ -4118,16 +4118,16 @@
       <c r="R12" s="86" t="s">
         <v>612</v>
       </c>
-      <c r="S12" s="104" t="s">
+      <c r="S12" s="105" t="s">
         <v>226</v>
       </c>
-      <c r="T12" s="104"/>
-      <c r="U12" s="104"/>
-      <c r="V12" s="104"/>
-      <c r="W12" s="104"/>
-      <c r="X12" s="104"/>
-      <c r="Y12" s="104"/>
-      <c r="Z12" s="104"/>
+      <c r="T12" s="105"/>
+      <c r="U12" s="105"/>
+      <c r="V12" s="105"/>
+      <c r="W12" s="105"/>
+      <c r="X12" s="105"/>
+      <c r="Y12" s="105"/>
+      <c r="Z12" s="105"/>
       <c r="AA12" s="65"/>
       <c r="AB12" s="65"/>
       <c r="AC12" s="65"/>
@@ -4197,16 +4197,16 @@
       <c r="R13" s="86" t="s">
         <v>625</v>
       </c>
-      <c r="S13" s="102" t="s">
+      <c r="S13" s="104" t="s">
         <v>231</v>
       </c>
-      <c r="T13" s="102"/>
-      <c r="U13" s="102"/>
-      <c r="V13" s="102"/>
-      <c r="W13" s="102"/>
-      <c r="X13" s="102"/>
-      <c r="Y13" s="102"/>
-      <c r="Z13" s="102"/>
+      <c r="T13" s="104"/>
+      <c r="U13" s="104"/>
+      <c r="V13" s="104"/>
+      <c r="W13" s="104"/>
+      <c r="X13" s="104"/>
+      <c r="Y13" s="104"/>
+      <c r="Z13" s="104"/>
       <c r="AA13" s="43"/>
       <c r="AB13" s="43"/>
       <c r="AC13" s="43"/>
@@ -4274,15 +4274,15 @@
       <c r="R14" s="86" t="s">
         <v>627</v>
       </c>
-      <c r="S14" s="102" t="s">
+      <c r="S14" s="104" t="s">
         <v>148</v>
       </c>
-      <c r="T14" s="102"/>
-      <c r="U14" s="102"/>
-      <c r="V14" s="102"/>
-      <c r="W14" s="102"/>
-      <c r="X14" s="102"/>
-      <c r="Y14" s="102"/>
+      <c r="T14" s="104"/>
+      <c r="U14" s="104"/>
+      <c r="V14" s="104"/>
+      <c r="W14" s="104"/>
+      <c r="X14" s="104"/>
+      <c r="Y14" s="104"/>
       <c r="Z14" s="43"/>
       <c r="AA14" s="43"/>
       <c r="AB14" s="43"/>
@@ -4355,16 +4355,16 @@
       <c r="R15" s="86" t="s">
         <v>629</v>
       </c>
-      <c r="S15" s="105" t="s">
+      <c r="S15" s="103" t="s">
         <v>86</v>
       </c>
-      <c r="T15" s="105"/>
-      <c r="U15" s="105"/>
-      <c r="V15" s="105"/>
-      <c r="W15" s="105"/>
-      <c r="X15" s="105"/>
-      <c r="Y15" s="105"/>
-      <c r="Z15" s="105"/>
+      <c r="T15" s="103"/>
+      <c r="U15" s="103"/>
+      <c r="V15" s="103"/>
+      <c r="W15" s="103"/>
+      <c r="X15" s="103"/>
+      <c r="Y15" s="103"/>
+      <c r="Z15" s="103"/>
       <c r="AA15" s="51"/>
       <c r="AB15" s="43"/>
       <c r="AC15" s="43"/>
@@ -4436,17 +4436,17 @@
       <c r="R16" s="86" t="s">
         <v>630</v>
       </c>
-      <c r="S16" s="105" t="s">
+      <c r="S16" s="103" t="s">
         <v>234</v>
       </c>
-      <c r="T16" s="105"/>
-      <c r="U16" s="105"/>
-      <c r="V16" s="105"/>
-      <c r="W16" s="105"/>
-      <c r="X16" s="105"/>
-      <c r="Y16" s="105"/>
-      <c r="Z16" s="105"/>
-      <c r="AA16" s="105"/>
+      <c r="T16" s="103"/>
+      <c r="U16" s="103"/>
+      <c r="V16" s="103"/>
+      <c r="W16" s="103"/>
+      <c r="X16" s="103"/>
+      <c r="Y16" s="103"/>
+      <c r="Z16" s="103"/>
+      <c r="AA16" s="103"/>
       <c r="AB16" s="43"/>
       <c r="AC16" s="43"/>
       <c r="AD16" s="43"/>
@@ -4517,16 +4517,16 @@
       <c r="R17" s="86" t="s">
         <v>632</v>
       </c>
-      <c r="S17" s="105" t="s">
+      <c r="S17" s="103" t="s">
         <v>84</v>
       </c>
-      <c r="T17" s="105"/>
-      <c r="U17" s="105"/>
-      <c r="V17" s="105"/>
-      <c r="W17" s="105"/>
-      <c r="X17" s="105"/>
-      <c r="Y17" s="105"/>
-      <c r="Z17" s="105"/>
+      <c r="T17" s="103"/>
+      <c r="U17" s="103"/>
+      <c r="V17" s="103"/>
+      <c r="W17" s="103"/>
+      <c r="X17" s="103"/>
+      <c r="Y17" s="103"/>
+      <c r="Z17" s="103"/>
       <c r="AA17" s="51"/>
       <c r="AB17" s="43"/>
       <c r="AC17" s="43"/>
@@ -4598,14 +4598,14 @@
       <c r="R18" s="86" t="s">
         <v>632</v>
       </c>
-      <c r="S18" s="105" t="s">
+      <c r="S18" s="103" t="s">
         <v>82</v>
       </c>
-      <c r="T18" s="105"/>
-      <c r="U18" s="105"/>
-      <c r="V18" s="105"/>
-      <c r="W18" s="105"/>
-      <c r="X18" s="105"/>
+      <c r="T18" s="103"/>
+      <c r="U18" s="103"/>
+      <c r="V18" s="103"/>
+      <c r="W18" s="103"/>
+      <c r="X18" s="103"/>
       <c r="Y18" s="51"/>
       <c r="Z18" s="51"/>
       <c r="AA18" s="51"/>
@@ -4679,15 +4679,15 @@
       <c r="R19" s="86" t="s">
         <v>634</v>
       </c>
-      <c r="S19" s="105" t="s">
+      <c r="S19" s="103" t="s">
         <v>96</v>
       </c>
-      <c r="T19" s="105"/>
-      <c r="U19" s="105"/>
-      <c r="V19" s="105"/>
-      <c r="W19" s="105"/>
-      <c r="X19" s="105"/>
-      <c r="Y19" s="105"/>
+      <c r="T19" s="103"/>
+      <c r="U19" s="103"/>
+      <c r="V19" s="103"/>
+      <c r="W19" s="103"/>
+      <c r="X19" s="103"/>
+      <c r="Y19" s="103"/>
       <c r="Z19" s="51"/>
       <c r="AA19" s="51"/>
       <c r="AB19" s="43"/>
@@ -4760,16 +4760,16 @@
       <c r="R20" s="86" t="s">
         <v>636</v>
       </c>
-      <c r="S20" s="105" t="s">
+      <c r="S20" s="103" t="s">
         <v>235</v>
       </c>
-      <c r="T20" s="105"/>
-      <c r="U20" s="105"/>
-      <c r="V20" s="105"/>
-      <c r="W20" s="105"/>
-      <c r="X20" s="105"/>
-      <c r="Y20" s="105"/>
-      <c r="Z20" s="105"/>
+      <c r="T20" s="103"/>
+      <c r="U20" s="103"/>
+      <c r="V20" s="103"/>
+      <c r="W20" s="103"/>
+      <c r="X20" s="103"/>
+      <c r="Y20" s="103"/>
+      <c r="Z20" s="103"/>
       <c r="AA20" s="51"/>
       <c r="AB20" s="43"/>
       <c r="AC20" s="43"/>
@@ -4841,15 +4841,15 @@
       <c r="R21" s="86" t="s">
         <v>610</v>
       </c>
-      <c r="S21" s="105" t="s">
+      <c r="S21" s="103" t="s">
         <v>236</v>
       </c>
-      <c r="T21" s="105"/>
-      <c r="U21" s="105"/>
-      <c r="V21" s="105"/>
-      <c r="W21" s="105"/>
-      <c r="X21" s="105"/>
-      <c r="Y21" s="105"/>
+      <c r="T21" s="103"/>
+      <c r="U21" s="103"/>
+      <c r="V21" s="103"/>
+      <c r="W21" s="103"/>
+      <c r="X21" s="103"/>
+      <c r="Y21" s="103"/>
       <c r="Z21" s="51"/>
       <c r="AA21" s="51"/>
       <c r="AB21" s="43"/>
@@ -4922,16 +4922,16 @@
       <c r="R22" s="86" t="s">
         <v>639</v>
       </c>
-      <c r="S22" s="105" t="s">
+      <c r="S22" s="103" t="s">
         <v>238</v>
       </c>
-      <c r="T22" s="105"/>
-      <c r="U22" s="105"/>
-      <c r="V22" s="105"/>
-      <c r="W22" s="105"/>
-      <c r="X22" s="105"/>
-      <c r="Y22" s="105"/>
-      <c r="Z22" s="105"/>
+      <c r="T22" s="103"/>
+      <c r="U22" s="103"/>
+      <c r="V22" s="103"/>
+      <c r="W22" s="103"/>
+      <c r="X22" s="103"/>
+      <c r="Y22" s="103"/>
+      <c r="Z22" s="103"/>
       <c r="AA22" s="51"/>
       <c r="AB22" s="43"/>
       <c r="AC22" s="43"/>
@@ -5003,15 +5003,15 @@
       <c r="R23" s="86" t="s">
         <v>632</v>
       </c>
-      <c r="S23" s="105" t="s">
+      <c r="S23" s="103" t="s">
         <v>98</v>
       </c>
-      <c r="T23" s="105"/>
-      <c r="U23" s="105"/>
-      <c r="V23" s="105"/>
-      <c r="W23" s="105"/>
-      <c r="X23" s="105"/>
-      <c r="Y23" s="105"/>
+      <c r="T23" s="103"/>
+      <c r="U23" s="103"/>
+      <c r="V23" s="103"/>
+      <c r="W23" s="103"/>
+      <c r="X23" s="103"/>
+      <c r="Y23" s="103"/>
       <c r="Z23" s="51"/>
       <c r="AA23" s="51"/>
       <c r="AB23" s="43"/>
@@ -5084,15 +5084,15 @@
       <c r="R24" s="86" t="s">
         <v>641</v>
       </c>
-      <c r="S24" s="110" t="s">
+      <c r="S24" s="106" t="s">
         <v>240</v>
       </c>
-      <c r="T24" s="110"/>
-      <c r="U24" s="110"/>
-      <c r="V24" s="110"/>
-      <c r="W24" s="110"/>
-      <c r="X24" s="110"/>
-      <c r="Y24" s="110"/>
+      <c r="T24" s="106"/>
+      <c r="U24" s="106"/>
+      <c r="V24" s="106"/>
+      <c r="W24" s="106"/>
+      <c r="X24" s="106"/>
+      <c r="Y24" s="106"/>
       <c r="Z24" s="50"/>
       <c r="AA24" s="50"/>
       <c r="AB24" s="43"/>
@@ -5165,15 +5165,15 @@
       <c r="R25" s="86" t="s">
         <v>668</v>
       </c>
-      <c r="S25" s="110" t="s">
+      <c r="S25" s="106" t="s">
         <v>112</v>
       </c>
-      <c r="T25" s="110"/>
-      <c r="U25" s="110"/>
-      <c r="V25" s="110"/>
-      <c r="W25" s="110"/>
-      <c r="X25" s="110"/>
-      <c r="Y25" s="110"/>
+      <c r="T25" s="106"/>
+      <c r="U25" s="106"/>
+      <c r="V25" s="106"/>
+      <c r="W25" s="106"/>
+      <c r="X25" s="106"/>
+      <c r="Y25" s="106"/>
       <c r="Z25" s="50"/>
       <c r="AA25" s="50"/>
       <c r="AB25" s="43"/>
@@ -5246,15 +5246,15 @@
       <c r="R26" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S26" s="110" t="s">
+      <c r="S26" s="106" t="s">
         <v>108</v>
       </c>
-      <c r="T26" s="110"/>
-      <c r="U26" s="110"/>
-      <c r="V26" s="110"/>
-      <c r="W26" s="110"/>
-      <c r="X26" s="110"/>
-      <c r="Y26" s="110"/>
+      <c r="T26" s="106"/>
+      <c r="U26" s="106"/>
+      <c r="V26" s="106"/>
+      <c r="W26" s="106"/>
+      <c r="X26" s="106"/>
+      <c r="Y26" s="106"/>
       <c r="Z26" s="50"/>
       <c r="AA26" s="50"/>
       <c r="AB26" s="43"/>
@@ -5327,16 +5327,16 @@
       <c r="R27" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S27" s="110" t="s">
+      <c r="S27" s="106" t="s">
         <v>243</v>
       </c>
-      <c r="T27" s="110"/>
-      <c r="U27" s="110"/>
-      <c r="V27" s="110"/>
-      <c r="W27" s="110"/>
-      <c r="X27" s="110"/>
-      <c r="Y27" s="110"/>
-      <c r="Z27" s="110"/>
+      <c r="T27" s="106"/>
+      <c r="U27" s="106"/>
+      <c r="V27" s="106"/>
+      <c r="W27" s="106"/>
+      <c r="X27" s="106"/>
+      <c r="Y27" s="106"/>
+      <c r="Z27" s="106"/>
       <c r="AA27" s="50"/>
       <c r="AB27" s="43"/>
       <c r="AC27" s="43"/>
@@ -5408,16 +5408,16 @@
       <c r="R28" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S28" s="110" t="s">
+      <c r="S28" s="106" t="s">
         <v>245</v>
       </c>
-      <c r="T28" s="110"/>
-      <c r="U28" s="110"/>
-      <c r="V28" s="110"/>
-      <c r="W28" s="110"/>
-      <c r="X28" s="110"/>
-      <c r="Y28" s="110"/>
-      <c r="Z28" s="110"/>
+      <c r="T28" s="106"/>
+      <c r="U28" s="106"/>
+      <c r="V28" s="106"/>
+      <c r="W28" s="106"/>
+      <c r="X28" s="106"/>
+      <c r="Y28" s="106"/>
+      <c r="Z28" s="106"/>
       <c r="AA28" s="50"/>
       <c r="AB28" s="43"/>
       <c r="AC28" s="43"/>
@@ -5489,16 +5489,16 @@
       <c r="R29" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S29" s="110" t="s">
+      <c r="S29" s="106" t="s">
         <v>247</v>
       </c>
-      <c r="T29" s="110"/>
-      <c r="U29" s="110"/>
-      <c r="V29" s="110"/>
-      <c r="W29" s="110"/>
-      <c r="X29" s="110"/>
-      <c r="Y29" s="110"/>
-      <c r="Z29" s="110"/>
+      <c r="T29" s="106"/>
+      <c r="U29" s="106"/>
+      <c r="V29" s="106"/>
+      <c r="W29" s="106"/>
+      <c r="X29" s="106"/>
+      <c r="Y29" s="106"/>
+      <c r="Z29" s="106"/>
       <c r="AA29" s="50"/>
       <c r="AB29" s="43"/>
       <c r="AC29" s="43"/>
@@ -5570,15 +5570,15 @@
       <c r="R30" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S30" s="110" t="s">
+      <c r="S30" s="106" t="s">
         <v>249</v>
       </c>
-      <c r="T30" s="110"/>
-      <c r="U30" s="110"/>
-      <c r="V30" s="110"/>
-      <c r="W30" s="110"/>
-      <c r="X30" s="110"/>
-      <c r="Y30" s="110"/>
+      <c r="T30" s="106"/>
+      <c r="U30" s="106"/>
+      <c r="V30" s="106"/>
+      <c r="W30" s="106"/>
+      <c r="X30" s="106"/>
+      <c r="Y30" s="106"/>
       <c r="Z30" s="50"/>
       <c r="AA30" s="50"/>
       <c r="AB30" s="43"/>
@@ -5651,16 +5651,16 @@
       <c r="R31" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S31" s="111" t="s">
+      <c r="S31" s="109" t="s">
         <v>115</v>
       </c>
-      <c r="T31" s="111"/>
-      <c r="U31" s="111"/>
-      <c r="V31" s="111"/>
-      <c r="W31" s="111"/>
-      <c r="X31" s="111"/>
-      <c r="Y31" s="111"/>
-      <c r="Z31" s="111"/>
+      <c r="T31" s="109"/>
+      <c r="U31" s="109"/>
+      <c r="V31" s="109"/>
+      <c r="W31" s="109"/>
+      <c r="X31" s="109"/>
+      <c r="Y31" s="109"/>
+      <c r="Z31" s="109"/>
       <c r="AA31" s="52"/>
       <c r="AB31" s="43"/>
       <c r="AC31" s="43"/>
@@ -5728,15 +5728,15 @@
         <v>706</v>
       </c>
       <c r="R32" s="86"/>
-      <c r="S32" s="109" t="s">
+      <c r="S32" s="110" t="s">
         <v>252</v>
       </c>
-      <c r="T32" s="109"/>
-      <c r="U32" s="109"/>
-      <c r="V32" s="109"/>
-      <c r="W32" s="109"/>
-      <c r="X32" s="109"/>
-      <c r="Y32" s="109"/>
+      <c r="T32" s="110"/>
+      <c r="U32" s="110"/>
+      <c r="V32" s="110"/>
+      <c r="W32" s="110"/>
+      <c r="X32" s="110"/>
+      <c r="Y32" s="110"/>
       <c r="Z32" s="53"/>
       <c r="AA32" s="53"/>
       <c r="AB32" s="43"/>
@@ -5774,10 +5774,10 @@
       <c r="G33" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="H33" s="109" t="s">
+      <c r="H33" s="110" t="s">
         <v>7</v>
       </c>
-      <c r="I33" s="109"/>
+      <c r="I33" s="110"/>
       <c r="J33" s="53" t="s">
         <v>213</v>
       </c>
@@ -5805,16 +5805,16 @@
       <c r="R33" s="86" t="s">
         <v>708</v>
       </c>
-      <c r="S33" s="109" t="s">
+      <c r="S33" s="110" t="s">
         <v>253</v>
       </c>
-      <c r="T33" s="109"/>
-      <c r="U33" s="109"/>
-      <c r="V33" s="109"/>
-      <c r="W33" s="109"/>
-      <c r="X33" s="109"/>
-      <c r="Y33" s="109"/>
-      <c r="Z33" s="109"/>
+      <c r="T33" s="110"/>
+      <c r="U33" s="110"/>
+      <c r="V33" s="110"/>
+      <c r="W33" s="110"/>
+      <c r="X33" s="110"/>
+      <c r="Y33" s="110"/>
+      <c r="Z33" s="110"/>
       <c r="AA33" s="53"/>
       <c r="AB33" s="43"/>
       <c r="AC33" s="43"/>
@@ -5884,15 +5884,15 @@
       <c r="R34" s="86" t="s">
         <v>708</v>
       </c>
-      <c r="S34" s="109" t="s">
+      <c r="S34" s="110" t="s">
         <v>254</v>
       </c>
-      <c r="T34" s="109"/>
-      <c r="U34" s="109"/>
-      <c r="V34" s="109"/>
-      <c r="W34" s="109"/>
-      <c r="X34" s="109"/>
-      <c r="Y34" s="109"/>
+      <c r="T34" s="110"/>
+      <c r="U34" s="110"/>
+      <c r="V34" s="110"/>
+      <c r="W34" s="110"/>
+      <c r="X34" s="110"/>
+      <c r="Y34" s="110"/>
       <c r="Z34" s="53"/>
       <c r="AA34" s="53"/>
       <c r="AB34" s="43"/>
@@ -5961,15 +5961,15 @@
         <v>709</v>
       </c>
       <c r="R35" s="86"/>
-      <c r="S35" s="109" t="s">
+      <c r="S35" s="110" t="s">
         <v>255</v>
       </c>
-      <c r="T35" s="109"/>
-      <c r="U35" s="109"/>
-      <c r="V35" s="109"/>
-      <c r="W35" s="109"/>
-      <c r="X35" s="109"/>
-      <c r="Y35" s="109"/>
+      <c r="T35" s="110"/>
+      <c r="U35" s="110"/>
+      <c r="V35" s="110"/>
+      <c r="W35" s="110"/>
+      <c r="X35" s="110"/>
+      <c r="Y35" s="110"/>
       <c r="Z35" s="53"/>
       <c r="AA35" s="53"/>
       <c r="AB35" s="43"/>
@@ -6040,14 +6040,14 @@
       <c r="R36" s="86" t="s">
         <v>712</v>
       </c>
-      <c r="S36" s="109" t="s">
+      <c r="S36" s="110" t="s">
         <v>256</v>
       </c>
-      <c r="T36" s="109"/>
-      <c r="U36" s="109"/>
-      <c r="V36" s="109"/>
-      <c r="W36" s="109"/>
-      <c r="X36" s="109"/>
+      <c r="T36" s="110"/>
+      <c r="U36" s="110"/>
+      <c r="V36" s="110"/>
+      <c r="W36" s="110"/>
+      <c r="X36" s="110"/>
       <c r="Y36" s="53"/>
       <c r="Z36" s="53"/>
       <c r="AA36" s="53"/>
@@ -6117,16 +6117,16 @@
         <v>689</v>
       </c>
       <c r="R37" s="86"/>
-      <c r="S37" s="109" t="s">
+      <c r="S37" s="110" t="s">
         <v>257</v>
       </c>
-      <c r="T37" s="109"/>
-      <c r="U37" s="109"/>
-      <c r="V37" s="109"/>
-      <c r="W37" s="109"/>
-      <c r="X37" s="109"/>
-      <c r="Y37" s="109"/>
-      <c r="Z37" s="109"/>
+      <c r="T37" s="110"/>
+      <c r="U37" s="110"/>
+      <c r="V37" s="110"/>
+      <c r="W37" s="110"/>
+      <c r="X37" s="110"/>
+      <c r="Y37" s="110"/>
+      <c r="Z37" s="110"/>
       <c r="AA37" s="53"/>
       <c r="AB37" s="43"/>
       <c r="AC37" s="43"/>
@@ -6194,17 +6194,17 @@
         <v>689</v>
       </c>
       <c r="R38" s="86"/>
-      <c r="S38" s="109" t="s">
+      <c r="S38" s="110" t="s">
         <v>258</v>
       </c>
-      <c r="T38" s="109"/>
-      <c r="U38" s="109"/>
-      <c r="V38" s="109"/>
-      <c r="W38" s="109"/>
-      <c r="X38" s="109"/>
-      <c r="Y38" s="109"/>
-      <c r="Z38" s="109"/>
-      <c r="AA38" s="109"/>
+      <c r="T38" s="110"/>
+      <c r="U38" s="110"/>
+      <c r="V38" s="110"/>
+      <c r="W38" s="110"/>
+      <c r="X38" s="110"/>
+      <c r="Y38" s="110"/>
+      <c r="Z38" s="110"/>
+      <c r="AA38" s="110"/>
       <c r="AB38" s="43"/>
       <c r="AC38" s="43"/>
       <c r="AD38" s="43"/>
@@ -6275,14 +6275,14 @@
       <c r="R39" s="86" t="s">
         <v>715</v>
       </c>
-      <c r="S39" s="108" t="s">
+      <c r="S39" s="107" t="s">
         <v>166</v>
       </c>
-      <c r="T39" s="108"/>
-      <c r="U39" s="108"/>
-      <c r="V39" s="108"/>
-      <c r="W39" s="108"/>
-      <c r="X39" s="108"/>
+      <c r="T39" s="107"/>
+      <c r="U39" s="107"/>
+      <c r="V39" s="107"/>
+      <c r="W39" s="107"/>
+      <c r="X39" s="107"/>
       <c r="Y39" s="54"/>
       <c r="Z39" s="54"/>
       <c r="AA39" s="54"/>
@@ -6356,14 +6356,14 @@
       <c r="R40" s="86" t="s">
         <v>624</v>
       </c>
-      <c r="S40" s="108" t="s">
+      <c r="S40" s="107" t="s">
         <v>263</v>
       </c>
-      <c r="T40" s="108"/>
-      <c r="U40" s="108"/>
-      <c r="V40" s="108"/>
-      <c r="W40" s="108"/>
-      <c r="X40" s="108"/>
+      <c r="T40" s="107"/>
+      <c r="U40" s="107"/>
+      <c r="V40" s="107"/>
+      <c r="W40" s="107"/>
+      <c r="X40" s="107"/>
       <c r="Y40" s="54"/>
       <c r="Z40" s="54"/>
       <c r="AA40" s="54"/>
@@ -6435,16 +6435,16 @@
       <c r="R41" s="86" t="s">
         <v>719</v>
       </c>
-      <c r="S41" s="108" t="s">
+      <c r="S41" s="107" t="s">
         <v>264</v>
       </c>
-      <c r="T41" s="108"/>
-      <c r="U41" s="108"/>
-      <c r="V41" s="108"/>
-      <c r="W41" s="108"/>
-      <c r="X41" s="108"/>
-      <c r="Y41" s="108"/>
-      <c r="Z41" s="108"/>
+      <c r="T41" s="107"/>
+      <c r="U41" s="107"/>
+      <c r="V41" s="107"/>
+      <c r="W41" s="107"/>
+      <c r="X41" s="107"/>
+      <c r="Y41" s="107"/>
+      <c r="Z41" s="107"/>
       <c r="AA41" s="54"/>
       <c r="AB41" s="43"/>
       <c r="AC41" s="43"/>
@@ -6516,17 +6516,17 @@
       <c r="R42" s="86" t="s">
         <v>719</v>
       </c>
-      <c r="S42" s="108" t="s">
+      <c r="S42" s="107" t="s">
         <v>161</v>
       </c>
-      <c r="T42" s="108"/>
-      <c r="U42" s="108"/>
-      <c r="V42" s="108"/>
-      <c r="W42" s="108"/>
-      <c r="X42" s="108"/>
-      <c r="Y42" s="108"/>
-      <c r="Z42" s="108"/>
-      <c r="AA42" s="108"/>
+      <c r="T42" s="107"/>
+      <c r="U42" s="107"/>
+      <c r="V42" s="107"/>
+      <c r="W42" s="107"/>
+      <c r="X42" s="107"/>
+      <c r="Y42" s="107"/>
+      <c r="Z42" s="107"/>
+      <c r="AA42" s="107"/>
       <c r="AB42" s="43"/>
       <c r="AC42" s="43"/>
       <c r="AD42" s="43"/>
@@ -6597,16 +6597,16 @@
       <c r="R43" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S43" s="108" t="s">
+      <c r="S43" s="107" t="s">
         <v>265</v>
       </c>
-      <c r="T43" s="108"/>
-      <c r="U43" s="108"/>
-      <c r="V43" s="108"/>
-      <c r="W43" s="108"/>
-      <c r="X43" s="108"/>
-      <c r="Y43" s="108"/>
-      <c r="Z43" s="108"/>
+      <c r="T43" s="107"/>
+      <c r="U43" s="107"/>
+      <c r="V43" s="107"/>
+      <c r="W43" s="107"/>
+      <c r="X43" s="107"/>
+      <c r="Y43" s="107"/>
+      <c r="Z43" s="107"/>
       <c r="AA43" s="54"/>
       <c r="AB43" s="43"/>
       <c r="AC43" s="43"/>
@@ -6678,15 +6678,15 @@
       <c r="R44" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S44" s="108" t="s">
+      <c r="S44" s="107" t="s">
         <v>158</v>
       </c>
-      <c r="T44" s="108"/>
-      <c r="U44" s="108"/>
-      <c r="V44" s="108"/>
-      <c r="W44" s="108"/>
-      <c r="X44" s="108"/>
-      <c r="Y44" s="108"/>
+      <c r="T44" s="107"/>
+      <c r="U44" s="107"/>
+      <c r="V44" s="107"/>
+      <c r="W44" s="107"/>
+      <c r="X44" s="107"/>
+      <c r="Y44" s="107"/>
       <c r="Z44" s="54"/>
       <c r="AA44" s="54"/>
       <c r="AB44" s="43"/>
@@ -6757,16 +6757,16 @@
       <c r="R45" s="86" t="s">
         <v>719</v>
       </c>
-      <c r="S45" s="108" t="s">
+      <c r="S45" s="107" t="s">
         <v>266</v>
       </c>
-      <c r="T45" s="108"/>
-      <c r="U45" s="108"/>
-      <c r="V45" s="108"/>
-      <c r="W45" s="108"/>
-      <c r="X45" s="108"/>
-      <c r="Y45" s="108"/>
-      <c r="Z45" s="108"/>
+      <c r="T45" s="107"/>
+      <c r="U45" s="107"/>
+      <c r="V45" s="107"/>
+      <c r="W45" s="107"/>
+      <c r="X45" s="107"/>
+      <c r="Y45" s="107"/>
+      <c r="Z45" s="107"/>
       <c r="AA45" s="54"/>
       <c r="AB45" s="43"/>
       <c r="AC45" s="43"/>
@@ -6834,14 +6834,14 @@
       <c r="R46" s="86" t="s">
         <v>632</v>
       </c>
-      <c r="S46" s="108" t="s">
+      <c r="S46" s="107" t="s">
         <v>132</v>
       </c>
-      <c r="T46" s="108"/>
-      <c r="U46" s="108"/>
-      <c r="V46" s="108"/>
-      <c r="W46" s="108"/>
-      <c r="X46" s="108"/>
+      <c r="T46" s="107"/>
+      <c r="U46" s="107"/>
+      <c r="V46" s="107"/>
+      <c r="W46" s="107"/>
+      <c r="X46" s="107"/>
       <c r="Y46" s="54"/>
       <c r="Z46" s="54"/>
       <c r="AA46" s="54"/>
@@ -6915,15 +6915,15 @@
       <c r="R47" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S47" s="108" t="s">
+      <c r="S47" s="107" t="s">
         <v>136</v>
       </c>
-      <c r="T47" s="108"/>
-      <c r="U47" s="108"/>
-      <c r="V47" s="108"/>
-      <c r="W47" s="108"/>
-      <c r="X47" s="108"/>
-      <c r="Y47" s="108"/>
+      <c r="T47" s="107"/>
+      <c r="U47" s="107"/>
+      <c r="V47" s="107"/>
+      <c r="W47" s="107"/>
+      <c r="X47" s="107"/>
+      <c r="Y47" s="107"/>
       <c r="Z47" s="54"/>
       <c r="AA47" s="54"/>
       <c r="AB47" s="43"/>
@@ -6996,16 +6996,16 @@
       <c r="R48" s="86" t="s">
         <v>636</v>
       </c>
-      <c r="S48" s="108" t="s">
+      <c r="S48" s="107" t="s">
         <v>178</v>
       </c>
-      <c r="T48" s="108"/>
-      <c r="U48" s="108"/>
-      <c r="V48" s="108"/>
-      <c r="W48" s="108"/>
-      <c r="X48" s="108"/>
-      <c r="Y48" s="108"/>
-      <c r="Z48" s="108"/>
+      <c r="T48" s="107"/>
+      <c r="U48" s="107"/>
+      <c r="V48" s="107"/>
+      <c r="W48" s="107"/>
+      <c r="X48" s="107"/>
+      <c r="Y48" s="107"/>
+      <c r="Z48" s="107"/>
       <c r="AA48" s="54"/>
       <c r="AB48" s="43"/>
       <c r="AC48" s="43"/>
@@ -7077,17 +7077,17 @@
       <c r="R49" s="86" t="s">
         <v>730</v>
       </c>
-      <c r="S49" s="108" t="s">
+      <c r="S49" s="107" t="s">
         <v>268</v>
       </c>
-      <c r="T49" s="108"/>
-      <c r="U49" s="108"/>
-      <c r="V49" s="108"/>
-      <c r="W49" s="108"/>
-      <c r="X49" s="108"/>
-      <c r="Y49" s="108"/>
-      <c r="Z49" s="108"/>
-      <c r="AA49" s="108"/>
+      <c r="T49" s="107"/>
+      <c r="U49" s="107"/>
+      <c r="V49" s="107"/>
+      <c r="W49" s="107"/>
+      <c r="X49" s="107"/>
+      <c r="Y49" s="107"/>
+      <c r="Z49" s="107"/>
+      <c r="AA49" s="107"/>
       <c r="AB49" s="43"/>
       <c r="AC49" s="43"/>
       <c r="AD49" s="43"/>
@@ -7158,15 +7158,15 @@
       <c r="R50" s="86" t="s">
         <v>730</v>
       </c>
-      <c r="S50" s="108" t="s">
+      <c r="S50" s="107" t="s">
         <v>269</v>
       </c>
-      <c r="T50" s="108"/>
-      <c r="U50" s="108"/>
-      <c r="V50" s="108"/>
-      <c r="W50" s="108"/>
-      <c r="X50" s="108"/>
-      <c r="Y50" s="108"/>
+      <c r="T50" s="107"/>
+      <c r="U50" s="107"/>
+      <c r="V50" s="107"/>
+      <c r="W50" s="107"/>
+      <c r="X50" s="107"/>
+      <c r="Y50" s="107"/>
       <c r="Z50" s="54"/>
       <c r="AA50" s="54"/>
       <c r="AB50" s="43"/>
@@ -7235,16 +7235,16 @@
       <c r="R51" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S51" s="108" t="s">
+      <c r="S51" s="107" t="s">
         <v>170</v>
       </c>
-      <c r="T51" s="108"/>
-      <c r="U51" s="108"/>
-      <c r="V51" s="108"/>
-      <c r="W51" s="108"/>
-      <c r="X51" s="108"/>
-      <c r="Y51" s="108"/>
-      <c r="Z51" s="108"/>
+      <c r="T51" s="107"/>
+      <c r="U51" s="107"/>
+      <c r="V51" s="107"/>
+      <c r="W51" s="107"/>
+      <c r="X51" s="107"/>
+      <c r="Y51" s="107"/>
+      <c r="Z51" s="107"/>
       <c r="AA51" s="54"/>
       <c r="AB51" s="43"/>
       <c r="AC51" s="43"/>
@@ -7314,16 +7314,16 @@
       <c r="R52" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S52" s="102" t="s">
+      <c r="S52" s="104" t="s">
         <v>130</v>
       </c>
-      <c r="T52" s="102"/>
-      <c r="U52" s="102"/>
-      <c r="V52" s="102"/>
-      <c r="W52" s="102"/>
-      <c r="X52" s="102"/>
-      <c r="Y52" s="102"/>
-      <c r="Z52" s="102"/>
+      <c r="T52" s="104"/>
+      <c r="U52" s="104"/>
+      <c r="V52" s="104"/>
+      <c r="W52" s="104"/>
+      <c r="X52" s="104"/>
+      <c r="Y52" s="104"/>
+      <c r="Z52" s="104"/>
       <c r="AA52" s="43"/>
       <c r="AB52" s="43"/>
       <c r="AC52" s="43"/>
@@ -7393,16 +7393,16 @@
       <c r="R53" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S53" s="102" t="s">
+      <c r="S53" s="104" t="s">
         <v>272</v>
       </c>
-      <c r="T53" s="102"/>
-      <c r="U53" s="102"/>
-      <c r="V53" s="102"/>
-      <c r="W53" s="102"/>
-      <c r="X53" s="102"/>
-      <c r="Y53" s="102"/>
-      <c r="Z53" s="102"/>
+      <c r="T53" s="104"/>
+      <c r="U53" s="104"/>
+      <c r="V53" s="104"/>
+      <c r="W53" s="104"/>
+      <c r="X53" s="104"/>
+      <c r="Y53" s="104"/>
+      <c r="Z53" s="104"/>
       <c r="AA53" s="43"/>
       <c r="AB53" s="43"/>
       <c r="AC53" s="43"/>
@@ -7470,15 +7470,15 @@
       <c r="R54" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S54" s="102" t="s">
+      <c r="S54" s="104" t="s">
         <v>145</v>
       </c>
-      <c r="T54" s="102"/>
-      <c r="U54" s="102"/>
-      <c r="V54" s="102"/>
-      <c r="W54" s="102"/>
-      <c r="X54" s="102"/>
-      <c r="Y54" s="102"/>
+      <c r="T54" s="104"/>
+      <c r="U54" s="104"/>
+      <c r="V54" s="104"/>
+      <c r="W54" s="104"/>
+      <c r="X54" s="104"/>
+      <c r="Y54" s="104"/>
       <c r="Z54" s="43"/>
       <c r="AA54" s="43"/>
       <c r="AB54" s="43"/>
@@ -7551,16 +7551,16 @@
       <c r="R55" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S55" s="107" t="s">
+      <c r="S55" s="112" t="s">
         <v>260</v>
       </c>
-      <c r="T55" s="107"/>
-      <c r="U55" s="107"/>
-      <c r="V55" s="107"/>
-      <c r="W55" s="107"/>
-      <c r="X55" s="107"/>
-      <c r="Y55" s="107"/>
-      <c r="Z55" s="107"/>
+      <c r="T55" s="112"/>
+      <c r="U55" s="112"/>
+      <c r="V55" s="112"/>
+      <c r="W55" s="112"/>
+      <c r="X55" s="112"/>
+      <c r="Y55" s="112"/>
+      <c r="Z55" s="112"/>
       <c r="AA55" s="75"/>
       <c r="AB55" s="75"/>
       <c r="AC55" s="75"/>
@@ -7632,14 +7632,14 @@
       <c r="R56" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S56" s="107" t="s">
+      <c r="S56" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="T56" s="107"/>
-      <c r="U56" s="107"/>
-      <c r="V56" s="107"/>
-      <c r="W56" s="107"/>
-      <c r="X56" s="107"/>
+      <c r="T56" s="112"/>
+      <c r="U56" s="112"/>
+      <c r="V56" s="112"/>
+      <c r="W56" s="112"/>
+      <c r="X56" s="112"/>
       <c r="Y56" s="75"/>
       <c r="Z56" s="75"/>
       <c r="AA56" s="75"/>
@@ -7713,14 +7713,14 @@
       <c r="R57" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S57" s="107" t="s">
+      <c r="S57" s="112" t="s">
         <v>276</v>
       </c>
-      <c r="T57" s="107"/>
-      <c r="U57" s="107"/>
-      <c r="V57" s="107"/>
-      <c r="W57" s="107"/>
-      <c r="X57" s="107"/>
+      <c r="T57" s="112"/>
+      <c r="U57" s="112"/>
+      <c r="V57" s="112"/>
+      <c r="W57" s="112"/>
+      <c r="X57" s="112"/>
       <c r="Y57" s="75"/>
       <c r="Z57" s="75"/>
       <c r="AA57" s="75"/>
@@ -7794,14 +7794,14 @@
       <c r="R58" s="86" t="s">
         <v>753</v>
       </c>
-      <c r="S58" s="107" t="s">
+      <c r="S58" s="112" t="s">
         <v>278</v>
       </c>
-      <c r="T58" s="107"/>
-      <c r="U58" s="107"/>
-      <c r="V58" s="107"/>
-      <c r="W58" s="107"/>
-      <c r="X58" s="107"/>
+      <c r="T58" s="112"/>
+      <c r="U58" s="112"/>
+      <c r="V58" s="112"/>
+      <c r="W58" s="112"/>
+      <c r="X58" s="112"/>
       <c r="Y58" s="75"/>
       <c r="Z58" s="75"/>
       <c r="AA58" s="75"/>
@@ -7875,15 +7875,15 @@
       <c r="R59" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S59" s="107" t="s">
+      <c r="S59" s="112" t="s">
         <v>68</v>
       </c>
-      <c r="T59" s="107"/>
-      <c r="U59" s="107"/>
-      <c r="V59" s="107"/>
-      <c r="W59" s="107"/>
-      <c r="X59" s="107"/>
-      <c r="Y59" s="107"/>
+      <c r="T59" s="112"/>
+      <c r="U59" s="112"/>
+      <c r="V59" s="112"/>
+      <c r="W59" s="112"/>
+      <c r="X59" s="112"/>
+      <c r="Y59" s="112"/>
       <c r="Z59" s="75"/>
       <c r="AA59" s="75"/>
       <c r="AB59" s="75"/>
@@ -7956,14 +7956,14 @@
       <c r="R60" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S60" s="107" t="s">
+      <c r="S60" s="112" t="s">
         <v>126</v>
       </c>
-      <c r="T60" s="107"/>
-      <c r="U60" s="107"/>
-      <c r="V60" s="107"/>
-      <c r="W60" s="107"/>
-      <c r="X60" s="107"/>
+      <c r="T60" s="112"/>
+      <c r="U60" s="112"/>
+      <c r="V60" s="112"/>
+      <c r="W60" s="112"/>
+      <c r="X60" s="112"/>
       <c r="Y60" s="75"/>
       <c r="Z60" s="75"/>
       <c r="AA60" s="75"/>
@@ -8037,15 +8037,15 @@
       <c r="R61" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S61" s="102" t="s">
+      <c r="S61" s="104" t="s">
         <v>281</v>
       </c>
-      <c r="T61" s="102"/>
-      <c r="U61" s="102"/>
-      <c r="V61" s="102"/>
-      <c r="W61" s="102"/>
-      <c r="X61" s="102"/>
-      <c r="Y61" s="102"/>
+      <c r="T61" s="104"/>
+      <c r="U61" s="104"/>
+      <c r="V61" s="104"/>
+      <c r="W61" s="104"/>
+      <c r="X61" s="104"/>
+      <c r="Y61" s="104"/>
       <c r="Z61" s="43"/>
       <c r="AA61" s="43"/>
       <c r="AB61" s="43"/>
@@ -8118,16 +8118,16 @@
       <c r="R62" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S62" s="102" t="s">
+      <c r="S62" s="104" t="s">
         <v>282</v>
       </c>
-      <c r="T62" s="102"/>
-      <c r="U62" s="102"/>
-      <c r="V62" s="102"/>
-      <c r="W62" s="102"/>
-      <c r="X62" s="102"/>
-      <c r="Y62" s="102"/>
-      <c r="Z62" s="102"/>
+      <c r="T62" s="104"/>
+      <c r="U62" s="104"/>
+      <c r="V62" s="104"/>
+      <c r="W62" s="104"/>
+      <c r="X62" s="104"/>
+      <c r="Y62" s="104"/>
+      <c r="Z62" s="104"/>
       <c r="AA62" s="43"/>
       <c r="AB62" s="43"/>
       <c r="AC62" s="43"/>
@@ -8199,15 +8199,15 @@
       <c r="R63" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S63" s="102" t="s">
+      <c r="S63" s="104" t="s">
         <v>284</v>
       </c>
-      <c r="T63" s="102"/>
-      <c r="U63" s="102"/>
-      <c r="V63" s="102"/>
-      <c r="W63" s="102"/>
-      <c r="X63" s="102"/>
-      <c r="Y63" s="102"/>
+      <c r="T63" s="104"/>
+      <c r="U63" s="104"/>
+      <c r="V63" s="104"/>
+      <c r="W63" s="104"/>
+      <c r="X63" s="104"/>
+      <c r="Y63" s="104"/>
       <c r="Z63" s="43"/>
       <c r="AA63" s="43"/>
       <c r="AB63" s="43"/>
@@ -8280,15 +8280,15 @@
       <c r="R64" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S64" s="102" t="s">
+      <c r="S64" s="104" t="s">
         <v>70</v>
       </c>
-      <c r="T64" s="102"/>
-      <c r="U64" s="102"/>
-      <c r="V64" s="102"/>
-      <c r="W64" s="102"/>
-      <c r="X64" s="102"/>
-      <c r="Y64" s="102"/>
+      <c r="T64" s="104"/>
+      <c r="U64" s="104"/>
+      <c r="V64" s="104"/>
+      <c r="W64" s="104"/>
+      <c r="X64" s="104"/>
+      <c r="Y64" s="104"/>
       <c r="Z64" s="43"/>
       <c r="AA64" s="43"/>
       <c r="AB64" s="43"/>
@@ -8361,16 +8361,16 @@
       <c r="R65" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S65" s="102" t="s">
+      <c r="S65" s="104" t="s">
         <v>286</v>
       </c>
-      <c r="T65" s="102"/>
-      <c r="U65" s="102"/>
-      <c r="V65" s="102"/>
-      <c r="W65" s="102"/>
-      <c r="X65" s="102"/>
-      <c r="Y65" s="102"/>
-      <c r="Z65" s="102"/>
+      <c r="T65" s="104"/>
+      <c r="U65" s="104"/>
+      <c r="V65" s="104"/>
+      <c r="W65" s="104"/>
+      <c r="X65" s="104"/>
+      <c r="Y65" s="104"/>
+      <c r="Z65" s="104"/>
       <c r="AA65" s="43"/>
       <c r="AB65" s="43"/>
       <c r="AC65" s="43"/>
@@ -8442,16 +8442,16 @@
       <c r="R66" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S66" s="102" t="s">
+      <c r="S66" s="104" t="s">
         <v>287</v>
       </c>
-      <c r="T66" s="102"/>
-      <c r="U66" s="102"/>
-      <c r="V66" s="102"/>
-      <c r="W66" s="102"/>
-      <c r="X66" s="102"/>
-      <c r="Y66" s="102"/>
-      <c r="Z66" s="102"/>
+      <c r="T66" s="104"/>
+      <c r="U66" s="104"/>
+      <c r="V66" s="104"/>
+      <c r="W66" s="104"/>
+      <c r="X66" s="104"/>
+      <c r="Y66" s="104"/>
+      <c r="Z66" s="104"/>
       <c r="AA66" s="43"/>
       <c r="AB66" s="43"/>
       <c r="AC66" s="43"/>
@@ -8523,16 +8523,16 @@
       <c r="R67" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S67" s="103" t="s">
+      <c r="S67" s="113" t="s">
         <v>288</v>
       </c>
-      <c r="T67" s="103"/>
-      <c r="U67" s="103"/>
-      <c r="V67" s="103"/>
-      <c r="W67" s="103"/>
-      <c r="X67" s="103"/>
-      <c r="Y67" s="103"/>
-      <c r="Z67" s="103"/>
+      <c r="T67" s="113"/>
+      <c r="U67" s="113"/>
+      <c r="V67" s="113"/>
+      <c r="W67" s="113"/>
+      <c r="X67" s="113"/>
+      <c r="Y67" s="113"/>
+      <c r="Z67" s="113"/>
       <c r="AA67" s="82"/>
       <c r="AB67" s="82"/>
       <c r="AC67" s="82"/>
@@ -8604,16 +8604,16 @@
       <c r="R68" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S68" s="103" t="s">
+      <c r="S68" s="113" t="s">
         <v>288</v>
       </c>
-      <c r="T68" s="103"/>
-      <c r="U68" s="103"/>
-      <c r="V68" s="103"/>
-      <c r="W68" s="103"/>
-      <c r="X68" s="103"/>
-      <c r="Y68" s="103"/>
-      <c r="Z68" s="103"/>
+      <c r="T68" s="113"/>
+      <c r="U68" s="113"/>
+      <c r="V68" s="113"/>
+      <c r="W68" s="113"/>
+      <c r="X68" s="113"/>
+      <c r="Y68" s="113"/>
+      <c r="Z68" s="113"/>
       <c r="AA68" s="82"/>
       <c r="AB68" s="82"/>
       <c r="AC68" s="82"/>
@@ -8685,16 +8685,16 @@
       <c r="R69" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S69" s="103" t="s">
+      <c r="S69" s="113" t="s">
         <v>289</v>
       </c>
-      <c r="T69" s="103"/>
-      <c r="U69" s="103"/>
-      <c r="V69" s="103"/>
-      <c r="W69" s="103"/>
-      <c r="X69" s="103"/>
-      <c r="Y69" s="103"/>
-      <c r="Z69" s="103"/>
+      <c r="T69" s="113"/>
+      <c r="U69" s="113"/>
+      <c r="V69" s="113"/>
+      <c r="W69" s="113"/>
+      <c r="X69" s="113"/>
+      <c r="Y69" s="113"/>
+      <c r="Z69" s="113"/>
       <c r="AA69" s="82"/>
       <c r="AB69" s="82"/>
       <c r="AC69" s="82"/>
@@ -8758,15 +8758,15 @@
         <v>748</v>
       </c>
       <c r="R70" s="86"/>
-      <c r="S70" s="102" t="s">
+      <c r="S70" s="104" t="s">
         <v>75</v>
       </c>
-      <c r="T70" s="102"/>
-      <c r="U70" s="102"/>
-      <c r="V70" s="102"/>
-      <c r="W70" s="102"/>
-      <c r="X70" s="102"/>
-      <c r="Y70" s="102"/>
+      <c r="T70" s="104"/>
+      <c r="U70" s="104"/>
+      <c r="V70" s="104"/>
+      <c r="W70" s="104"/>
+      <c r="X70" s="104"/>
+      <c r="Y70" s="104"/>
       <c r="Z70" s="43"/>
       <c r="AA70" s="43"/>
       <c r="AB70" s="43"/>
@@ -8831,14 +8831,14 @@
         <v>748</v>
       </c>
       <c r="R71" s="86"/>
-      <c r="S71" s="102" t="s">
+      <c r="S71" s="104" t="s">
         <v>89</v>
       </c>
-      <c r="T71" s="102"/>
-      <c r="U71" s="102"/>
-      <c r="V71" s="102"/>
-      <c r="W71" s="102"/>
-      <c r="X71" s="102"/>
+      <c r="T71" s="104"/>
+      <c r="U71" s="104"/>
+      <c r="V71" s="104"/>
+      <c r="W71" s="104"/>
+      <c r="X71" s="104"/>
       <c r="Y71" s="43"/>
       <c r="Z71" s="43"/>
       <c r="AA71" s="43"/>
@@ -8908,16 +8908,16 @@
       <c r="R72" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S72" s="105" t="s">
+      <c r="S72" s="103" t="s">
         <v>91</v>
       </c>
-      <c r="T72" s="105"/>
-      <c r="U72" s="105"/>
-      <c r="V72" s="105"/>
-      <c r="W72" s="105"/>
-      <c r="X72" s="105"/>
-      <c r="Y72" s="105"/>
-      <c r="Z72" s="105"/>
+      <c r="T72" s="103"/>
+      <c r="U72" s="103"/>
+      <c r="V72" s="103"/>
+      <c r="W72" s="103"/>
+      <c r="X72" s="103"/>
+      <c r="Y72" s="103"/>
+      <c r="Z72" s="103"/>
       <c r="AA72" s="51"/>
       <c r="AB72" s="43"/>
       <c r="AC72" s="43"/>
@@ -8956,10 +8956,10 @@
       <c r="G73" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="H73" s="105" t="s">
+      <c r="H73" s="103" t="s">
         <v>10</v>
       </c>
-      <c r="I73" s="105"/>
+      <c r="I73" s="103"/>
       <c r="J73" s="51" t="s">
         <v>213</v>
       </c>
@@ -8987,15 +8987,15 @@
       <c r="R73" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S73" s="105" t="s">
+      <c r="S73" s="103" t="s">
         <v>293</v>
       </c>
-      <c r="T73" s="105"/>
-      <c r="U73" s="105"/>
-      <c r="V73" s="105"/>
-      <c r="W73" s="105"/>
-      <c r="X73" s="105"/>
-      <c r="Y73" s="105"/>
+      <c r="T73" s="103"/>
+      <c r="U73" s="103"/>
+      <c r="V73" s="103"/>
+      <c r="W73" s="103"/>
+      <c r="X73" s="103"/>
+      <c r="Y73" s="103"/>
       <c r="Z73" s="51"/>
       <c r="AA73" s="51"/>
       <c r="AB73" s="43"/>
@@ -9035,10 +9035,10 @@
       <c r="G74" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="H74" s="105" t="s">
+      <c r="H74" s="103" t="s">
         <v>10</v>
       </c>
-      <c r="I74" s="105"/>
+      <c r="I74" s="103"/>
       <c r="J74" s="51" t="s">
         <v>213</v>
       </c>
@@ -9066,16 +9066,16 @@
       <c r="R74" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S74" s="105" t="s">
+      <c r="S74" s="103" t="s">
         <v>106</v>
       </c>
-      <c r="T74" s="105"/>
-      <c r="U74" s="105"/>
-      <c r="V74" s="105"/>
-      <c r="W74" s="105"/>
-      <c r="X74" s="105"/>
-      <c r="Y74" s="105"/>
-      <c r="Z74" s="105"/>
+      <c r="T74" s="103"/>
+      <c r="U74" s="103"/>
+      <c r="V74" s="103"/>
+      <c r="W74" s="103"/>
+      <c r="X74" s="103"/>
+      <c r="Y74" s="103"/>
+      <c r="Z74" s="103"/>
       <c r="AA74" s="51"/>
       <c r="AB74" s="43"/>
       <c r="AC74" s="43"/>
@@ -9145,15 +9145,15 @@
       <c r="R75" s="86" t="s">
         <v>740</v>
       </c>
-      <c r="S75" s="105" t="s">
+      <c r="S75" s="103" t="s">
         <v>152</v>
       </c>
-      <c r="T75" s="105"/>
-      <c r="U75" s="105"/>
-      <c r="V75" s="105"/>
-      <c r="W75" s="105"/>
-      <c r="X75" s="105"/>
-      <c r="Y75" s="105"/>
+      <c r="T75" s="103"/>
+      <c r="U75" s="103"/>
+      <c r="V75" s="103"/>
+      <c r="W75" s="103"/>
+      <c r="X75" s="103"/>
+      <c r="Y75" s="103"/>
       <c r="Z75" s="51"/>
       <c r="AA75" s="51"/>
       <c r="AB75" s="43"/>
@@ -9193,10 +9193,10 @@
       <c r="G76" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="H76" s="105" t="s">
+      <c r="H76" s="103" t="s">
         <v>10</v>
       </c>
-      <c r="I76" s="105"/>
+      <c r="I76" s="103"/>
       <c r="J76" s="51" t="s">
         <v>213</v>
       </c>
@@ -9224,15 +9224,15 @@
       <c r="R76" s="86" t="s">
         <v>674</v>
       </c>
-      <c r="S76" s="105" t="s">
+      <c r="S76" s="103" t="s">
         <v>296</v>
       </c>
-      <c r="T76" s="105"/>
-      <c r="U76" s="105"/>
-      <c r="V76" s="105"/>
-      <c r="W76" s="105"/>
-      <c r="X76" s="105"/>
-      <c r="Y76" s="105"/>
+      <c r="T76" s="103"/>
+      <c r="U76" s="103"/>
+      <c r="V76" s="103"/>
+      <c r="W76" s="103"/>
+      <c r="X76" s="103"/>
+      <c r="Y76" s="103"/>
       <c r="Z76" s="51"/>
       <c r="AA76" s="51"/>
       <c r="AB76" s="43"/>
@@ -9305,16 +9305,16 @@
       <c r="R77" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S77" s="105" t="s">
+      <c r="S77" s="103" t="s">
         <v>297</v>
       </c>
-      <c r="T77" s="105"/>
-      <c r="U77" s="105"/>
-      <c r="V77" s="105"/>
-      <c r="W77" s="105"/>
-      <c r="X77" s="105"/>
-      <c r="Y77" s="105"/>
-      <c r="Z77" s="105"/>
+      <c r="T77" s="103"/>
+      <c r="U77" s="103"/>
+      <c r="V77" s="103"/>
+      <c r="W77" s="103"/>
+      <c r="X77" s="103"/>
+      <c r="Y77" s="103"/>
+      <c r="Z77" s="103"/>
       <c r="AA77" s="51"/>
       <c r="AB77" s="43"/>
       <c r="AC77" s="43"/>
@@ -9386,16 +9386,16 @@
       <c r="R78" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S78" s="106" t="s">
+      <c r="S78" s="111" t="s">
         <v>295</v>
       </c>
-      <c r="T78" s="106"/>
-      <c r="U78" s="106"/>
-      <c r="V78" s="106"/>
-      <c r="W78" s="106"/>
-      <c r="X78" s="106"/>
-      <c r="Y78" s="106"/>
-      <c r="Z78" s="106"/>
+      <c r="T78" s="111"/>
+      <c r="U78" s="111"/>
+      <c r="V78" s="111"/>
+      <c r="W78" s="111"/>
+      <c r="X78" s="111"/>
+      <c r="Y78" s="111"/>
+      <c r="Z78" s="111"/>
       <c r="AA78" s="44"/>
       <c r="AB78" s="43"/>
       <c r="AC78" s="43"/>
@@ -9467,14 +9467,14 @@
       <c r="R79" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S79" s="102" t="s">
+      <c r="S79" s="104" t="s">
         <v>301</v>
       </c>
-      <c r="T79" s="102"/>
-      <c r="U79" s="102"/>
-      <c r="V79" s="102"/>
-      <c r="W79" s="102"/>
-      <c r="X79" s="102"/>
+      <c r="T79" s="104"/>
+      <c r="U79" s="104"/>
+      <c r="V79" s="104"/>
+      <c r="W79" s="104"/>
+      <c r="X79" s="104"/>
       <c r="Y79" s="43"/>
       <c r="Z79" s="43"/>
       <c r="AA79" s="43"/>
@@ -9548,15 +9548,15 @@
       <c r="R80" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S80" s="102" t="s">
+      <c r="S80" s="104" t="s">
         <v>303</v>
       </c>
-      <c r="T80" s="102"/>
-      <c r="U80" s="102"/>
-      <c r="V80" s="102"/>
-      <c r="W80" s="102"/>
-      <c r="X80" s="102"/>
-      <c r="Y80" s="102"/>
+      <c r="T80" s="104"/>
+      <c r="U80" s="104"/>
+      <c r="V80" s="104"/>
+      <c r="W80" s="104"/>
+      <c r="X80" s="104"/>
+      <c r="Y80" s="104"/>
       <c r="Z80" s="43"/>
       <c r="AA80" s="43"/>
       <c r="AB80" s="43"/>
@@ -9629,13 +9629,13 @@
       <c r="R81" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S81" s="102" t="s">
+      <c r="S81" s="104" t="s">
         <v>305</v>
       </c>
-      <c r="T81" s="102"/>
-      <c r="U81" s="102"/>
-      <c r="V81" s="102"/>
-      <c r="W81" s="102"/>
+      <c r="T81" s="104"/>
+      <c r="U81" s="104"/>
+      <c r="V81" s="104"/>
+      <c r="W81" s="104"/>
       <c r="X81" s="43"/>
       <c r="Y81" s="43"/>
       <c r="Z81" s="43"/>
@@ -9710,17 +9710,17 @@
       <c r="R82" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S82" s="102" t="s">
+      <c r="S82" s="104" t="s">
         <v>307</v>
       </c>
-      <c r="T82" s="102"/>
-      <c r="U82" s="102"/>
-      <c r="V82" s="102"/>
-      <c r="W82" s="102"/>
-      <c r="X82" s="102"/>
-      <c r="Y82" s="102"/>
-      <c r="Z82" s="102"/>
-      <c r="AA82" s="102"/>
+      <c r="T82" s="104"/>
+      <c r="U82" s="104"/>
+      <c r="V82" s="104"/>
+      <c r="W82" s="104"/>
+      <c r="X82" s="104"/>
+      <c r="Y82" s="104"/>
+      <c r="Z82" s="104"/>
+      <c r="AA82" s="104"/>
       <c r="AB82" s="43"/>
       <c r="AC82" s="43"/>
       <c r="AD82" s="43"/>
@@ -9791,15 +9791,15 @@
       <c r="R83" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S83" s="102" t="s">
+      <c r="S83" s="104" t="s">
         <v>309</v>
       </c>
-      <c r="T83" s="102"/>
-      <c r="U83" s="102"/>
-      <c r="V83" s="102"/>
-      <c r="W83" s="102"/>
-      <c r="X83" s="102"/>
-      <c r="Y83" s="102"/>
+      <c r="T83" s="104"/>
+      <c r="U83" s="104"/>
+      <c r="V83" s="104"/>
+      <c r="W83" s="104"/>
+      <c r="X83" s="104"/>
+      <c r="Y83" s="104"/>
       <c r="Z83" s="43"/>
       <c r="AA83" s="43"/>
       <c r="AB83" s="43"/>
@@ -9872,14 +9872,14 @@
       <c r="R84" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S84" s="102" t="s">
+      <c r="S84" s="104" t="s">
         <v>311</v>
       </c>
-      <c r="T84" s="102"/>
-      <c r="U84" s="102"/>
-      <c r="V84" s="102"/>
-      <c r="W84" s="102"/>
-      <c r="X84" s="102"/>
+      <c r="T84" s="104"/>
+      <c r="U84" s="104"/>
+      <c r="V84" s="104"/>
+      <c r="W84" s="104"/>
+      <c r="X84" s="104"/>
       <c r="Y84" s="43"/>
       <c r="Z84" s="43"/>
       <c r="AA84" s="43"/>
@@ -9953,14 +9953,14 @@
       <c r="R85" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S85" s="102" t="s">
+      <c r="S85" s="104" t="s">
         <v>313</v>
       </c>
-      <c r="T85" s="102"/>
-      <c r="U85" s="102"/>
-      <c r="V85" s="102"/>
-      <c r="W85" s="102"/>
-      <c r="X85" s="102"/>
+      <c r="T85" s="104"/>
+      <c r="U85" s="104"/>
+      <c r="V85" s="104"/>
+      <c r="W85" s="104"/>
+      <c r="X85" s="104"/>
       <c r="Y85" s="43"/>
       <c r="Z85" s="43"/>
       <c r="AA85" s="43"/>
@@ -10034,14 +10034,14 @@
       <c r="R86" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S86" s="102" t="s">
+      <c r="S86" s="104" t="s">
         <v>315</v>
       </c>
-      <c r="T86" s="102"/>
-      <c r="U86" s="102"/>
-      <c r="V86" s="102"/>
-      <c r="W86" s="102"/>
-      <c r="X86" s="102"/>
+      <c r="T86" s="104"/>
+      <c r="U86" s="104"/>
+      <c r="V86" s="104"/>
+      <c r="W86" s="104"/>
+      <c r="X86" s="104"/>
       <c r="Y86" s="43"/>
       <c r="Z86" s="43"/>
       <c r="AA86" s="43"/>
@@ -10115,14 +10115,14 @@
       <c r="R87" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S87" s="102" t="s">
+      <c r="S87" s="104" t="s">
         <v>317</v>
       </c>
-      <c r="T87" s="102"/>
-      <c r="U87" s="102"/>
-      <c r="V87" s="102"/>
-      <c r="W87" s="102"/>
-      <c r="X87" s="102"/>
+      <c r="T87" s="104"/>
+      <c r="U87" s="104"/>
+      <c r="V87" s="104"/>
+      <c r="W87" s="104"/>
+      <c r="X87" s="104"/>
       <c r="Y87" s="43"/>
       <c r="Z87" s="43"/>
       <c r="AA87" s="43"/>
@@ -10194,15 +10194,15 @@
       <c r="R88" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S88" s="102" t="s">
+      <c r="S88" s="104" t="s">
         <v>321</v>
       </c>
-      <c r="T88" s="102"/>
-      <c r="U88" s="102"/>
-      <c r="V88" s="102"/>
-      <c r="W88" s="102"/>
-      <c r="X88" s="102"/>
-      <c r="Y88" s="102"/>
+      <c r="T88" s="104"/>
+      <c r="U88" s="104"/>
+      <c r="V88" s="104"/>
+      <c r="W88" s="104"/>
+      <c r="X88" s="104"/>
+      <c r="Y88" s="104"/>
       <c r="Z88" s="43"/>
       <c r="AA88" s="43"/>
       <c r="AB88" s="43"/>
@@ -10240,10 +10240,10 @@
       <c r="G89" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="H89" s="102" t="s">
+      <c r="H89" s="104" t="s">
         <v>17</v>
       </c>
-      <c r="I89" s="102"/>
+      <c r="I89" s="104"/>
       <c r="J89" s="43" t="s">
         <v>213</v>
       </c>
@@ -10271,15 +10271,15 @@
       <c r="R89" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S89" s="102" t="s">
+      <c r="S89" s="104" t="s">
         <v>323</v>
       </c>
-      <c r="T89" s="102"/>
-      <c r="U89" s="102"/>
-      <c r="V89" s="102"/>
-      <c r="W89" s="102"/>
-      <c r="X89" s="102"/>
-      <c r="Y89" s="102"/>
+      <c r="T89" s="104"/>
+      <c r="U89" s="104"/>
+      <c r="V89" s="104"/>
+      <c r="W89" s="104"/>
+      <c r="X89" s="104"/>
+      <c r="Y89" s="104"/>
       <c r="Z89" s="43"/>
       <c r="AA89" s="43"/>
       <c r="AB89" s="43"/>
@@ -10350,15 +10350,15 @@
       <c r="R90" s="86" t="s">
         <v>686</v>
       </c>
-      <c r="S90" s="102" t="s">
+      <c r="S90" s="104" t="s">
         <v>325</v>
       </c>
-      <c r="T90" s="102"/>
-      <c r="U90" s="102"/>
-      <c r="V90" s="102"/>
-      <c r="W90" s="102"/>
-      <c r="X90" s="102"/>
-      <c r="Y90" s="102"/>
+      <c r="T90" s="104"/>
+      <c r="U90" s="104"/>
+      <c r="V90" s="104"/>
+      <c r="W90" s="104"/>
+      <c r="X90" s="104"/>
+      <c r="Y90" s="104"/>
       <c r="Z90" s="43"/>
       <c r="AA90" s="43"/>
       <c r="AB90" s="43"/>
@@ -10389,10 +10389,10 @@
       <c r="D91" s="51" t="s">
         <v>326</v>
       </c>
-      <c r="E91" s="105" t="s">
+      <c r="E91" s="103" t="s">
         <v>327</v>
       </c>
-      <c r="F91" s="105"/>
+      <c r="F91" s="103"/>
       <c r="G91" s="51" t="s">
         <v>604</v>
       </c>
@@ -10429,16 +10429,16 @@
       <c r="R91" s="86" t="s">
         <v>689</v>
       </c>
-      <c r="S91" s="105" t="s">
+      <c r="S91" s="103" t="s">
         <v>80</v>
       </c>
-      <c r="T91" s="105"/>
-      <c r="U91" s="105"/>
-      <c r="V91" s="105"/>
-      <c r="W91" s="105"/>
-      <c r="X91" s="105"/>
-      <c r="Y91" s="105"/>
-      <c r="Z91" s="105"/>
+      <c r="T91" s="103"/>
+      <c r="U91" s="103"/>
+      <c r="V91" s="103"/>
+      <c r="W91" s="103"/>
+      <c r="X91" s="103"/>
+      <c r="Y91" s="103"/>
+      <c r="Z91" s="103"/>
       <c r="AA91" s="51"/>
       <c r="AB91" s="51"/>
       <c r="AC91" s="51"/>
@@ -10468,10 +10468,10 @@
       <c r="D92" s="51" t="s">
         <v>326</v>
       </c>
-      <c r="E92" s="105" t="s">
+      <c r="E92" s="103" t="s">
         <v>327</v>
       </c>
-      <c r="F92" s="105"/>
+      <c r="F92" s="103"/>
       <c r="G92" s="51" t="s">
         <v>604</v>
       </c>
@@ -10508,16 +10508,16 @@
       <c r="R92" s="86" t="s">
         <v>610</v>
       </c>
-      <c r="S92" s="105" t="s">
+      <c r="S92" s="103" t="s">
         <v>328</v>
       </c>
-      <c r="T92" s="105"/>
-      <c r="U92" s="105"/>
-      <c r="V92" s="105"/>
-      <c r="W92" s="105"/>
-      <c r="X92" s="105"/>
-      <c r="Y92" s="105"/>
-      <c r="Z92" s="105"/>
+      <c r="T92" s="103"/>
+      <c r="U92" s="103"/>
+      <c r="V92" s="103"/>
+      <c r="W92" s="103"/>
+      <c r="X92" s="103"/>
+      <c r="Y92" s="103"/>
+      <c r="Z92" s="103"/>
       <c r="AA92" s="51"/>
       <c r="AB92" s="51"/>
       <c r="AC92" s="51"/>
@@ -10547,10 +10547,10 @@
       <c r="D93" s="51" t="s">
         <v>326</v>
       </c>
-      <c r="E93" s="105" t="s">
+      <c r="E93" s="103" t="s">
         <v>327</v>
       </c>
-      <c r="F93" s="105"/>
+      <c r="F93" s="103"/>
       <c r="G93" s="51" t="s">
         <v>604</v>
       </c>
@@ -10583,16 +10583,16 @@
         <v>628</v>
       </c>
       <c r="R93" s="86"/>
-      <c r="S93" s="105" t="s">
+      <c r="S93" s="103" t="s">
         <v>329</v>
       </c>
-      <c r="T93" s="105"/>
-      <c r="U93" s="105"/>
-      <c r="V93" s="105"/>
-      <c r="W93" s="105"/>
-      <c r="X93" s="105"/>
-      <c r="Y93" s="105"/>
-      <c r="Z93" s="105"/>
+      <c r="T93" s="103"/>
+      <c r="U93" s="103"/>
+      <c r="V93" s="103"/>
+      <c r="W93" s="103"/>
+      <c r="X93" s="103"/>
+      <c r="Y93" s="103"/>
+      <c r="Z93" s="103"/>
       <c r="AA93" s="51"/>
       <c r="AB93" s="51"/>
       <c r="AC93" s="51"/>
@@ -10664,17 +10664,17 @@
       <c r="R94" s="86" t="s">
         <v>662</v>
       </c>
-      <c r="S94" s="102" t="s">
+      <c r="S94" s="104" t="s">
         <v>174</v>
       </c>
-      <c r="T94" s="102"/>
-      <c r="U94" s="102"/>
-      <c r="V94" s="102"/>
-      <c r="W94" s="102"/>
-      <c r="X94" s="102"/>
-      <c r="Y94" s="102"/>
-      <c r="Z94" s="102"/>
-      <c r="AA94" s="102"/>
+      <c r="T94" s="104"/>
+      <c r="U94" s="104"/>
+      <c r="V94" s="104"/>
+      <c r="W94" s="104"/>
+      <c r="X94" s="104"/>
+      <c r="Y94" s="104"/>
+      <c r="Z94" s="104"/>
+      <c r="AA94" s="104"/>
       <c r="AB94" s="43"/>
       <c r="AC94" s="43"/>
       <c r="AD94" s="43"/>
@@ -10703,10 +10703,10 @@
       <c r="D95" s="43" t="s">
         <v>601</v>
       </c>
-      <c r="E95" s="102" t="s">
+      <c r="E95" s="104" t="s">
         <v>331</v>
       </c>
-      <c r="F95" s="102"/>
+      <c r="F95" s="104"/>
       <c r="G95" s="43" t="s">
         <v>7</v>
       </c>
@@ -10739,15 +10739,15 @@
         <v>682</v>
       </c>
       <c r="R95" s="86"/>
-      <c r="S95" s="102" t="s">
+      <c r="S95" s="104" t="s">
         <v>150</v>
       </c>
-      <c r="T95" s="102"/>
-      <c r="U95" s="102"/>
-      <c r="V95" s="102"/>
-      <c r="W95" s="102"/>
-      <c r="X95" s="102"/>
-      <c r="Y95" s="102"/>
+      <c r="T95" s="104"/>
+      <c r="U95" s="104"/>
+      <c r="V95" s="104"/>
+      <c r="W95" s="104"/>
+      <c r="X95" s="104"/>
+      <c r="Y95" s="104"/>
       <c r="Z95" s="43"/>
       <c r="AA95" s="43"/>
       <c r="AB95" s="43"/>
@@ -10778,10 +10778,10 @@
       <c r="D96" s="43" t="s">
         <v>601</v>
       </c>
-      <c r="E96" s="102" t="s">
+      <c r="E96" s="104" t="s">
         <v>331</v>
       </c>
-      <c r="F96" s="102"/>
+      <c r="F96" s="104"/>
       <c r="G96" s="43" t="s">
         <v>7</v>
       </c>
@@ -10812,16 +10812,16 @@
         <v>680</v>
       </c>
       <c r="R96" s="86"/>
-      <c r="S96" s="102" t="s">
+      <c r="S96" s="104" t="s">
         <v>172</v>
       </c>
-      <c r="T96" s="102"/>
-      <c r="U96" s="102"/>
-      <c r="V96" s="102"/>
-      <c r="W96" s="102"/>
-      <c r="X96" s="102"/>
-      <c r="Y96" s="102"/>
-      <c r="Z96" s="102"/>
+      <c r="T96" s="104"/>
+      <c r="U96" s="104"/>
+      <c r="V96" s="104"/>
+      <c r="W96" s="104"/>
+      <c r="X96" s="104"/>
+      <c r="Y96" s="104"/>
+      <c r="Z96" s="104"/>
       <c r="AA96" s="43"/>
       <c r="AB96" s="43"/>
       <c r="AC96" s="43"/>
@@ -10851,10 +10851,10 @@
       <c r="D97" s="43" t="s">
         <v>601</v>
       </c>
-      <c r="E97" s="102" t="s">
+      <c r="E97" s="104" t="s">
         <v>331</v>
       </c>
-      <c r="F97" s="102"/>
+      <c r="F97" s="104"/>
       <c r="G97" s="43" t="s">
         <v>7</v>
       </c>
@@ -10889,16 +10889,16 @@
         <v>679</v>
       </c>
       <c r="R97" s="86"/>
-      <c r="S97" s="102" t="s">
+      <c r="S97" s="104" t="s">
         <v>182</v>
       </c>
-      <c r="T97" s="102"/>
-      <c r="U97" s="102"/>
-      <c r="V97" s="102"/>
-      <c r="W97" s="102"/>
-      <c r="X97" s="102"/>
-      <c r="Y97" s="102"/>
-      <c r="Z97" s="102"/>
+      <c r="T97" s="104"/>
+      <c r="U97" s="104"/>
+      <c r="V97" s="104"/>
+      <c r="W97" s="104"/>
+      <c r="X97" s="104"/>
+      <c r="Y97" s="104"/>
+      <c r="Z97" s="104"/>
       <c r="AA97" s="43"/>
       <c r="AB97" s="43"/>
       <c r="AC97" s="43"/>
@@ -10966,16 +10966,16 @@
       <c r="R98" s="86" t="s">
         <v>612</v>
       </c>
-      <c r="S98" s="104" t="s">
+      <c r="S98" s="105" t="s">
         <v>102</v>
       </c>
-      <c r="T98" s="104"/>
-      <c r="U98" s="104"/>
-      <c r="V98" s="104"/>
-      <c r="W98" s="104"/>
-      <c r="X98" s="104"/>
-      <c r="Y98" s="104"/>
-      <c r="Z98" s="104"/>
+      <c r="T98" s="105"/>
+      <c r="U98" s="105"/>
+      <c r="V98" s="105"/>
+      <c r="W98" s="105"/>
+      <c r="X98" s="105"/>
+      <c r="Y98" s="105"/>
+      <c r="Z98" s="105"/>
       <c r="AA98" s="65"/>
       <c r="AB98" s="65"/>
       <c r="AC98" s="65"/>
@@ -11043,16 +11043,16 @@
       <c r="R99" s="86" t="s">
         <v>674</v>
       </c>
-      <c r="S99" s="104" t="s">
+      <c r="S99" s="105" t="s">
         <v>259</v>
       </c>
-      <c r="T99" s="104"/>
-      <c r="U99" s="104"/>
-      <c r="V99" s="104"/>
-      <c r="W99" s="104"/>
-      <c r="X99" s="104"/>
-      <c r="Y99" s="104"/>
-      <c r="Z99" s="104"/>
+      <c r="T99" s="105"/>
+      <c r="U99" s="105"/>
+      <c r="V99" s="105"/>
+      <c r="W99" s="105"/>
+      <c r="X99" s="105"/>
+      <c r="Y99" s="105"/>
+      <c r="Z99" s="105"/>
       <c r="AA99" s="65"/>
       <c r="AB99" s="65"/>
       <c r="AC99" s="65"/>
@@ -11120,16 +11120,16 @@
       <c r="R100" s="86" t="s">
         <v>672</v>
       </c>
-      <c r="S100" s="104" t="s">
+      <c r="S100" s="105" t="s">
         <v>187</v>
       </c>
-      <c r="T100" s="104"/>
-      <c r="U100" s="104"/>
-      <c r="V100" s="104"/>
-      <c r="W100" s="104"/>
-      <c r="X100" s="104"/>
-      <c r="Y100" s="104"/>
-      <c r="Z100" s="104"/>
+      <c r="T100" s="105"/>
+      <c r="U100" s="105"/>
+      <c r="V100" s="105"/>
+      <c r="W100" s="105"/>
+      <c r="X100" s="105"/>
+      <c r="Y100" s="105"/>
+      <c r="Z100" s="105"/>
       <c r="AA100" s="65"/>
       <c r="AB100" s="65"/>
       <c r="AC100" s="65"/>
@@ -11793,24 +11793,24 @@
     </row>
     <row r="116" spans="1:41" ht="12.75">
       <c r="A116" s="80"/>
-      <c r="B116" s="113"/>
-      <c r="C116" s="113"/>
-      <c r="D116" s="113"/>
-      <c r="E116" s="113"/>
-      <c r="F116" s="113"/>
-      <c r="G116" s="113"/>
-      <c r="H116" s="113"/>
-      <c r="I116" s="113"/>
-      <c r="J116" s="113"/>
-      <c r="K116" s="113"/>
-      <c r="L116" s="113"/>
-      <c r="M116" s="113"/>
-      <c r="N116" s="113"/>
-      <c r="O116" s="113"/>
-      <c r="P116" s="113"/>
-      <c r="Q116" s="113"/>
-      <c r="R116" s="113"/>
-      <c r="S116" s="113"/>
+      <c r="B116" s="102"/>
+      <c r="C116" s="102"/>
+      <c r="D116" s="102"/>
+      <c r="E116" s="102"/>
+      <c r="F116" s="102"/>
+      <c r="G116" s="102"/>
+      <c r="H116" s="102"/>
+      <c r="I116" s="102"/>
+      <c r="J116" s="102"/>
+      <c r="K116" s="102"/>
+      <c r="L116" s="102"/>
+      <c r="M116" s="102"/>
+      <c r="N116" s="102"/>
+      <c r="O116" s="102"/>
+      <c r="P116" s="102"/>
+      <c r="Q116" s="102"/>
+      <c r="R116" s="102"/>
+      <c r="S116" s="102"/>
       <c r="T116" s="80"/>
       <c r="U116" s="80"/>
       <c r="V116" s="80"/>
@@ -12137,24 +12137,24 @@
     </row>
     <row r="124" spans="1:41" ht="12.75">
       <c r="A124" s="80"/>
-      <c r="B124" s="113"/>
-      <c r="C124" s="113"/>
-      <c r="D124" s="113"/>
-      <c r="E124" s="113"/>
-      <c r="F124" s="113"/>
-      <c r="G124" s="113"/>
-      <c r="H124" s="113"/>
-      <c r="I124" s="113"/>
-      <c r="J124" s="113"/>
-      <c r="K124" s="113"/>
-      <c r="L124" s="113"/>
-      <c r="M124" s="113"/>
-      <c r="N124" s="113"/>
-      <c r="O124" s="113"/>
-      <c r="P124" s="113"/>
-      <c r="Q124" s="113"/>
-      <c r="R124" s="113"/>
-      <c r="S124" s="113"/>
+      <c r="B124" s="102"/>
+      <c r="C124" s="102"/>
+      <c r="D124" s="102"/>
+      <c r="E124" s="102"/>
+      <c r="F124" s="102"/>
+      <c r="G124" s="102"/>
+      <c r="H124" s="102"/>
+      <c r="I124" s="102"/>
+      <c r="J124" s="102"/>
+      <c r="K124" s="102"/>
+      <c r="L124" s="102"/>
+      <c r="M124" s="102"/>
+      <c r="N124" s="102"/>
+      <c r="O124" s="102"/>
+      <c r="P124" s="102"/>
+      <c r="Q124" s="102"/>
+      <c r="R124" s="102"/>
+      <c r="S124" s="102"/>
       <c r="T124" s="80"/>
       <c r="U124" s="80"/>
       <c r="V124" s="80"/>
@@ -12395,24 +12395,24 @@
     </row>
     <row r="130" spans="1:41" ht="12.75">
       <c r="A130" s="80"/>
-      <c r="B130" s="113"/>
-      <c r="C130" s="113"/>
-      <c r="D130" s="113"/>
-      <c r="E130" s="113"/>
-      <c r="F130" s="113"/>
-      <c r="G130" s="113"/>
-      <c r="H130" s="113"/>
-      <c r="I130" s="113"/>
-      <c r="J130" s="113"/>
-      <c r="K130" s="113"/>
-      <c r="L130" s="113"/>
-      <c r="M130" s="113"/>
-      <c r="N130" s="113"/>
-      <c r="O130" s="113"/>
-      <c r="P130" s="113"/>
-      <c r="Q130" s="113"/>
-      <c r="R130" s="113"/>
-      <c r="S130" s="113"/>
+      <c r="B130" s="102"/>
+      <c r="C130" s="102"/>
+      <c r="D130" s="102"/>
+      <c r="E130" s="102"/>
+      <c r="F130" s="102"/>
+      <c r="G130" s="102"/>
+      <c r="H130" s="102"/>
+      <c r="I130" s="102"/>
+      <c r="J130" s="102"/>
+      <c r="K130" s="102"/>
+      <c r="L130" s="102"/>
+      <c r="M130" s="102"/>
+      <c r="N130" s="102"/>
+      <c r="O130" s="102"/>
+      <c r="P130" s="102"/>
+      <c r="Q130" s="102"/>
+      <c r="R130" s="102"/>
+      <c r="S130" s="102"/>
       <c r="T130" s="80"/>
       <c r="U130" s="80"/>
       <c r="V130" s="80"/>
@@ -12782,20 +12782,20 @@
     </row>
     <row r="139" spans="1:41" ht="12.75">
       <c r="A139" s="80"/>
-      <c r="B139" s="113"/>
-      <c r="C139" s="113"/>
-      <c r="D139" s="113"/>
-      <c r="E139" s="113"/>
-      <c r="F139" s="113"/>
-      <c r="G139" s="113"/>
-      <c r="H139" s="113"/>
-      <c r="I139" s="113"/>
-      <c r="J139" s="113"/>
-      <c r="K139" s="113"/>
-      <c r="L139" s="113"/>
-      <c r="M139" s="113"/>
-      <c r="N139" s="113"/>
-      <c r="O139" s="113"/>
+      <c r="B139" s="102"/>
+      <c r="C139" s="102"/>
+      <c r="D139" s="102"/>
+      <c r="E139" s="102"/>
+      <c r="F139" s="102"/>
+      <c r="G139" s="102"/>
+      <c r="H139" s="102"/>
+      <c r="I139" s="102"/>
+      <c r="J139" s="102"/>
+      <c r="K139" s="102"/>
+      <c r="L139" s="102"/>
+      <c r="M139" s="102"/>
+      <c r="N139" s="102"/>
+      <c r="O139" s="102"/>
       <c r="P139" s="93"/>
       <c r="Q139" s="93"/>
       <c r="R139" s="93"/>
@@ -49505,98 +49505,6 @@
   </sheetData>
   <autoFilter ref="A1:AI895" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <mergeCells count="116">
-    <mergeCell ref="B116:S116"/>
-    <mergeCell ref="B124:S124"/>
-    <mergeCell ref="B130:S130"/>
-    <mergeCell ref="B139:O139"/>
-    <mergeCell ref="E91:F91"/>
-    <mergeCell ref="S91:Z91"/>
-    <mergeCell ref="E92:F92"/>
-    <mergeCell ref="S92:Z92"/>
-    <mergeCell ref="E93:F93"/>
-    <mergeCell ref="S93:Z93"/>
-    <mergeCell ref="S94:AA94"/>
-    <mergeCell ref="E95:F95"/>
-    <mergeCell ref="E96:F96"/>
-    <mergeCell ref="S96:Z96"/>
-    <mergeCell ref="S95:Y95"/>
-    <mergeCell ref="S100:Z100"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="S2:X2"/>
-    <mergeCell ref="S3:Y3"/>
-    <mergeCell ref="S7:Z7"/>
-    <mergeCell ref="S9:Z9"/>
-    <mergeCell ref="S10:Y10"/>
-    <mergeCell ref="S14:Y14"/>
-    <mergeCell ref="S16:AA16"/>
-    <mergeCell ref="S18:X18"/>
-    <mergeCell ref="S1:T1"/>
-    <mergeCell ref="S4:X4"/>
-    <mergeCell ref="S5:Y5"/>
-    <mergeCell ref="S6:Y6"/>
-    <mergeCell ref="S8:Y8"/>
-    <mergeCell ref="S11:Y11"/>
-    <mergeCell ref="S17:Z17"/>
-    <mergeCell ref="S21:Y21"/>
-    <mergeCell ref="S12:Z12"/>
-    <mergeCell ref="S13:Z13"/>
-    <mergeCell ref="S15:Z15"/>
-    <mergeCell ref="S29:Z29"/>
-    <mergeCell ref="S31:Z31"/>
-    <mergeCell ref="S22:Z22"/>
-    <mergeCell ref="S23:Y23"/>
-    <mergeCell ref="S25:Y25"/>
-    <mergeCell ref="S26:Y26"/>
-    <mergeCell ref="S19:Y19"/>
-    <mergeCell ref="S20:Z20"/>
-    <mergeCell ref="S24:Y24"/>
-    <mergeCell ref="S27:Z27"/>
-    <mergeCell ref="S28:Z28"/>
-    <mergeCell ref="S30:Y30"/>
-    <mergeCell ref="S32:Y32"/>
-    <mergeCell ref="S33:Z33"/>
-    <mergeCell ref="S34:Y34"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="S35:Y35"/>
-    <mergeCell ref="S36:X36"/>
-    <mergeCell ref="S37:Z37"/>
-    <mergeCell ref="S38:AA38"/>
-    <mergeCell ref="S39:X39"/>
-    <mergeCell ref="S40:X40"/>
-    <mergeCell ref="S41:Z41"/>
-    <mergeCell ref="S42:AA42"/>
-    <mergeCell ref="S43:Z43"/>
-    <mergeCell ref="S44:Y44"/>
-    <mergeCell ref="S45:Z45"/>
-    <mergeCell ref="S46:X46"/>
-    <mergeCell ref="S47:Y47"/>
-    <mergeCell ref="S53:Z53"/>
-    <mergeCell ref="S48:Z48"/>
-    <mergeCell ref="S49:AA49"/>
-    <mergeCell ref="S50:Y50"/>
-    <mergeCell ref="S51:Z51"/>
-    <mergeCell ref="S52:Z52"/>
-    <mergeCell ref="S73:Y73"/>
-    <mergeCell ref="S75:Y75"/>
-    <mergeCell ref="S76:Y76"/>
-    <mergeCell ref="S77:Z77"/>
-    <mergeCell ref="S78:Z78"/>
-    <mergeCell ref="S79:X79"/>
-    <mergeCell ref="S54:Y54"/>
-    <mergeCell ref="S55:Z55"/>
-    <mergeCell ref="S56:X56"/>
-    <mergeCell ref="S57:X57"/>
-    <mergeCell ref="S64:Y64"/>
-    <mergeCell ref="S69:Z69"/>
-    <mergeCell ref="S58:X58"/>
-    <mergeCell ref="S59:Y59"/>
-    <mergeCell ref="S60:X60"/>
-    <mergeCell ref="S61:Y61"/>
-    <mergeCell ref="S62:Z62"/>
-    <mergeCell ref="S63:Y63"/>
-    <mergeCell ref="S65:Z65"/>
-    <mergeCell ref="S66:Z66"/>
-    <mergeCell ref="S67:Z67"/>
     <mergeCell ref="S90:Y90"/>
     <mergeCell ref="S87:X87"/>
     <mergeCell ref="S88:Y88"/>
@@ -49621,6 +49529,98 @@
     <mergeCell ref="S82:AA82"/>
     <mergeCell ref="S84:X84"/>
     <mergeCell ref="S85:X85"/>
+    <mergeCell ref="S73:Y73"/>
+    <mergeCell ref="S75:Y75"/>
+    <mergeCell ref="S76:Y76"/>
+    <mergeCell ref="S77:Z77"/>
+    <mergeCell ref="S78:Z78"/>
+    <mergeCell ref="S79:X79"/>
+    <mergeCell ref="S54:Y54"/>
+    <mergeCell ref="S55:Z55"/>
+    <mergeCell ref="S56:X56"/>
+    <mergeCell ref="S57:X57"/>
+    <mergeCell ref="S64:Y64"/>
+    <mergeCell ref="S69:Z69"/>
+    <mergeCell ref="S58:X58"/>
+    <mergeCell ref="S59:Y59"/>
+    <mergeCell ref="S60:X60"/>
+    <mergeCell ref="S61:Y61"/>
+    <mergeCell ref="S62:Z62"/>
+    <mergeCell ref="S63:Y63"/>
+    <mergeCell ref="S65:Z65"/>
+    <mergeCell ref="S66:Z66"/>
+    <mergeCell ref="S67:Z67"/>
+    <mergeCell ref="S40:X40"/>
+    <mergeCell ref="S41:Z41"/>
+    <mergeCell ref="S42:AA42"/>
+    <mergeCell ref="S43:Z43"/>
+    <mergeCell ref="S44:Y44"/>
+    <mergeCell ref="S45:Z45"/>
+    <mergeCell ref="S46:X46"/>
+    <mergeCell ref="S47:Y47"/>
+    <mergeCell ref="S53:Z53"/>
+    <mergeCell ref="S48:Z48"/>
+    <mergeCell ref="S49:AA49"/>
+    <mergeCell ref="S50:Y50"/>
+    <mergeCell ref="S51:Z51"/>
+    <mergeCell ref="S52:Z52"/>
+    <mergeCell ref="S32:Y32"/>
+    <mergeCell ref="S33:Z33"/>
+    <mergeCell ref="S34:Y34"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="S35:Y35"/>
+    <mergeCell ref="S36:X36"/>
+    <mergeCell ref="S37:Z37"/>
+    <mergeCell ref="S38:AA38"/>
+    <mergeCell ref="S39:X39"/>
+    <mergeCell ref="S29:Z29"/>
+    <mergeCell ref="S31:Z31"/>
+    <mergeCell ref="S22:Z22"/>
+    <mergeCell ref="S23:Y23"/>
+    <mergeCell ref="S25:Y25"/>
+    <mergeCell ref="S26:Y26"/>
+    <mergeCell ref="S19:Y19"/>
+    <mergeCell ref="S20:Z20"/>
+    <mergeCell ref="S24:Y24"/>
+    <mergeCell ref="S27:Z27"/>
+    <mergeCell ref="S28:Z28"/>
+    <mergeCell ref="S30:Y30"/>
+    <mergeCell ref="S1:T1"/>
+    <mergeCell ref="S4:X4"/>
+    <mergeCell ref="S5:Y5"/>
+    <mergeCell ref="S6:Y6"/>
+    <mergeCell ref="S8:Y8"/>
+    <mergeCell ref="S11:Y11"/>
+    <mergeCell ref="S17:Z17"/>
+    <mergeCell ref="S21:Y21"/>
+    <mergeCell ref="S12:Z12"/>
+    <mergeCell ref="S13:Z13"/>
+    <mergeCell ref="S15:Z15"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="S2:X2"/>
+    <mergeCell ref="S3:Y3"/>
+    <mergeCell ref="S7:Z7"/>
+    <mergeCell ref="S9:Z9"/>
+    <mergeCell ref="S10:Y10"/>
+    <mergeCell ref="S14:Y14"/>
+    <mergeCell ref="S16:AA16"/>
+    <mergeCell ref="S18:X18"/>
+    <mergeCell ref="B116:S116"/>
+    <mergeCell ref="B124:S124"/>
+    <mergeCell ref="B130:S130"/>
+    <mergeCell ref="B139:O139"/>
+    <mergeCell ref="E91:F91"/>
+    <mergeCell ref="S91:Z91"/>
+    <mergeCell ref="E92:F92"/>
+    <mergeCell ref="S92:Z92"/>
+    <mergeCell ref="E93:F93"/>
+    <mergeCell ref="S93:Z93"/>
+    <mergeCell ref="S94:AA94"/>
+    <mergeCell ref="E95:F95"/>
+    <mergeCell ref="E96:F96"/>
+    <mergeCell ref="S96:Z96"/>
+    <mergeCell ref="S95:Y95"/>
+    <mergeCell ref="S100:Z100"/>
   </mergeCells>
   <phoneticPr fontId="21" type="noConversion"/>
   <hyperlinks>

</xml_diff>